<commit_message>
Introduced crop transitions for entering and leaving a level.  The number of tiles was reduced from 32 to 30 to free up sufficient memory to implement the feature.
</commit_message>
<xml_diff>
--- a/docs/Memory.xlsx
+++ b/docs/Memory.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\Beeb\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\Beeb\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E5EAC4E-741D-4B83-BA2D-D5DEE8403802}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22B15ADB-FA11-402E-B161-F2813FFFFEEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12950" yWindow="3250" windowWidth="24870" windowHeight="17050" xr2:uid="{C0DF3A0D-E6A9-4F13-8EDD-5DE46AD6E0DB}"/>
+    <workbookView xWindow="19110" yWindow="0" windowWidth="19380" windowHeight="20970" xr2:uid="{C0DF3A0D-E6A9-4F13-8EDD-5DE46AD6E0DB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="74">
   <si>
     <t>Quantity</t>
   </si>
@@ -134,9 +134,6 @@
     <t>Level palette</t>
   </si>
   <si>
-    <t>Level tiles</t>
-  </si>
-  <si>
     <t>Level tile grid</t>
   </si>
   <si>
@@ -146,9 +143,6 @@
     <t>sound effects</t>
   </si>
   <si>
-    <t>level palette</t>
-  </si>
-  <si>
     <t>game object arrays</t>
   </si>
   <si>
@@ -255,6 +249,15 @@
   </si>
   <si>
     <t>Draw object jump tables</t>
+  </si>
+  <si>
+    <t>29 level tiles</t>
+  </si>
+  <si>
+    <t>Black palette</t>
+  </si>
+  <si>
+    <t>black palette</t>
   </si>
 </sst>
 </file>
@@ -645,7 +648,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="94">
+  <cellXfs count="97">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
@@ -870,6 +873,11 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1205,12 +1213,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10CD322F-64B0-476A-AEFE-F468CB566666}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="B1:R100"/>
+  <dimension ref="B1:R101"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="2.81640625" customWidth="1"/>
     <col min="2" max="2" width="18.1796875" customWidth="1"/>
-    <col min="3" max="16" width="9.7265625" customWidth="1"/>
+    <col min="3" max="5" width="9.7265625" customWidth="1"/>
+    <col min="6" max="6" width="10.81640625" customWidth="1"/>
+    <col min="7" max="16" width="9.7265625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:18" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
@@ -1322,7 +1332,7 @@
     </row>
     <row r="5" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B5" s="36" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C5" s="9">
         <v>10</v>
@@ -1375,7 +1385,7 @@
     </row>
     <row r="6" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B6" s="1" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C6" s="19">
         <v>1</v>
@@ -1428,7 +1438,7 @@
     </row>
     <row r="7" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B7" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C7" s="19">
         <v>11</v>
@@ -1482,7 +1492,7 @@
     </row>
     <row r="8" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B8" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C8" s="19">
         <v>4</v>
@@ -1536,7 +1546,7 @@
     </row>
     <row r="9" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B9" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C9" s="19">
         <v>11</v>
@@ -1590,7 +1600,7 @@
     </row>
     <row r="10" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B10" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C10" s="19">
         <v>4</v>
@@ -1644,7 +1654,7 @@
     </row>
     <row r="11" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B11" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C11" s="19">
         <v>1</v>
@@ -1750,7 +1760,7 @@
     </row>
     <row r="13" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B13" s="38" t="s">
-        <v>36</v>
+        <v>73</v>
       </c>
       <c r="C13" s="34">
         <v>1</v>
@@ -1922,7 +1932,7 @@
       <c r="E19" s="56"/>
       <c r="F19" s="58"/>
       <c r="H19" s="59" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="I19" s="53"/>
       <c r="J19" s="60" t="s">
@@ -1932,7 +1942,7 @@
         <v>2</v>
       </c>
       <c r="L19" s="60" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="M19" s="53"/>
       <c r="N19" s="54"/>
@@ -1951,17 +1961,17 @@
       <c r="E20" s="56"/>
       <c r="F20" s="58"/>
       <c r="H20" s="47" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="I20" s="17"/>
       <c r="J20" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="K20" s="30">
         <v>30</v>
       </c>
       <c r="L20" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="N20" s="48"/>
     </row>
@@ -1974,7 +1984,7 @@
         <v>64</v>
       </c>
       <c r="D21" s="68" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E21" s="69"/>
       <c r="F21" s="70"/>
@@ -1983,13 +1993,13 @@
       </c>
       <c r="I21" s="17"/>
       <c r="J21" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="K21" s="30">
         <v>64</v>
       </c>
       <c r="L21" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="N21" s="48"/>
     </row>
@@ -2011,13 +2021,13 @@
       </c>
       <c r="I22" s="17"/>
       <c r="J22" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="K22" s="30">
         <v>64</v>
       </c>
       <c r="L22" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="N22" s="48"/>
     </row>
@@ -2034,17 +2044,17 @@
       </c>
       <c r="F23" s="48"/>
       <c r="H23" s="47" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I23" s="17"/>
       <c r="J23" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="K23" s="30">
         <v>44</v>
       </c>
       <c r="L23" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="N23" s="48"/>
     </row>
@@ -2062,17 +2072,17 @@
       </c>
       <c r="F24" s="48"/>
       <c r="H24" s="47" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="I24" s="17"/>
       <c r="J24" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="K24" s="30">
         <v>12</v>
       </c>
       <c r="L24" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="N24" s="48"/>
     </row>
@@ -2085,22 +2095,22 @@
         <v>32</v>
       </c>
       <c r="D25" s="69" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E25" s="69"/>
       <c r="F25" s="70"/>
       <c r="H25" s="49" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="I25" s="50"/>
       <c r="J25" s="50" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="K25" s="16">
         <v>20</v>
       </c>
       <c r="L25" s="51" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="M25" s="51"/>
       <c r="N25" s="52"/>
@@ -2114,7 +2124,7 @@
         <v>480</v>
       </c>
       <c r="D26" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="F26" s="48"/>
       <c r="H26" s="17"/>
@@ -2130,7 +2140,7 @@
         <v>48</v>
       </c>
       <c r="D27" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="F27" s="48"/>
     </row>
@@ -2157,7 +2167,7 @@
         <v>96</v>
       </c>
       <c r="D29" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="F29" s="48"/>
     </row>
@@ -2170,7 +2180,7 @@
         <v>16</v>
       </c>
       <c r="D30" s="68" t="s">
-        <v>31</v>
+        <v>72</v>
       </c>
       <c r="E30" s="69"/>
       <c r="F30" s="70"/>
@@ -2198,7 +2208,7 @@
         <v>64</v>
       </c>
       <c r="D32" s="63" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F32" s="48"/>
     </row>
@@ -2255,7 +2265,7 @@
         <v>32</v>
       </c>
       <c r="D36" s="63" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F36" s="48"/>
     </row>
@@ -2268,7 +2278,7 @@
         <v>64</v>
       </c>
       <c r="D37" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="F37" s="48"/>
     </row>
@@ -2281,7 +2291,7 @@
         <v>160</v>
       </c>
       <c r="D38" s="77" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E38" s="77"/>
       <c r="F38" s="78"/>
@@ -2323,7 +2333,7 @@
         <v>96</v>
       </c>
       <c r="D41" s="68" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E41" s="69"/>
       <c r="F41" s="70"/>
@@ -2351,7 +2361,7 @@
         <v>48</v>
       </c>
       <c r="D43" s="63" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F43" s="48"/>
     </row>
@@ -2377,7 +2387,7 @@
         <v>12</v>
       </c>
       <c r="D45" s="63" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="F45" s="48"/>
     </row>
@@ -2390,7 +2400,7 @@
         <v>20</v>
       </c>
       <c r="D46" s="68" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E46" s="69"/>
       <c r="F46" s="70"/>
@@ -2402,7 +2412,7 @@
       </c>
       <c r="C47" s="71">
         <f>HEX2DEC(B49)-HEX2DEC(B47)</f>
-        <v>7680</v>
+        <v>7792</v>
       </c>
       <c r="D47" s="72" t="s">
         <v>10</v>
@@ -2413,33 +2423,33 @@
     <row r="48" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B48" s="74" t="str">
         <f t="shared" ref="B48" si="18">DEC2HEX(HEX2DEC(B49)-C48)</f>
-        <v>2BA0</v>
+        <v>2C10</v>
       </c>
       <c r="C48" s="30">
         <v>864</v>
       </c>
       <c r="D48" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F48" s="48"/>
     </row>
     <row r="49" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B49" s="47" t="str">
-        <f t="shared" ref="B49:B51" si="19">DEC2HEX(HEX2DEC(B50)-C49)</f>
-        <v>2F00</v>
+        <f t="shared" ref="B49:B52" si="19">DEC2HEX(HEX2DEC(B50)-C49)</f>
+        <v>2F70</v>
       </c>
       <c r="C49" s="30">
         <v>96</v>
       </c>
       <c r="D49" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="F49" s="48"/>
     </row>
     <row r="50" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B50" s="67" t="str">
-        <f>DEC2HEX(HEX2DEC(B51)-C50)</f>
-        <v>2F60</v>
+        <f t="shared" si="19"/>
+        <v>2FD0</v>
       </c>
       <c r="C50" s="33">
         <f>$D$11</f>
@@ -2453,47 +2463,55 @@
     </row>
     <row r="51" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B51" s="47" t="str">
-        <f t="shared" si="19"/>
-        <v>3040</v>
-      </c>
-      <c r="C51" s="30">
-        <f>64*31</f>
-        <v>1984</v>
-      </c>
-      <c r="D51" s="17" t="s">
-        <v>32</v>
-      </c>
+        <f>DEC2HEX(HEX2DEC(B52)-C51)</f>
+        <v>30B0</v>
+      </c>
+      <c r="C51" s="94">
+        <v>16</v>
+      </c>
+      <c r="D51" s="96" t="s">
+        <v>31</v>
+      </c>
+      <c r="E51" s="95"/>
       <c r="F51" s="48"/>
     </row>
     <row r="52" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B52" s="47" t="str">
-        <f t="shared" ref="B52" si="20">DEC2HEX(HEX2DEC(B53)-C52)</f>
+        <f t="shared" si="19"/>
+        <v>30C0</v>
+      </c>
+      <c r="C52" s="30">
+        <v>1856</v>
+      </c>
+      <c r="D52" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="F52" s="48"/>
+    </row>
+    <row r="53" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B53" s="47" t="str">
+        <f t="shared" ref="B53" si="20">DEC2HEX(HEX2DEC(B54)-C53)</f>
         <v>3800</v>
       </c>
-      <c r="C52" s="30">
+      <c r="C53" s="30">
         <f>2048</f>
         <v>2048</v>
       </c>
-      <c r="D52" s="17" t="s">
-        <v>33</v>
-      </c>
-      <c r="F52" s="48"/>
-    </row>
-    <row r="53" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B53" s="49">
+      <c r="D53" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="F53" s="48"/>
+    </row>
+    <row r="54" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B54" s="49">
         <v>4000</v>
       </c>
-      <c r="C53" s="16"/>
-      <c r="D53" s="50" t="s">
+      <c r="C54" s="16"/>
+      <c r="D54" s="50" t="s">
         <v>21</v>
       </c>
-      <c r="E53" s="51"/>
-      <c r="F53" s="52"/>
-    </row>
-    <row r="54" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B54" s="17"/>
-      <c r="C54" s="17"/>
-      <c r="D54" s="17"/>
+      <c r="E54" s="51"/>
+      <c r="F54" s="52"/>
     </row>
     <row r="55" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B55" s="17"/>
@@ -2516,7 +2534,7 @@
       <c r="D58" s="17"/>
     </row>
     <row r="59" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B59" s="46"/>
+      <c r="B59" s="17"/>
       <c r="C59" s="17"/>
       <c r="D59" s="17"/>
     </row>
@@ -2592,6 +2610,8 @@
     </row>
     <row r="74" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B74" s="46"/>
+      <c r="C74" s="17"/>
+      <c r="D74" s="17"/>
     </row>
     <row r="75" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B75" s="46"/>
@@ -2669,7 +2689,10 @@
       <c r="B99" s="46"/>
     </row>
     <row r="100" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B100" s="45"/>
+      <c r="B100" s="46"/>
+    </row>
+    <row r="101" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B101" s="45"/>
     </row>
   </sheetData>
   <mergeCells count="12">

</xml_diff>

<commit_message>
Checked in MMB with updated docs
</commit_message>
<xml_diff>
--- a/docs/Memory.xlsx
+++ b/docs/Memory.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\Beeb\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22B15ADB-FA11-402E-B161-F2813FFFFEEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B93991C1-EE0B-49C3-96A9-177978B25915}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19110" yWindow="0" windowWidth="19380" windowHeight="20970" xr2:uid="{C0DF3A0D-E6A9-4F13-8EDD-5DE46AD6E0DB}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="76">
   <si>
     <t>Quantity</t>
   </si>
@@ -258,6 +258,12 @@
   </si>
   <si>
     <t>black palette</t>
+  </si>
+  <si>
+    <t>zero-page game variables</t>
+  </si>
+  <si>
+    <t>zero-page MOS variables</t>
   </si>
 </sst>
 </file>
@@ -289,7 +295,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -302,6 +308,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="32">
     <border>
@@ -648,7 +660,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="97">
+  <cellXfs count="103">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
@@ -802,7 +814,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -837,12 +848,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -873,11 +879,29 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1225,35 +1249,35 @@
   <sheetData>
     <row r="1" spans="2:18" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="2" spans="2:18" x14ac:dyDescent="0.35">
-      <c r="B2" s="88" t="s">
+      <c r="B2" s="84" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="90" t="s">
-        <v>0</v>
-      </c>
-      <c r="D2" s="85" t="s">
+      <c r="C2" s="86" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" s="81" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="84" t="s">
+      <c r="E2" s="80" t="s">
         <v>24</v>
       </c>
-      <c r="F2" s="87"/>
-      <c r="G2" s="84" t="s">
+      <c r="F2" s="83"/>
+      <c r="G2" s="80" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="85"/>
-      <c r="I2" s="86" t="s">
+      <c r="H2" s="81"/>
+      <c r="I2" s="82" t="s">
         <v>12</v>
       </c>
-      <c r="J2" s="87"/>
-      <c r="K2" s="84" t="s">
+      <c r="J2" s="83"/>
+      <c r="K2" s="80" t="s">
         <v>14</v>
       </c>
-      <c r="L2" s="85"/>
-      <c r="M2" s="86" t="s">
+      <c r="L2" s="81"/>
+      <c r="M2" s="82" t="s">
         <v>15</v>
       </c>
-      <c r="N2" s="87"/>
+      <c r="N2" s="83"/>
       <c r="O2" s="43" t="s">
         <v>6</v>
       </c>
@@ -1264,35 +1288,35 @@
       <c r="R2" s="15"/>
     </row>
     <row r="3" spans="2:18" x14ac:dyDescent="0.35">
-      <c r="B3" s="89"/>
-      <c r="C3" s="91"/>
-      <c r="D3" s="92"/>
-      <c r="E3" s="91" t="s">
+      <c r="B3" s="85"/>
+      <c r="C3" s="87"/>
+      <c r="D3" s="88"/>
+      <c r="E3" s="87" t="s">
         <v>25</v>
       </c>
-      <c r="F3" s="93"/>
-      <c r="G3" s="91" t="s">
+      <c r="F3" s="89"/>
+      <c r="G3" s="87" t="s">
         <v>25</v>
       </c>
-      <c r="H3" s="92"/>
+      <c r="H3" s="88"/>
       <c r="I3" s="41"/>
       <c r="J3" s="40"/>
-      <c r="K3" s="91" t="s">
+      <c r="K3" s="87" t="s">
         <v>25</v>
       </c>
-      <c r="L3" s="92"/>
-      <c r="M3" s="93" t="s">
+      <c r="L3" s="88"/>
+      <c r="M3" s="89" t="s">
         <v>25</v>
       </c>
-      <c r="N3" s="93"/>
+      <c r="N3" s="89"/>
       <c r="O3" s="42"/>
       <c r="P3" s="24"/>
       <c r="R3" s="15"/>
     </row>
     <row r="4" spans="2:18" x14ac:dyDescent="0.35">
-      <c r="B4" s="89"/>
-      <c r="C4" s="91"/>
-      <c r="D4" s="92"/>
+      <c r="B4" s="85"/>
+      <c r="C4" s="87"/>
+      <c r="D4" s="88"/>
       <c r="E4" s="21" t="s">
         <v>0</v>
       </c>
@@ -1920,13 +1944,13 @@
       <c r="P18" s="3"/>
     </row>
     <row r="19" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B19" s="64" t="s">
+      <c r="B19" s="63" t="s">
         <v>7</v>
       </c>
       <c r="C19" s="57" t="s">
         <v>22</v>
       </c>
-      <c r="D19" s="65" t="s">
+      <c r="D19" s="64" t="s">
         <v>8</v>
       </c>
       <c r="E19" s="56"/>
@@ -1949,14 +1973,13 @@
     </row>
     <row r="20" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B20" s="62">
-        <v>100</v>
-      </c>
-      <c r="C20" s="66">
-        <f>(24*32/4)</f>
-        <v>192</v>
+        <v>0</v>
+      </c>
+      <c r="C20" s="65">
+        <v>144</v>
       </c>
       <c r="D20" s="56" t="s">
-        <v>26</v>
+        <v>74</v>
       </c>
       <c r="E20" s="56"/>
       <c r="F20" s="58"/>
@@ -1976,18 +1999,17 @@
       <c r="N20" s="48"/>
     </row>
     <row r="21" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B21" s="67" t="str">
-        <f t="shared" ref="B21:B47" si="17">DEC2HEX(HEX2DEC(B20)+C20)</f>
-        <v>1C0</v>
-      </c>
-      <c r="C21" s="33">
-        <v>64</v>
-      </c>
-      <c r="D21" s="68" t="s">
-        <v>33</v>
-      </c>
-      <c r="E21" s="69"/>
-      <c r="F21" s="70"/>
+      <c r="B21" s="99">
+        <v>90</v>
+      </c>
+      <c r="C21" s="100">
+        <v>112</v>
+      </c>
+      <c r="D21" s="101" t="s">
+        <v>75</v>
+      </c>
+      <c r="E21" s="101"/>
+      <c r="F21" s="102"/>
       <c r="H21" s="47" t="s">
         <v>17</v>
       </c>
@@ -2004,18 +2026,18 @@
       <c r="N21" s="48"/>
     </row>
     <row r="22" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B22" s="75" t="str">
-        <f t="shared" si="17"/>
-        <v>200</v>
-      </c>
-      <c r="C22" s="76">
-        <v>256</v>
-      </c>
-      <c r="D22" s="77" t="s">
-        <v>9</v>
-      </c>
-      <c r="E22" s="77"/>
-      <c r="F22" s="78"/>
+      <c r="B22" s="73">
+        <v>100</v>
+      </c>
+      <c r="C22" s="31">
+        <f>(24*32/4)</f>
+        <v>192</v>
+      </c>
+      <c r="D22" s="90" t="s">
+        <v>26</v>
+      </c>
+      <c r="E22" s="90"/>
+      <c r="F22" s="98"/>
       <c r="H22" s="47" t="s">
         <v>18</v>
       </c>
@@ -2032,17 +2054,18 @@
       <c r="N22" s="48"/>
     </row>
     <row r="23" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B23" s="47" t="str">
-        <f t="shared" si="17"/>
-        <v>300</v>
-      </c>
-      <c r="C23" s="30">
-        <v>192</v>
-      </c>
-      <c r="D23" t="s">
-        <v>26</v>
-      </c>
-      <c r="F23" s="48"/>
+      <c r="B23" s="66" t="str">
+        <f t="shared" ref="B23:B49" si="17">DEC2HEX(HEX2DEC(B22)+C22)</f>
+        <v>1C0</v>
+      </c>
+      <c r="C23" s="33">
+        <v>64</v>
+      </c>
+      <c r="D23" s="67" t="s">
+        <v>33</v>
+      </c>
+      <c r="E23" s="68"/>
+      <c r="F23" s="69"/>
       <c r="H23" s="47" t="s">
         <v>34</v>
       </c>
@@ -2059,18 +2082,18 @@
       <c r="N23" s="48"/>
     </row>
     <row r="24" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B24" s="47" t="str">
+      <c r="B24" s="74" t="str">
         <f t="shared" si="17"/>
-        <v>3C0</v>
-      </c>
-      <c r="C24" s="30">
-        <f>$D$8</f>
-        <v>32</v>
-      </c>
-      <c r="D24" s="63" t="s">
-        <v>27</v>
-      </c>
-      <c r="F24" s="48"/>
+        <v>200</v>
+      </c>
+      <c r="C24" s="75">
+        <v>256</v>
+      </c>
+      <c r="D24" s="76" t="s">
+        <v>9</v>
+      </c>
+      <c r="E24" s="76"/>
+      <c r="F24" s="77"/>
       <c r="H24" s="47" t="s">
         <v>47</v>
       </c>
@@ -2087,18 +2110,18 @@
       <c r="N24" s="48"/>
     </row>
     <row r="25" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B25" s="67" t="str">
+      <c r="B25" s="47" t="str">
         <f t="shared" si="17"/>
-        <v>3E0</v>
-      </c>
-      <c r="C25" s="33">
-        <v>32</v>
-      </c>
-      <c r="D25" s="69" t="s">
-        <v>69</v>
-      </c>
-      <c r="E25" s="69"/>
-      <c r="F25" s="70"/>
+        <v>300</v>
+      </c>
+      <c r="C25" s="91">
+        <v>192</v>
+      </c>
+      <c r="D25" s="92" t="s">
+        <v>26</v>
+      </c>
+      <c r="E25" s="92"/>
+      <c r="F25" s="48"/>
       <c r="H25" s="49" t="s">
         <v>65</v>
       </c>
@@ -2118,410 +2141,442 @@
     <row r="26" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B26" s="47" t="str">
         <f t="shared" si="17"/>
-        <v>400</v>
-      </c>
-      <c r="C26" s="30">
-        <v>480</v>
-      </c>
-      <c r="D26" t="s">
-        <v>54</v>
-      </c>
+        <v>3C0</v>
+      </c>
+      <c r="C26" s="91">
+        <f>$D$8</f>
+        <v>32</v>
+      </c>
+      <c r="D26" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="E26" s="92"/>
       <c r="F26" s="48"/>
       <c r="H26" s="17"/>
       <c r="I26" s="17"/>
       <c r="K26" s="30"/>
     </row>
     <row r="27" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B27" s="47" t="str">
+      <c r="B27" s="66" t="str">
         <f t="shared" si="17"/>
-        <v>5E0</v>
-      </c>
-      <c r="C27" s="30">
-        <v>48</v>
-      </c>
-      <c r="D27" t="s">
-        <v>55</v>
-      </c>
-      <c r="F27" s="48"/>
+        <v>3E0</v>
+      </c>
+      <c r="C27" s="33">
+        <v>32</v>
+      </c>
+      <c r="D27" s="68" t="s">
+        <v>69</v>
+      </c>
+      <c r="E27" s="68"/>
+      <c r="F27" s="69"/>
     </row>
     <row r="28" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B28" s="47" t="str">
         <f t="shared" si="17"/>
-        <v>610</v>
-      </c>
-      <c r="C28" s="30">
-        <v>384</v>
-      </c>
-      <c r="D28" t="s">
-        <v>20</v>
-      </c>
+        <v>400</v>
+      </c>
+      <c r="C28" s="91">
+        <v>480</v>
+      </c>
+      <c r="D28" s="92" t="s">
+        <v>54</v>
+      </c>
+      <c r="E28" s="92"/>
       <c r="F28" s="48"/>
       <c r="I28" s="55"/>
     </row>
     <row r="29" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B29" s="47" t="str">
         <f t="shared" si="17"/>
+        <v>5E0</v>
+      </c>
+      <c r="C29" s="91">
+        <v>48</v>
+      </c>
+      <c r="D29" s="92" t="s">
+        <v>55</v>
+      </c>
+      <c r="E29" s="92"/>
+      <c r="F29" s="48"/>
+    </row>
+    <row r="30" spans="2:16" x14ac:dyDescent="0.35">
+      <c r="B30" s="47" t="str">
+        <f t="shared" si="17"/>
+        <v>610</v>
+      </c>
+      <c r="C30" s="91">
+        <v>384</v>
+      </c>
+      <c r="D30" s="92" t="s">
+        <v>20</v>
+      </c>
+      <c r="E30" s="92"/>
+      <c r="F30" s="48"/>
+    </row>
+    <row r="31" spans="2:16" x14ac:dyDescent="0.35">
+      <c r="B31" s="47" t="str">
+        <f t="shared" si="17"/>
         <v>790</v>
       </c>
-      <c r="C29" s="30">
+      <c r="C31" s="91">
         <v>96</v>
       </c>
-      <c r="D29" t="s">
+      <c r="D31" s="92" t="s">
         <v>56</v>
       </c>
-      <c r="F29" s="48"/>
-    </row>
-    <row r="30" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B30" s="67" t="str">
+      <c r="E31" s="92"/>
+      <c r="F31" s="48"/>
+    </row>
+    <row r="32" spans="2:16" x14ac:dyDescent="0.35">
+      <c r="B32" s="66" t="str">
         <f t="shared" si="17"/>
         <v>7F0</v>
       </c>
-      <c r="C30" s="33">
+      <c r="C32" s="33">
         <v>16</v>
       </c>
-      <c r="D30" s="68" t="s">
+      <c r="D32" s="67" t="s">
         <v>72</v>
       </c>
-      <c r="E30" s="69"/>
-      <c r="F30" s="70"/>
-    </row>
-    <row r="31" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B31" s="79" t="str">
+      <c r="E32" s="68"/>
+      <c r="F32" s="69"/>
+    </row>
+    <row r="33" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B33" s="78" t="str">
         <f t="shared" si="17"/>
         <v>800</v>
       </c>
-      <c r="C31" s="80">
+      <c r="C33" s="94">
         <v>128</v>
       </c>
-      <c r="D31" s="81" t="s">
+      <c r="D33" s="95" t="s">
         <v>29</v>
       </c>
-      <c r="E31" s="81"/>
-      <c r="F31" s="82"/>
-    </row>
-    <row r="32" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B32" s="47" t="str">
+      <c r="E33" s="95"/>
+      <c r="F33" s="79"/>
+    </row>
+    <row r="34" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B34" s="47" t="str">
         <f t="shared" si="17"/>
         <v>880</v>
       </c>
-      <c r="C32" s="30">
+      <c r="C34" s="91">
         <v>64</v>
       </c>
-      <c r="D32" s="63" t="s">
+      <c r="D34" s="93" t="s">
         <v>57</v>
       </c>
-      <c r="F32" s="48"/>
-    </row>
-    <row r="33" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B33" s="75" t="str">
+      <c r="E34" s="92"/>
+      <c r="F34" s="48"/>
+    </row>
+    <row r="35" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B35" s="74" t="str">
         <f t="shared" si="17"/>
         <v>8C0</v>
       </c>
-      <c r="C33" s="76">
+      <c r="C35" s="75">
         <f>2*$D$8</f>
         <v>64</v>
       </c>
-      <c r="D33" s="77" t="s">
+      <c r="D35" s="76" t="s">
         <v>29</v>
       </c>
-      <c r="E33" s="77"/>
-      <c r="F33" s="78"/>
-      <c r="H33" s="55"/>
-    </row>
-    <row r="34" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B34" s="47" t="str">
+      <c r="E35" s="76"/>
+      <c r="F35" s="77"/>
+    </row>
+    <row r="36" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B36" s="47" t="str">
         <f t="shared" si="17"/>
         <v>900</v>
       </c>
-      <c r="C34" s="30">
+      <c r="C36" s="91">
         <v>960</v>
       </c>
-      <c r="D34" t="s">
+      <c r="D36" s="92" t="s">
         <v>19</v>
       </c>
-      <c r="F34" s="48"/>
-    </row>
-    <row r="35" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B35" s="67" t="str">
+      <c r="E36" s="92"/>
+      <c r="F36" s="48"/>
+    </row>
+    <row r="37" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B37" s="66" t="str">
         <f t="shared" si="17"/>
         <v>CC0</v>
       </c>
-      <c r="C35" s="33">
+      <c r="C37" s="33">
         <v>64</v>
       </c>
-      <c r="D35" s="69" t="s">
+      <c r="D37" s="68" t="s">
         <v>28</v>
       </c>
-      <c r="E35" s="69"/>
-      <c r="F35" s="70"/>
-      <c r="H35" s="55"/>
-    </row>
-    <row r="36" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B36" s="47" t="str">
+      <c r="E37" s="68"/>
+      <c r="F37" s="69"/>
+    </row>
+    <row r="38" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B38" s="47" t="str">
         <f t="shared" si="17"/>
         <v>D00</v>
       </c>
-      <c r="C36" s="30">
+      <c r="C38" s="91">
         <v>32</v>
       </c>
-      <c r="D36" s="63" t="s">
+      <c r="D38" s="93" t="s">
         <v>68</v>
       </c>
-      <c r="F36" s="48"/>
-    </row>
-    <row r="37" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B37" s="47" t="str">
-        <f t="shared" si="17"/>
+      <c r="E38" s="92"/>
+      <c r="F38" s="48"/>
+    </row>
+    <row r="39" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B39" s="47" t="str">
+        <f>DEC2HEX(HEX2DEC(B38)+C38)</f>
         <v>D20</v>
       </c>
-      <c r="C37" s="30">
+      <c r="C39" s="91">
         <v>64</v>
       </c>
-      <c r="D37" t="s">
+      <c r="D39" s="92" t="s">
         <v>58</v>
       </c>
-      <c r="F37" s="48"/>
-    </row>
-    <row r="38" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B38" s="75" t="str">
+      <c r="E39" s="92"/>
+      <c r="F39" s="48"/>
+    </row>
+    <row r="40" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B40" s="74" t="str">
         <f t="shared" si="17"/>
         <v>D60</v>
       </c>
-      <c r="C38" s="76">
+      <c r="C40" s="75">
         <v>160</v>
       </c>
-      <c r="D38" s="77" t="s">
+      <c r="D40" s="76" t="s">
         <v>59</v>
       </c>
-      <c r="E38" s="77"/>
-      <c r="F38" s="78"/>
-      <c r="H38" s="3"/>
-    </row>
-    <row r="39" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B39" s="47" t="str">
+      <c r="E40" s="76"/>
+      <c r="F40" s="77"/>
+    </row>
+    <row r="41" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B41" s="47" t="str">
         <f t="shared" si="17"/>
         <v>E00</v>
       </c>
-      <c r="C39" s="30">
+      <c r="C41" s="91">
         <v>384</v>
       </c>
-      <c r="D39" s="63" t="s">
+      <c r="D41" s="93" t="s">
         <v>20</v>
       </c>
-      <c r="F39" s="48"/>
-      <c r="H39" s="3"/>
-    </row>
-    <row r="40" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B40" s="47" t="str">
+      <c r="E41" s="92"/>
+      <c r="F41" s="48"/>
+    </row>
+    <row r="42" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B42" s="47" t="str">
         <f t="shared" si="17"/>
         <v>F80</v>
       </c>
-      <c r="C40" s="30">
+      <c r="C42" s="91">
         <v>32</v>
       </c>
-      <c r="D40" s="63" t="s">
+      <c r="D42" s="93" t="s">
         <v>27</v>
       </c>
-      <c r="F40" s="48"/>
-    </row>
-    <row r="41" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B41" s="67" t="str">
+      <c r="E42" s="92"/>
+      <c r="F42" s="48"/>
+    </row>
+    <row r="43" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B43" s="66" t="str">
         <f t="shared" si="17"/>
         <v>FA0</v>
       </c>
-      <c r="C41" s="33">
+      <c r="C43" s="33">
         <v>96</v>
       </c>
-      <c r="D41" s="68" t="s">
+      <c r="D43" s="67" t="s">
         <v>60</v>
       </c>
-      <c r="E41" s="69"/>
-      <c r="F41" s="70"/>
-    </row>
-    <row r="42" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B42" s="79" t="str">
+      <c r="E43" s="68"/>
+      <c r="F43" s="69"/>
+    </row>
+    <row r="44" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B44" s="78" t="str">
         <f t="shared" si="17"/>
         <v>1000</v>
       </c>
-      <c r="C42" s="80">
+      <c r="C44" s="94">
         <v>144</v>
       </c>
-      <c r="D42" s="83" t="s">
+      <c r="D44" s="96" t="s">
         <v>23</v>
       </c>
-      <c r="E42" s="81"/>
-      <c r="F42" s="82"/>
-    </row>
-    <row r="43" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B43" s="47" t="str">
+      <c r="E44" s="95"/>
+      <c r="F44" s="79"/>
+    </row>
+    <row r="45" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B45" s="47" t="str">
         <f t="shared" si="17"/>
         <v>1090</v>
       </c>
-      <c r="C43" s="30">
+      <c r="C45" s="91">
         <v>48</v>
       </c>
-      <c r="D43" s="63" t="s">
+      <c r="D45" s="93" t="s">
         <v>61</v>
       </c>
-      <c r="F43" s="48"/>
-    </row>
-    <row r="44" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B44" s="47" t="str">
+      <c r="E45" s="92"/>
+      <c r="F45" s="48"/>
+    </row>
+    <row r="46" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B46" s="47" t="str">
         <f t="shared" si="17"/>
         <v>10C0</v>
       </c>
-      <c r="C44" s="30">
+      <c r="C46" s="91">
         <v>32</v>
       </c>
-      <c r="D44" s="63" t="s">
+      <c r="D46" s="93" t="s">
         <v>23</v>
       </c>
-      <c r="F44" s="48"/>
-    </row>
-    <row r="45" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B45" s="47" t="str">
+      <c r="E46" s="92"/>
+      <c r="F46" s="48"/>
+    </row>
+    <row r="47" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B47" s="47" t="str">
         <f t="shared" si="17"/>
         <v>10E0</v>
       </c>
-      <c r="C45" s="30">
+      <c r="C47" s="91">
         <v>12</v>
       </c>
-      <c r="D45" s="63" t="s">
+      <c r="D47" s="93" t="s">
         <v>67</v>
       </c>
-      <c r="F45" s="48"/>
-    </row>
-    <row r="46" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B46" s="67" t="str">
+      <c r="E47" s="92"/>
+      <c r="F47" s="48"/>
+    </row>
+    <row r="48" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B48" s="66" t="str">
         <f t="shared" si="17"/>
         <v>10EC</v>
       </c>
-      <c r="C46" s="33">
+      <c r="C48" s="33">
         <v>20</v>
       </c>
-      <c r="D46" s="68" t="s">
+      <c r="D48" s="67" t="s">
         <v>70</v>
       </c>
-      <c r="E46" s="69"/>
-      <c r="F46" s="70"/>
-    </row>
-    <row r="47" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B47" s="47" t="str">
+      <c r="E48" s="68"/>
+      <c r="F48" s="69"/>
+    </row>
+    <row r="49" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B49" s="47" t="str">
         <f t="shared" si="17"/>
         <v>1100</v>
       </c>
-      <c r="C47" s="71">
-        <f>HEX2DEC(B49)-HEX2DEC(B47)</f>
-        <v>7792</v>
-      </c>
-      <c r="D47" s="72" t="s">
+      <c r="C49" s="70">
+        <f>HEX2DEC(B50)-HEX2DEC(B49)</f>
+        <v>6928</v>
+      </c>
+      <c r="D49" s="71" t="s">
         <v>10</v>
       </c>
-      <c r="E47" s="72"/>
-      <c r="F47" s="73"/>
-    </row>
-    <row r="48" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B48" s="74" t="str">
-        <f t="shared" ref="B48" si="18">DEC2HEX(HEX2DEC(B49)-C48)</f>
+      <c r="E49" s="71"/>
+      <c r="F49" s="72"/>
+    </row>
+    <row r="50" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B50" s="73" t="str">
+        <f>DEC2HEX(HEX2DEC(B51)-C50)</f>
         <v>2C10</v>
       </c>
-      <c r="C48" s="30">
+      <c r="C50" s="91">
         <v>864</v>
       </c>
-      <c r="D48" t="s">
+      <c r="D50" s="92" t="s">
         <v>62</v>
       </c>
-      <c r="F48" s="48"/>
-    </row>
-    <row r="49" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B49" s="47" t="str">
-        <f t="shared" ref="B49:B52" si="19">DEC2HEX(HEX2DEC(B50)-C49)</f>
+      <c r="E50" s="92"/>
+      <c r="F50" s="48"/>
+    </row>
+    <row r="51" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B51" s="47" t="str">
+        <f t="shared" ref="B51" si="18">DEC2HEX(HEX2DEC(B52)-C51)</f>
         <v>2F70</v>
       </c>
-      <c r="C49" s="30">
+      <c r="C51" s="91">
         <v>96</v>
       </c>
-      <c r="D49" t="s">
+      <c r="D51" s="92" t="s">
         <v>64</v>
       </c>
-      <c r="F49" s="48"/>
-    </row>
-    <row r="50" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B50" s="67" t="str">
-        <f t="shared" si="19"/>
+      <c r="E51" s="92"/>
+      <c r="F51" s="48"/>
+    </row>
+    <row r="52" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B52" s="66" t="str">
+        <f>DEC2HEX(HEX2DEC(B53)-C52)</f>
         <v>2FD0</v>
       </c>
-      <c r="C50" s="33">
+      <c r="C52" s="33">
         <f>$D$11</f>
         <v>224</v>
       </c>
-      <c r="D50" s="69" t="s">
+      <c r="D52" s="68" t="s">
         <v>30</v>
       </c>
-      <c r="E50" s="69"/>
-      <c r="F50" s="70"/>
-    </row>
-    <row r="51" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B51" s="47" t="str">
-        <f>DEC2HEX(HEX2DEC(B52)-C51)</f>
-        <v>30B0</v>
-      </c>
-      <c r="C51" s="94">
-        <v>16</v>
-      </c>
-      <c r="D51" s="96" t="s">
-        <v>31</v>
-      </c>
-      <c r="E51" s="95"/>
-      <c r="F51" s="48"/>
-    </row>
-    <row r="52" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B52" s="47" t="str">
-        <f t="shared" si="19"/>
-        <v>30C0</v>
-      </c>
-      <c r="C52" s="30">
-        <v>1856</v>
-      </c>
-      <c r="D52" s="17" t="s">
-        <v>71</v>
-      </c>
-      <c r="F52" s="48"/>
+      <c r="E52" s="68"/>
+      <c r="F52" s="69"/>
     </row>
     <row r="53" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B53" s="47" t="str">
-        <f t="shared" ref="B53" si="20">DEC2HEX(HEX2DEC(B54)-C53)</f>
+        <f>DEC2HEX(HEX2DEC(B54)-C53)</f>
+        <v>30B0</v>
+      </c>
+      <c r="C53" s="91">
+        <v>16</v>
+      </c>
+      <c r="D53" s="92" t="s">
+        <v>31</v>
+      </c>
+      <c r="E53" s="92"/>
+      <c r="F53" s="48"/>
+    </row>
+    <row r="54" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B54" s="47" t="str">
+        <f>DEC2HEX(HEX2DEC(B55)-C54)</f>
+        <v>30C0</v>
+      </c>
+      <c r="C54" s="91">
+        <v>1856</v>
+      </c>
+      <c r="D54" s="97" t="s">
+        <v>71</v>
+      </c>
+      <c r="E54" s="92"/>
+      <c r="F54" s="48"/>
+    </row>
+    <row r="55" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B55" s="47" t="str">
+        <f t="shared" ref="B55" si="19">DEC2HEX(HEX2DEC(B56)-C55)</f>
         <v>3800</v>
       </c>
-      <c r="C53" s="30">
+      <c r="C55" s="91">
         <f>2048</f>
         <v>2048</v>
       </c>
-      <c r="D53" s="17" t="s">
+      <c r="D55" s="97" t="s">
         <v>32</v>
       </c>
-      <c r="F53" s="48"/>
-    </row>
-    <row r="54" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B54" s="49">
+      <c r="E55" s="92"/>
+      <c r="F55" s="48"/>
+    </row>
+    <row r="56" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B56" s="49">
         <v>4000</v>
       </c>
-      <c r="C54" s="16"/>
-      <c r="D54" s="50" t="s">
+      <c r="C56" s="16"/>
+      <c r="D56" s="50" t="s">
         <v>21</v>
       </c>
-      <c r="E54" s="51"/>
-      <c r="F54" s="52"/>
-    </row>
-    <row r="55" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B55" s="17"/>
-      <c r="C55" s="17"/>
-      <c r="D55" s="17"/>
-    </row>
-    <row r="56" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B56" s="17"/>
-      <c r="C56" s="17"/>
-      <c r="D56" s="17"/>
+      <c r="E56" s="51"/>
+      <c r="F56" s="52"/>
     </row>
     <row r="57" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B57" s="17"/>

</xml_diff>

<commit_message>
Updated address locations to align with last change
</commit_message>
<xml_diff>
--- a/docs/Memory.xlsx
+++ b/docs/Memory.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\Beeb\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A643EA7F-F269-4E71-A2B0-74126C1D3C8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD664BD7-8369-419F-BBF5-E144CA1B4552}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12840" yWindow="1620" windowWidth="20890" windowHeight="19260" xr2:uid="{C0DF3A0D-E6A9-4F13-8EDD-5DE46AD6E0DB}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{C0DF3A0D-E6A9-4F13-8EDD-5DE46AD6E0DB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="101">
   <si>
     <t>Quantity</t>
   </si>
@@ -270,13 +270,82 @@
   </si>
   <si>
     <t>Tile &amp; sprite high addr tbls (NMI workspace)</t>
+  </si>
+  <si>
+    <t>Level extents</t>
+  </si>
+  <si>
+    <t>Level tile types</t>
+  </si>
+  <si>
+    <t>401E</t>
+  </si>
+  <si>
+    <t>Level settings</t>
+  </si>
+  <si>
+    <t>Level object descriptors (48)</t>
+  </si>
+  <si>
+    <t>Level switch pairings</t>
+  </si>
+  <si>
+    <t>Level sprite data</t>
+  </si>
+  <si>
+    <t>4F83</t>
+  </si>
+  <si>
+    <t>Level initialization code</t>
+  </si>
+  <si>
+    <t>Mode 7 routines</t>
+  </si>
+  <si>
+    <t>Music data and code</t>
+  </si>
+  <si>
+    <t>7B00</t>
+  </si>
+  <si>
+    <t>DFS command page backup</t>
+  </si>
+  <si>
+    <t>7C00</t>
+  </si>
+  <si>
+    <t>Mode 7 screen</t>
+  </si>
+  <si>
+    <t>PCM load buffer</t>
+  </si>
+  <si>
+    <t>6E66</t>
+  </si>
+  <si>
+    <t>56B0</t>
+  </si>
+  <si>
+    <t>60FF</t>
+  </si>
+  <si>
+    <t>Titles, interstitial, or finale</t>
+  </si>
+  <si>
+    <t>40E3</t>
+  </si>
+  <si>
+    <t>6D8F</t>
+  </si>
+  <si>
+    <t>Unused memory</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -300,6 +369,18 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -716,7 +797,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="106">
+  <cellXfs count="128">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
@@ -965,6 +1046,56 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="11" fontId="3" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1300,7 +1431,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10CD322F-64B0-476A-AEFE-F468CB566666}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="B1:R103"/>
+  <dimension ref="B1:R101"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="2.81640625" customWidth="1"/>
@@ -2696,101 +2827,233 @@
       <c r="C59" s="17"/>
       <c r="D59" s="17"/>
     </row>
-    <row r="60" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="60" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B60" s="17"/>
       <c r="C60" s="17"/>
       <c r="D60" s="17"/>
     </row>
-    <row r="61" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B61" s="17"/>
-      <c r="C61" s="17"/>
-      <c r="D61" s="17"/>
+    <row r="61" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B61" s="117" t="s">
+        <v>7</v>
+      </c>
+      <c r="C61" s="61" t="s">
+        <v>20</v>
+      </c>
+      <c r="D61" s="118" t="s">
+        <v>8</v>
+      </c>
+      <c r="E61" s="119"/>
+      <c r="F61" s="120"/>
     </row>
     <row r="62" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B62" s="46"/>
-      <c r="C62" s="17"/>
-      <c r="D62" s="17"/>
+      <c r="B62" s="109">
+        <v>4000</v>
+      </c>
+      <c r="C62" s="107">
+        <f>HEX2DEC(B63)-HEX2DEC(B62)</f>
+        <v>2</v>
+      </c>
+      <c r="D62" s="108" t="s">
+        <v>78</v>
+      </c>
+      <c r="E62" s="106"/>
+      <c r="F62" s="110"/>
     </row>
     <row r="63" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B63" s="46"/>
-      <c r="C63" s="17"/>
-      <c r="D63" s="17"/>
+      <c r="B63" s="109">
+        <v>4002</v>
+      </c>
+      <c r="C63" s="107">
+        <f>HEX2DEC(B64)-HEX2DEC(B63)</f>
+        <v>28</v>
+      </c>
+      <c r="D63" s="108" t="s">
+        <v>79</v>
+      </c>
+      <c r="E63" s="106"/>
+      <c r="F63" s="110"/>
     </row>
     <row r="64" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B64" s="46"/>
-      <c r="C64" s="17"/>
-      <c r="D64" s="17"/>
-    </row>
-    <row r="65" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B65" s="46"/>
-      <c r="C65" s="17"/>
-      <c r="D65" s="17"/>
-    </row>
-    <row r="66" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B66" s="46"/>
-      <c r="C66" s="17"/>
-      <c r="D66" s="17"/>
-    </row>
-    <row r="67" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B67" s="46"/>
-      <c r="C67" s="17"/>
-      <c r="D67" s="17"/>
-    </row>
-    <row r="68" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B68" s="46"/>
-      <c r="C68" s="17"/>
-      <c r="D68" s="17"/>
-    </row>
-    <row r="69" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B69" s="46"/>
-      <c r="C69" s="17"/>
-      <c r="D69" s="17"/>
-    </row>
-    <row r="70" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B70" s="46"/>
-      <c r="C70" s="17"/>
-      <c r="D70" s="17"/>
-    </row>
-    <row r="71" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B71" s="46"/>
-      <c r="C71" s="17"/>
-      <c r="D71" s="17"/>
-    </row>
-    <row r="72" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B72" s="46"/>
-      <c r="C72" s="17"/>
-      <c r="D72" s="17"/>
-    </row>
-    <row r="73" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B73" s="46"/>
-      <c r="C73" s="17"/>
-      <c r="D73" s="17"/>
-    </row>
-    <row r="74" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B74" s="46"/>
-      <c r="C74" s="17"/>
-      <c r="D74" s="17"/>
-    </row>
-    <row r="75" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B75" s="46"/>
-      <c r="C75" s="17"/>
-      <c r="D75" s="17"/>
-    </row>
-    <row r="76" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B64" s="109" t="s">
+        <v>80</v>
+      </c>
+      <c r="C64" s="107">
+        <f t="shared" ref="C64:C75" si="20">HEX2DEC(B65)-HEX2DEC(B64)</f>
+        <v>5</v>
+      </c>
+      <c r="D64" s="108" t="s">
+        <v>81</v>
+      </c>
+      <c r="E64" s="106"/>
+      <c r="F64" s="110"/>
+    </row>
+    <row r="65" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B65" s="109">
+        <v>4023</v>
+      </c>
+      <c r="C65" s="107">
+        <f t="shared" si="20"/>
+        <v>192</v>
+      </c>
+      <c r="D65" s="108" t="s">
+        <v>82</v>
+      </c>
+      <c r="E65" s="106"/>
+      <c r="F65" s="110"/>
+    </row>
+    <row r="66" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B66" s="111" t="s">
+        <v>98</v>
+      </c>
+      <c r="C66" s="107">
+        <f t="shared" si="20"/>
+        <v>32</v>
+      </c>
+      <c r="D66" s="108" t="s">
+        <v>83</v>
+      </c>
+      <c r="E66" s="106"/>
+      <c r="F66" s="110"/>
+    </row>
+    <row r="67" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B67" s="109">
+        <v>4103</v>
+      </c>
+      <c r="C67" s="107">
+        <f t="shared" si="20"/>
+        <v>3712</v>
+      </c>
+      <c r="D67" s="108" t="s">
+        <v>84</v>
+      </c>
+      <c r="E67" s="106"/>
+      <c r="F67" s="110"/>
+    </row>
+    <row r="68" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B68" s="109" t="s">
+        <v>85</v>
+      </c>
+      <c r="C68" s="107">
+        <f t="shared" si="20"/>
+        <v>1761</v>
+      </c>
+      <c r="D68" s="108" t="s">
+        <v>86</v>
+      </c>
+      <c r="E68" s="106"/>
+      <c r="F68" s="110"/>
+    </row>
+    <row r="69" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B69" s="109">
+        <v>5664</v>
+      </c>
+      <c r="C69" s="107">
+        <f t="shared" si="20"/>
+        <v>76</v>
+      </c>
+      <c r="D69" s="108" t="s">
+        <v>87</v>
+      </c>
+      <c r="E69" s="106"/>
+      <c r="F69" s="110"/>
+    </row>
+    <row r="70" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B70" s="122" t="s">
+        <v>95</v>
+      </c>
+      <c r="C70" s="107">
+        <f t="shared" si="20"/>
+        <v>2639</v>
+      </c>
+      <c r="D70" s="121" t="s">
+        <v>97</v>
+      </c>
+      <c r="E70" s="106"/>
+      <c r="F70" s="110"/>
+    </row>
+    <row r="71" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B71" s="109" t="s">
+        <v>96</v>
+      </c>
+      <c r="C71" s="107">
+        <f t="shared" si="20"/>
+        <v>3216</v>
+      </c>
+      <c r="D71" s="108" t="s">
+        <v>88</v>
+      </c>
+      <c r="E71" s="106"/>
+      <c r="F71" s="110"/>
+    </row>
+    <row r="72" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B72" s="123" t="s">
+        <v>99</v>
+      </c>
+      <c r="C72" s="124">
+        <f t="shared" si="20"/>
+        <v>215</v>
+      </c>
+      <c r="D72" s="125" t="s">
+        <v>100</v>
+      </c>
+      <c r="E72" s="126"/>
+      <c r="F72" s="127"/>
+    </row>
+    <row r="73" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B73" s="111" t="s">
+        <v>94</v>
+      </c>
+      <c r="C73" s="107">
+        <f t="shared" si="20"/>
+        <v>3226</v>
+      </c>
+      <c r="D73" s="108" t="s">
+        <v>93</v>
+      </c>
+      <c r="E73" s="106"/>
+      <c r="F73" s="110"/>
+    </row>
+    <row r="74" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B74" s="109" t="s">
+        <v>89</v>
+      </c>
+      <c r="C74" s="107">
+        <f t="shared" si="20"/>
+        <v>256</v>
+      </c>
+      <c r="D74" s="108" t="s">
+        <v>90</v>
+      </c>
+      <c r="E74" s="106"/>
+      <c r="F74" s="110"/>
+    </row>
+    <row r="75" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B75" s="112" t="s">
+        <v>91</v>
+      </c>
+      <c r="C75" s="113">
+        <v>1024</v>
+      </c>
+      <c r="D75" s="114" t="s">
+        <v>92</v>
+      </c>
+      <c r="E75" s="115"/>
+      <c r="F75" s="116"/>
+    </row>
+    <row r="76" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B76" s="46"/>
-      <c r="C76" s="17"/>
-      <c r="D76" s="17"/>
-    </row>
-    <row r="77" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="C76" s="107"/>
+    </row>
+    <row r="77" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B77" s="46"/>
     </row>
-    <row r="78" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="78" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B78" s="46"/>
     </row>
-    <row r="79" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="79" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B79" s="46"/>
     </row>
-    <row r="80" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="80" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B80" s="46"/>
     </row>
     <row r="81" spans="2:2" x14ac:dyDescent="0.35">
@@ -2854,13 +3117,7 @@
       <c r="B100" s="46"/>
     </row>
     <row r="101" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B101" s="46"/>
-    </row>
-    <row r="102" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B102" s="46"/>
-    </row>
-    <row r="103" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B103" s="45"/>
+      <c r="B101" s="45"/>
     </row>
   </sheetData>
   <mergeCells count="12">

</xml_diff>

<commit_message>
Three changes:  - Various documentation updates  - Fixed regression where enemy weapon and 'exterminate' sound could continue after Dalek was destroyed  - Re-normalized enemy weapon strength setting, making the default value 256 instead of 128.
</commit_message>
<xml_diff>
--- a/docs/Memory.xlsx
+++ b/docs/Memory.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\Beeb\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD664BD7-8369-419F-BBF5-E144CA1B4552}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F01BA20F-4944-44A6-8C1D-2D7055F40E06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{C0DF3A0D-E6A9-4F13-8EDD-5DE46AD6E0DB}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="19380" windowHeight="20970" xr2:uid="{C0DF3A0D-E6A9-4F13-8EDD-5DE46AD6E0DB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="100">
   <si>
     <t>Quantity</t>
   </si>
@@ -323,22 +323,19 @@
     <t>6E66</t>
   </si>
   <si>
-    <t>56B0</t>
-  </si>
-  <si>
-    <t>60FF</t>
-  </si>
-  <si>
     <t>Titles, interstitial, or finale</t>
   </si>
   <si>
     <t>40E3</t>
   </si>
   <si>
-    <t>6D8F</t>
-  </si>
-  <si>
     <t>Unused memory</t>
+  </si>
+  <si>
+    <t>56B4</t>
+  </si>
+  <si>
+    <t>6D93</t>
   </si>
 </sst>
 </file>
@@ -797,7 +794,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="128">
+  <cellXfs count="120">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1016,6 +1013,48 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="11" fontId="3" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1046,56 +1085,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="11" fontId="3" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1441,35 +1430,35 @@
   <sheetData>
     <row r="1" spans="2:18" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="2" spans="2:18" x14ac:dyDescent="0.35">
-      <c r="B2" s="100" t="s">
+      <c r="B2" s="114" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="102" t="s">
-        <v>0</v>
-      </c>
-      <c r="D2" s="97" t="s">
+      <c r="C2" s="116" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" s="111" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="96" t="s">
+      <c r="E2" s="110" t="s">
         <v>22</v>
       </c>
-      <c r="F2" s="99"/>
-      <c r="G2" s="96" t="s">
+      <c r="F2" s="113"/>
+      <c r="G2" s="110" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="97"/>
-      <c r="I2" s="98" t="s">
+      <c r="H2" s="111"/>
+      <c r="I2" s="112" t="s">
         <v>12</v>
       </c>
-      <c r="J2" s="99"/>
-      <c r="K2" s="96" t="s">
+      <c r="J2" s="113"/>
+      <c r="K2" s="110" t="s">
         <v>14</v>
       </c>
-      <c r="L2" s="97"/>
-      <c r="M2" s="98" t="s">
+      <c r="L2" s="111"/>
+      <c r="M2" s="112" t="s">
         <v>15</v>
       </c>
-      <c r="N2" s="99"/>
+      <c r="N2" s="113"/>
       <c r="O2" s="43" t="s">
         <v>6</v>
       </c>
@@ -1480,35 +1469,35 @@
       <c r="R2" s="15"/>
     </row>
     <row r="3" spans="2:18" x14ac:dyDescent="0.35">
-      <c r="B3" s="101"/>
-      <c r="C3" s="103"/>
-      <c r="D3" s="104"/>
-      <c r="E3" s="103" t="s">
+      <c r="B3" s="115"/>
+      <c r="C3" s="117"/>
+      <c r="D3" s="118"/>
+      <c r="E3" s="117" t="s">
         <v>23</v>
       </c>
-      <c r="F3" s="105"/>
-      <c r="G3" s="103" t="s">
+      <c r="F3" s="119"/>
+      <c r="G3" s="117" t="s">
         <v>23</v>
       </c>
-      <c r="H3" s="104"/>
+      <c r="H3" s="118"/>
       <c r="I3" s="41"/>
       <c r="J3" s="40"/>
-      <c r="K3" s="103" t="s">
+      <c r="K3" s="117" t="s">
         <v>23</v>
       </c>
-      <c r="L3" s="104"/>
-      <c r="M3" s="105" t="s">
+      <c r="L3" s="118"/>
+      <c r="M3" s="119" t="s">
         <v>23</v>
       </c>
-      <c r="N3" s="105"/>
+      <c r="N3" s="119"/>
       <c r="O3" s="42"/>
       <c r="P3" s="24"/>
       <c r="R3" s="15"/>
     </row>
     <row r="4" spans="2:18" x14ac:dyDescent="0.35">
-      <c r="B4" s="101"/>
-      <c r="C4" s="103"/>
-      <c r="D4" s="104"/>
+      <c r="B4" s="115"/>
+      <c r="C4" s="117"/>
+      <c r="D4" s="118"/>
       <c r="E4" s="21" t="s">
         <v>0</v>
       </c>
@@ -2833,216 +2822,204 @@
       <c r="D60" s="17"/>
     </row>
     <row r="61" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B61" s="117" t="s">
+      <c r="B61" s="103" t="s">
         <v>7</v>
       </c>
       <c r="C61" s="61" t="s">
         <v>20</v>
       </c>
-      <c r="D61" s="118" t="s">
+      <c r="D61" s="104" t="s">
         <v>8</v>
       </c>
-      <c r="E61" s="119"/>
-      <c r="F61" s="120"/>
+      <c r="E61" s="53"/>
+      <c r="F61" s="54"/>
     </row>
     <row r="62" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B62" s="109">
+      <c r="B62" s="98">
         <v>4000</v>
       </c>
-      <c r="C62" s="107">
+      <c r="C62" s="96">
         <f>HEX2DEC(B63)-HEX2DEC(B62)</f>
         <v>2</v>
       </c>
-      <c r="D62" s="108" t="s">
+      <c r="D62" s="97" t="s">
         <v>78</v>
       </c>
-      <c r="E62" s="106"/>
-      <c r="F62" s="110"/>
+      <c r="F62" s="48"/>
     </row>
     <row r="63" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B63" s="109">
+      <c r="B63" s="98">
         <v>4002</v>
       </c>
-      <c r="C63" s="107">
+      <c r="C63" s="96">
         <f>HEX2DEC(B64)-HEX2DEC(B63)</f>
         <v>28</v>
       </c>
-      <c r="D63" s="108" t="s">
+      <c r="D63" s="97" t="s">
         <v>79</v>
       </c>
-      <c r="E63" s="106"/>
-      <c r="F63" s="110"/>
+      <c r="F63" s="48"/>
     </row>
     <row r="64" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B64" s="109" t="s">
+      <c r="B64" s="98" t="s">
         <v>80</v>
       </c>
-      <c r="C64" s="107">
-        <f t="shared" ref="C64:C75" si="20">HEX2DEC(B65)-HEX2DEC(B64)</f>
+      <c r="C64" s="96">
+        <f t="shared" ref="C64:C74" si="20">HEX2DEC(B65)-HEX2DEC(B64)</f>
         <v>5</v>
       </c>
-      <c r="D64" s="108" t="s">
+      <c r="D64" s="97" t="s">
         <v>81</v>
       </c>
-      <c r="E64" s="106"/>
-      <c r="F64" s="110"/>
+      <c r="F64" s="48"/>
     </row>
     <row r="65" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B65" s="109">
+      <c r="B65" s="98">
         <v>4023</v>
       </c>
-      <c r="C65" s="107">
+      <c r="C65" s="96">
         <f t="shared" si="20"/>
         <v>192</v>
       </c>
-      <c r="D65" s="108" t="s">
+      <c r="D65" s="97" t="s">
         <v>82</v>
       </c>
-      <c r="E65" s="106"/>
-      <c r="F65" s="110"/>
+      <c r="F65" s="48"/>
     </row>
     <row r="66" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B66" s="111" t="s">
-        <v>98</v>
-      </c>
-      <c r="C66" s="107">
+      <c r="B66" s="99" t="s">
+        <v>96</v>
+      </c>
+      <c r="C66" s="96">
         <f t="shared" si="20"/>
         <v>32</v>
       </c>
-      <c r="D66" s="108" t="s">
+      <c r="D66" s="97" t="s">
         <v>83</v>
       </c>
-      <c r="E66" s="106"/>
-      <c r="F66" s="110"/>
+      <c r="F66" s="48"/>
     </row>
     <row r="67" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B67" s="109">
+      <c r="B67" s="98">
         <v>4103</v>
       </c>
-      <c r="C67" s="107">
+      <c r="C67" s="96">
         <f t="shared" si="20"/>
         <v>3712</v>
       </c>
-      <c r="D67" s="108" t="s">
+      <c r="D67" s="97" t="s">
         <v>84</v>
       </c>
-      <c r="E67" s="106"/>
-      <c r="F67" s="110"/>
+      <c r="F67" s="48"/>
     </row>
     <row r="68" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B68" s="109" t="s">
+      <c r="B68" s="98" t="s">
         <v>85</v>
       </c>
-      <c r="C68" s="107">
+      <c r="C68" s="96">
         <f t="shared" si="20"/>
-        <v>1761</v>
-      </c>
-      <c r="D68" s="108" t="s">
+        <v>1765</v>
+      </c>
+      <c r="D68" s="97" t="s">
         <v>86</v>
       </c>
-      <c r="E68" s="106"/>
-      <c r="F68" s="110"/>
+      <c r="F68" s="48"/>
     </row>
     <row r="69" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B69" s="109">
-        <v>5664</v>
-      </c>
-      <c r="C69" s="107">
+      <c r="B69" s="98">
+        <v>5668</v>
+      </c>
+      <c r="C69" s="96">
         <f t="shared" si="20"/>
         <v>76</v>
       </c>
-      <c r="D69" s="108" t="s">
+      <c r="D69" s="97" t="s">
         <v>87</v>
       </c>
-      <c r="E69" s="106"/>
-      <c r="F69" s="110"/>
+      <c r="F69" s="48"/>
     </row>
     <row r="70" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B70" s="122" t="s">
-        <v>95</v>
-      </c>
-      <c r="C70" s="107">
+      <c r="B70" s="106" t="s">
+        <v>98</v>
+      </c>
+      <c r="C70" s="96">
         <f t="shared" si="20"/>
         <v>2639</v>
       </c>
-      <c r="D70" s="121" t="s">
-        <v>97</v>
-      </c>
-      <c r="E70" s="106"/>
-      <c r="F70" s="110"/>
+      <c r="D70" s="105" t="s">
+        <v>95</v>
+      </c>
+      <c r="F70" s="48"/>
     </row>
     <row r="71" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B71" s="109" t="s">
-        <v>96</v>
-      </c>
-      <c r="C71" s="107">
+      <c r="B71" s="98">
+        <v>6103</v>
+      </c>
+      <c r="C71" s="96">
         <f t="shared" si="20"/>
         <v>3216</v>
       </c>
-      <c r="D71" s="108" t="s">
+      <c r="D71" s="97" t="s">
         <v>88</v>
       </c>
-      <c r="E71" s="106"/>
-      <c r="F71" s="110"/>
+      <c r="F71" s="48"/>
     </row>
     <row r="72" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B72" s="123" t="s">
+      <c r="B72" s="107" t="s">
         <v>99</v>
       </c>
-      <c r="C72" s="124">
+      <c r="C72" s="108">
         <f t="shared" si="20"/>
-        <v>215</v>
-      </c>
-      <c r="D72" s="125" t="s">
-        <v>100</v>
-      </c>
-      <c r="E72" s="126"/>
-      <c r="F72" s="127"/>
+        <v>211</v>
+      </c>
+      <c r="D72" s="109" t="s">
+        <v>97</v>
+      </c>
+      <c r="E72" s="88"/>
+      <c r="F72" s="79"/>
     </row>
     <row r="73" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B73" s="111" t="s">
+      <c r="B73" s="99" t="s">
         <v>94</v>
       </c>
-      <c r="C73" s="107">
+      <c r="C73" s="96">
         <f t="shared" si="20"/>
         <v>3226</v>
       </c>
-      <c r="D73" s="108" t="s">
+      <c r="D73" s="97" t="s">
         <v>93</v>
       </c>
-      <c r="E73" s="106"/>
-      <c r="F73" s="110"/>
+      <c r="F73" s="48"/>
     </row>
     <row r="74" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B74" s="109" t="s">
+      <c r="B74" s="98" t="s">
         <v>89</v>
       </c>
-      <c r="C74" s="107">
+      <c r="C74" s="96">
         <f t="shared" si="20"/>
         <v>256</v>
       </c>
-      <c r="D74" s="108" t="s">
+      <c r="D74" s="97" t="s">
         <v>90</v>
       </c>
-      <c r="E74" s="106"/>
-      <c r="F74" s="110"/>
+      <c r="F74" s="48"/>
     </row>
     <row r="75" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B75" s="112" t="s">
+      <c r="B75" s="100" t="s">
         <v>91</v>
       </c>
-      <c r="C75" s="113">
+      <c r="C75" s="101">
         <v>1024</v>
       </c>
-      <c r="D75" s="114" t="s">
+      <c r="D75" s="102" t="s">
         <v>92</v>
       </c>
-      <c r="E75" s="115"/>
-      <c r="F75" s="116"/>
+      <c r="E75" s="51"/>
+      <c r="F75" s="52"/>
     </row>
     <row r="76" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B76" s="46"/>
-      <c r="C76" s="107"/>
+      <c r="C76" s="96"/>
     </row>
     <row r="77" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B77" s="46"/>

</xml_diff>

<commit_message>
Changes:  - Stop enemies from using their weapon when K9 is on an elevator  - Increased the size of switch pairings data block to 48 bytes.  - Consolidated god-mode code into thekeyboardInputHandlers routine  - Added debug mode to help test levels  - Defined missing size constants  - Updated documentation (for above)
</commit_message>
<xml_diff>
--- a/docs/Memory.xlsx
+++ b/docs/Memory.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\Beeb\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F01BA20F-4944-44A6-8C1D-2D7055F40E06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{368343B8-6635-409F-BB7D-20B0B80A1281}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="19380" windowHeight="20970" xr2:uid="{C0DF3A0D-E6A9-4F13-8EDD-5DE46AD6E0DB}"/>
+    <workbookView xWindow="19110" yWindow="0" windowWidth="19380" windowHeight="20970" xr2:uid="{C0DF3A0D-E6A9-4F13-8EDD-5DE46AD6E0DB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="102">
   <si>
     <t>Quantity</t>
   </si>
@@ -293,9 +293,6 @@
     <t>Level sprite data</t>
   </si>
   <si>
-    <t>4F83</t>
-  </si>
-  <si>
     <t>Level initialization code</t>
   </si>
   <si>
@@ -332,10 +329,19 @@
     <t>Unused memory</t>
   </si>
   <si>
-    <t>56B4</t>
-  </si>
-  <si>
-    <t>6D93</t>
+    <t>4113</t>
+  </si>
+  <si>
+    <t>4F93</t>
+  </si>
+  <si>
+    <t>5678</t>
+  </si>
+  <si>
+    <t>56C4</t>
+  </si>
+  <si>
+    <t>6DA3</t>
   </si>
 </sst>
 </file>
@@ -1019,15 +1025,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="11" fontId="3" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1043,12 +1040,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1084,6 +1075,21 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1430,35 +1436,35 @@
   <sheetData>
     <row r="1" spans="2:18" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="2" spans="2:18" x14ac:dyDescent="0.35">
-      <c r="B2" s="114" t="s">
+      <c r="B2" s="109" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="D2" s="111" t="s">
+      <c r="C2" s="111" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" s="106" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="110" t="s">
+      <c r="E2" s="105" t="s">
         <v>22</v>
       </c>
-      <c r="F2" s="113"/>
-      <c r="G2" s="110" t="s">
+      <c r="F2" s="108"/>
+      <c r="G2" s="105" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="111"/>
-      <c r="I2" s="112" t="s">
+      <c r="H2" s="106"/>
+      <c r="I2" s="107" t="s">
         <v>12</v>
       </c>
-      <c r="J2" s="113"/>
-      <c r="K2" s="110" t="s">
+      <c r="J2" s="108"/>
+      <c r="K2" s="105" t="s">
         <v>14</v>
       </c>
-      <c r="L2" s="111"/>
-      <c r="M2" s="112" t="s">
+      <c r="L2" s="106"/>
+      <c r="M2" s="107" t="s">
         <v>15</v>
       </c>
-      <c r="N2" s="113"/>
+      <c r="N2" s="108"/>
       <c r="O2" s="43" t="s">
         <v>6</v>
       </c>
@@ -1469,35 +1475,35 @@
       <c r="R2" s="15"/>
     </row>
     <row r="3" spans="2:18" x14ac:dyDescent="0.35">
-      <c r="B3" s="115"/>
-      <c r="C3" s="117"/>
-      <c r="D3" s="118"/>
-      <c r="E3" s="117" t="s">
+      <c r="B3" s="110"/>
+      <c r="C3" s="112"/>
+      <c r="D3" s="113"/>
+      <c r="E3" s="112" t="s">
         <v>23</v>
       </c>
-      <c r="F3" s="119"/>
-      <c r="G3" s="117" t="s">
+      <c r="F3" s="114"/>
+      <c r="G3" s="112" t="s">
         <v>23</v>
       </c>
-      <c r="H3" s="118"/>
+      <c r="H3" s="113"/>
       <c r="I3" s="41"/>
       <c r="J3" s="40"/>
-      <c r="K3" s="117" t="s">
+      <c r="K3" s="112" t="s">
         <v>23</v>
       </c>
-      <c r="L3" s="118"/>
-      <c r="M3" s="119" t="s">
+      <c r="L3" s="113"/>
+      <c r="M3" s="114" t="s">
         <v>23</v>
       </c>
-      <c r="N3" s="119"/>
+      <c r="N3" s="114"/>
       <c r="O3" s="42"/>
       <c r="P3" s="24"/>
       <c r="R3" s="15"/>
     </row>
     <row r="4" spans="2:18" x14ac:dyDescent="0.35">
-      <c r="B4" s="115"/>
-      <c r="C4" s="117"/>
-      <c r="D4" s="118"/>
+      <c r="B4" s="110"/>
+      <c r="C4" s="112"/>
+      <c r="D4" s="113"/>
       <c r="E4" s="21" t="s">
         <v>0</v>
       </c>
@@ -2822,20 +2828,20 @@
       <c r="D60" s="17"/>
     </row>
     <row r="61" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B61" s="103" t="s">
+      <c r="B61" s="100" t="s">
         <v>7</v>
       </c>
       <c r="C61" s="61" t="s">
         <v>20</v>
       </c>
-      <c r="D61" s="104" t="s">
+      <c r="D61" s="101" t="s">
         <v>8</v>
       </c>
       <c r="E61" s="53"/>
       <c r="F61" s="54"/>
     </row>
     <row r="62" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B62" s="98">
+      <c r="B62" s="115">
         <v>4000</v>
       </c>
       <c r="C62" s="96">
@@ -2848,7 +2854,7 @@
       <c r="F62" s="48"/>
     </row>
     <row r="63" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B63" s="98">
+      <c r="B63" s="115">
         <v>4002</v>
       </c>
       <c r="C63" s="96">
@@ -2861,7 +2867,7 @@
       <c r="F63" s="48"/>
     </row>
     <row r="64" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B64" s="98" t="s">
+      <c r="B64" s="115" t="s">
         <v>80</v>
       </c>
       <c r="C64" s="96">
@@ -2874,7 +2880,7 @@
       <c r="F64" s="48"/>
     </row>
     <row r="65" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B65" s="98">
+      <c r="B65" s="115">
         <v>4023</v>
       </c>
       <c r="C65" s="96">
@@ -2887,12 +2893,12 @@
       <c r="F65" s="48"/>
     </row>
     <row r="66" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B66" s="99" t="s">
-        <v>96</v>
+      <c r="B66" s="116" t="s">
+        <v>95</v>
       </c>
       <c r="C66" s="96">
         <f t="shared" si="20"/>
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="D66" s="97" t="s">
         <v>83</v>
@@ -2900,8 +2906,8 @@
       <c r="F66" s="48"/>
     </row>
     <row r="67" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B67" s="98">
-        <v>4103</v>
+      <c r="B67" s="115" t="s">
+        <v>97</v>
       </c>
       <c r="C67" s="96">
         <f t="shared" si="20"/>
@@ -2913,106 +2919,106 @@
       <c r="F67" s="48"/>
     </row>
     <row r="68" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B68" s="98" t="s">
-        <v>85</v>
+      <c r="B68" s="115" t="s">
+        <v>98</v>
       </c>
       <c r="C68" s="96">
         <f t="shared" si="20"/>
         <v>1765</v>
       </c>
       <c r="D68" s="97" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F68" s="48"/>
     </row>
     <row r="69" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B69" s="98">
-        <v>5668</v>
+      <c r="B69" s="115" t="s">
+        <v>99</v>
       </c>
       <c r="C69" s="96">
         <f t="shared" si="20"/>
         <v>76</v>
       </c>
       <c r="D69" s="97" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F69" s="48"/>
     </row>
     <row r="70" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B70" s="106" t="s">
-        <v>98</v>
+      <c r="B70" s="117" t="s">
+        <v>100</v>
       </c>
       <c r="C70" s="96">
         <f t="shared" si="20"/>
         <v>2639</v>
       </c>
-      <c r="D70" s="105" t="s">
-        <v>95</v>
+      <c r="D70" s="102" t="s">
+        <v>94</v>
       </c>
       <c r="F70" s="48"/>
     </row>
     <row r="71" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B71" s="98">
-        <v>6103</v>
+      <c r="B71" s="115">
+        <v>6113</v>
       </c>
       <c r="C71" s="96">
         <f t="shared" si="20"/>
         <v>3216</v>
       </c>
       <c r="D71" s="97" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F71" s="48"/>
     </row>
     <row r="72" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B72" s="107" t="s">
-        <v>99</v>
-      </c>
-      <c r="C72" s="108">
+      <c r="B72" s="118" t="s">
+        <v>101</v>
+      </c>
+      <c r="C72" s="103">
         <f t="shared" si="20"/>
-        <v>211</v>
-      </c>
-      <c r="D72" s="109" t="s">
-        <v>97</v>
+        <v>195</v>
+      </c>
+      <c r="D72" s="104" t="s">
+        <v>96</v>
       </c>
       <c r="E72" s="88"/>
       <c r="F72" s="79"/>
     </row>
     <row r="73" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B73" s="99" t="s">
-        <v>94</v>
+      <c r="B73" s="116" t="s">
+        <v>93</v>
       </c>
       <c r="C73" s="96">
         <f t="shared" si="20"/>
         <v>3226</v>
       </c>
       <c r="D73" s="97" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F73" s="48"/>
     </row>
     <row r="74" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B74" s="98" t="s">
-        <v>89</v>
+      <c r="B74" s="115" t="s">
+        <v>88</v>
       </c>
       <c r="C74" s="96">
         <f t="shared" si="20"/>
         <v>256</v>
       </c>
       <c r="D74" s="97" t="s">
+        <v>89</v>
+      </c>
+      <c r="F74" s="48"/>
+    </row>
+    <row r="75" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B75" s="119" t="s">
         <v>90</v>
       </c>
-      <c r="F74" s="48"/>
-    </row>
-    <row r="75" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B75" s="100" t="s">
+      <c r="C75" s="98">
+        <v>1024</v>
+      </c>
+      <c r="D75" s="99" t="s">
         <v>91</v>
-      </c>
-      <c r="C75" s="101">
-        <v>1024</v>
-      </c>
-      <c r="D75" s="102" t="s">
-        <v>92</v>
       </c>
       <c r="E75" s="51"/>
       <c r="F75" s="52"/>

</xml_diff>

<commit_message>
Two changes:  - Animate key bindings on instructions screen  - The movement sound can now be toggled on and off using the 'T' key  - Updated documentation
</commit_message>
<xml_diff>
--- a/docs/Memory.xlsx
+++ b/docs/Memory.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\Beeb\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\Beeb\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{368343B8-6635-409F-BB7D-20B0B80A1281}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{514D7200-570F-432B-9D25-AD6ACB55E3E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19110" yWindow="0" windowWidth="19380" windowHeight="20970" xr2:uid="{C0DF3A0D-E6A9-4F13-8EDD-5DE46AD6E0DB}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="12660" windowHeight="16010" xr2:uid="{C0DF3A0D-E6A9-4F13-8EDD-5DE46AD6E0DB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="101">
   <si>
     <t>Quantity</t>
   </si>
@@ -317,9 +317,6 @@
     <t>PCM load buffer</t>
   </si>
   <si>
-    <t>6E66</t>
-  </si>
-  <si>
     <t>Titles, interstitial, or finale</t>
   </si>
   <si>
@@ -335,13 +332,13 @@
     <t>4F93</t>
   </si>
   <si>
-    <t>5678</t>
-  </si>
-  <si>
     <t>56C4</t>
   </si>
   <si>
     <t>6DA3</t>
+  </si>
+  <si>
+    <t>6DF3</t>
   </si>
 </sst>
 </file>
@@ -1046,6 +1043,21 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1075,21 +1087,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1436,35 +1433,35 @@
   <sheetData>
     <row r="1" spans="2:18" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="2" spans="2:18" x14ac:dyDescent="0.35">
-      <c r="B2" s="109" t="s">
+      <c r="B2" s="114" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="111" t="s">
-        <v>0</v>
-      </c>
-      <c r="D2" s="106" t="s">
+      <c r="C2" s="116" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" s="111" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="105" t="s">
+      <c r="E2" s="110" t="s">
         <v>22</v>
       </c>
-      <c r="F2" s="108"/>
-      <c r="G2" s="105" t="s">
+      <c r="F2" s="113"/>
+      <c r="G2" s="110" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="106"/>
-      <c r="I2" s="107" t="s">
+      <c r="H2" s="111"/>
+      <c r="I2" s="112" t="s">
         <v>12</v>
       </c>
-      <c r="J2" s="108"/>
-      <c r="K2" s="105" t="s">
+      <c r="J2" s="113"/>
+      <c r="K2" s="110" t="s">
         <v>14</v>
       </c>
-      <c r="L2" s="106"/>
-      <c r="M2" s="107" t="s">
+      <c r="L2" s="111"/>
+      <c r="M2" s="112" t="s">
         <v>15</v>
       </c>
-      <c r="N2" s="108"/>
+      <c r="N2" s="113"/>
       <c r="O2" s="43" t="s">
         <v>6</v>
       </c>
@@ -1475,35 +1472,35 @@
       <c r="R2" s="15"/>
     </row>
     <row r="3" spans="2:18" x14ac:dyDescent="0.35">
-      <c r="B3" s="110"/>
-      <c r="C3" s="112"/>
-      <c r="D3" s="113"/>
-      <c r="E3" s="112" t="s">
+      <c r="B3" s="115"/>
+      <c r="C3" s="117"/>
+      <c r="D3" s="118"/>
+      <c r="E3" s="117" t="s">
         <v>23</v>
       </c>
-      <c r="F3" s="114"/>
-      <c r="G3" s="112" t="s">
+      <c r="F3" s="119"/>
+      <c r="G3" s="117" t="s">
         <v>23</v>
       </c>
-      <c r="H3" s="113"/>
+      <c r="H3" s="118"/>
       <c r="I3" s="41"/>
       <c r="J3" s="40"/>
-      <c r="K3" s="112" t="s">
+      <c r="K3" s="117" t="s">
         <v>23</v>
       </c>
-      <c r="L3" s="113"/>
-      <c r="M3" s="114" t="s">
+      <c r="L3" s="118"/>
+      <c r="M3" s="119" t="s">
         <v>23</v>
       </c>
-      <c r="N3" s="114"/>
+      <c r="N3" s="119"/>
       <c r="O3" s="42"/>
       <c r="P3" s="24"/>
       <c r="R3" s="15"/>
     </row>
     <row r="4" spans="2:18" x14ac:dyDescent="0.35">
-      <c r="B4" s="110"/>
-      <c r="C4" s="112"/>
-      <c r="D4" s="113"/>
+      <c r="B4" s="115"/>
+      <c r="C4" s="117"/>
+      <c r="D4" s="118"/>
       <c r="E4" s="21" t="s">
         <v>0</v>
       </c>
@@ -2841,7 +2838,7 @@
       <c r="F61" s="54"/>
     </row>
     <row r="62" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B62" s="115">
+      <c r="B62" s="105">
         <v>4000</v>
       </c>
       <c r="C62" s="96">
@@ -2854,7 +2851,7 @@
       <c r="F62" s="48"/>
     </row>
     <row r="63" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B63" s="115">
+      <c r="B63" s="105">
         <v>4002</v>
       </c>
       <c r="C63" s="96">
@@ -2867,7 +2864,7 @@
       <c r="F63" s="48"/>
     </row>
     <row r="64" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B64" s="115" t="s">
+      <c r="B64" s="105" t="s">
         <v>80</v>
       </c>
       <c r="C64" s="96">
@@ -2880,7 +2877,7 @@
       <c r="F64" s="48"/>
     </row>
     <row r="65" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B65" s="115">
+      <c r="B65" s="105">
         <v>4023</v>
       </c>
       <c r="C65" s="96">
@@ -2893,8 +2890,8 @@
       <c r="F65" s="48"/>
     </row>
     <row r="66" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B66" s="116" t="s">
-        <v>95</v>
+      <c r="B66" s="106" t="s">
+        <v>94</v>
       </c>
       <c r="C66" s="96">
         <f t="shared" si="20"/>
@@ -2906,8 +2903,8 @@
       <c r="F66" s="48"/>
     </row>
     <row r="67" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B67" s="115" t="s">
-        <v>97</v>
+      <c r="B67" s="105" t="s">
+        <v>96</v>
       </c>
       <c r="C67" s="96">
         <f t="shared" si="20"/>
@@ -2919,8 +2916,8 @@
       <c r="F67" s="48"/>
     </row>
     <row r="68" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B68" s="115" t="s">
-        <v>98</v>
+      <c r="B68" s="105" t="s">
+        <v>97</v>
       </c>
       <c r="C68" s="96">
         <f t="shared" si="20"/>
@@ -2932,8 +2929,8 @@
       <c r="F68" s="48"/>
     </row>
     <row r="69" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B69" s="115" t="s">
-        <v>99</v>
+      <c r="B69" s="105">
+        <v>5678</v>
       </c>
       <c r="C69" s="96">
         <f t="shared" si="20"/>
@@ -2945,25 +2942,25 @@
       <c r="F69" s="48"/>
     </row>
     <row r="70" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B70" s="117" t="s">
-        <v>100</v>
+      <c r="B70" s="107" t="s">
+        <v>98</v>
       </c>
       <c r="C70" s="96">
         <f t="shared" si="20"/>
-        <v>2639</v>
+        <v>2707</v>
       </c>
       <c r="D70" s="102" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F70" s="48"/>
     </row>
     <row r="71" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B71" s="115">
-        <v>6113</v>
+      <c r="B71" s="105">
+        <v>6157</v>
       </c>
       <c r="C71" s="96">
         <f t="shared" si="20"/>
-        <v>3216</v>
+        <v>3148</v>
       </c>
       <c r="D71" s="97" t="s">
         <v>87</v>
@@ -2971,26 +2968,26 @@
       <c r="F71" s="48"/>
     </row>
     <row r="72" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B72" s="118" t="s">
-        <v>101</v>
+      <c r="B72" s="108" t="s">
+        <v>99</v>
       </c>
       <c r="C72" s="103">
         <f t="shared" si="20"/>
-        <v>195</v>
+        <v>80</v>
       </c>
       <c r="D72" s="104" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E72" s="88"/>
       <c r="F72" s="79"/>
     </row>
     <row r="73" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B73" s="116" t="s">
-        <v>93</v>
+      <c r="B73" s="106" t="s">
+        <v>100</v>
       </c>
       <c r="C73" s="96">
         <f t="shared" si="20"/>
-        <v>3226</v>
+        <v>3341</v>
       </c>
       <c r="D73" s="97" t="s">
         <v>92</v>
@@ -2998,7 +2995,7 @@
       <c r="F73" s="48"/>
     </row>
     <row r="74" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B74" s="115" t="s">
+      <c r="B74" s="105" t="s">
         <v>88</v>
       </c>
       <c r="C74" s="96">
@@ -3011,7 +3008,7 @@
       <c r="F74" s="48"/>
     </row>
     <row r="75" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B75" s="119" t="s">
+      <c r="B75" s="109" t="s">
         <v>90</v>
       </c>
       <c r="C75" s="98">

</xml_diff>

<commit_message>
Removed unnecessary OS Vector reset code that prevented the game from running on the BBC Master.  Also fixed an issue where K9 could get stuck... resolved by enabling K9's laser at low health/battery levels. Also updated docs.
</commit_message>
<xml_diff>
--- a/docs/Memory.xlsx
+++ b/docs/Memory.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\Beeb\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\Beeb\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{514D7200-570F-432B-9D25-AD6ACB55E3E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29EFD09E-F193-473D-B062-CCB09E19EE2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="12660" windowHeight="16010" xr2:uid="{C0DF3A0D-E6A9-4F13-8EDD-5DE46AD6E0DB}"/>
+    <workbookView xWindow="11230" yWindow="2210" windowWidth="22000" windowHeight="19990" xr2:uid="{C0DF3A0D-E6A9-4F13-8EDD-5DE46AD6E0DB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -335,10 +335,10 @@
     <t>56C4</t>
   </si>
   <si>
-    <t>6DA3</t>
-  </si>
-  <si>
     <t>6DF3</t>
+  </si>
+  <si>
+    <t>6DBE</t>
   </si>
 </sst>
 </file>
@@ -2947,7 +2947,7 @@
       </c>
       <c r="C70" s="96">
         <f t="shared" si="20"/>
-        <v>2707</v>
+        <v>2654</v>
       </c>
       <c r="D70" s="102" t="s">
         <v>93</v>
@@ -2956,11 +2956,11 @@
     </row>
     <row r="71" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B71" s="105">
-        <v>6157</v>
+        <v>6122</v>
       </c>
       <c r="C71" s="96">
         <f t="shared" si="20"/>
-        <v>3148</v>
+        <v>3228</v>
       </c>
       <c r="D71" s="97" t="s">
         <v>87</v>
@@ -2969,11 +2969,11 @@
     </row>
     <row r="72" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B72" s="108" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C72" s="103">
         <f t="shared" si="20"/>
-        <v>80</v>
+        <v>53</v>
       </c>
       <c r="D72" s="104" t="s">
         <v>95</v>
@@ -2983,7 +2983,7 @@
     </row>
     <row r="73" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B73" s="106" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C73" s="96">
         <f t="shared" si="20"/>

</xml_diff>

<commit_message>
Changes to support the Model B+, at least on BeebEm.  Also updated documentation
</commit_message>
<xml_diff>
--- a/docs/Memory.xlsx
+++ b/docs/Memory.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\Beeb\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29EFD09E-F193-473D-B062-CCB09E19EE2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0E408FA-D27F-4CC0-BD4E-8DECEA286A4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11230" yWindow="2210" windowWidth="22000" windowHeight="19990" xr2:uid="{C0DF3A0D-E6A9-4F13-8EDD-5DE46AD6E0DB}"/>
+    <workbookView xWindow="1080" yWindow="1500" windowWidth="22000" windowHeight="19990" xr2:uid="{C0DF3A0D-E6A9-4F13-8EDD-5DE46AD6E0DB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -338,7 +338,7 @@
     <t>6DF3</t>
   </si>
   <si>
-    <t>6DBE</t>
+    <t>6DC1</t>
   </si>
 </sst>
 </file>
@@ -2947,7 +2947,7 @@
       </c>
       <c r="C70" s="96">
         <f t="shared" si="20"/>
-        <v>2654</v>
+        <v>2657</v>
       </c>
       <c r="D70" s="102" t="s">
         <v>93</v>
@@ -2956,7 +2956,7 @@
     </row>
     <row r="71" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B71" s="105">
-        <v>6122</v>
+        <v>6125</v>
       </c>
       <c r="C71" s="96">
         <f t="shared" si="20"/>
@@ -2973,7 +2973,7 @@
       </c>
       <c r="C72" s="103">
         <f t="shared" si="20"/>
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D72" s="104" t="s">
         <v>95</v>

</xml_diff>

<commit_message>
Reduced the weapon range for Weeping Angels as they use their teeth!
</commit_message>
<xml_diff>
--- a/docs/Memory.xlsx
+++ b/docs/Memory.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\Beeb\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0E408FA-D27F-4CC0-BD4E-8DECEA286A4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CE1A301-3054-4F50-8ED3-AA33F6301278}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1080" yWindow="1500" windowWidth="22000" windowHeight="19990" xr2:uid="{C0DF3A0D-E6A9-4F13-8EDD-5DE46AD6E0DB}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="19380" windowHeight="20970" xr2:uid="{C0DF3A0D-E6A9-4F13-8EDD-5DE46AD6E0DB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -320,25 +320,25 @@
     <t>Titles, interstitial, or finale</t>
   </si>
   <si>
+    <t>Unused memory</t>
+  </si>
+  <si>
+    <t>6E66</t>
+  </si>
+  <si>
     <t>40E3</t>
   </si>
   <si>
-    <t>Unused memory</t>
-  </si>
-  <si>
-    <t>4113</t>
-  </si>
-  <si>
     <t>4F93</t>
   </si>
   <si>
-    <t>56C4</t>
-  </si>
-  <si>
-    <t>6DF3</t>
-  </si>
-  <si>
-    <t>6DC1</t>
+    <t>56AC</t>
+  </si>
+  <si>
+    <t>60F9</t>
+  </si>
+  <si>
+    <t>6D95</t>
   </si>
 </sst>
 </file>
@@ -797,7 +797,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="120">
+  <cellXfs count="121">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1056,6 +1056,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="11" fontId="3" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1433,35 +1436,35 @@
   <sheetData>
     <row r="1" spans="2:18" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="2" spans="2:18" x14ac:dyDescent="0.35">
-      <c r="B2" s="114" t="s">
+      <c r="B2" s="115" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="116" t="s">
-        <v>0</v>
-      </c>
-      <c r="D2" s="111" t="s">
+      <c r="C2" s="117" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" s="112" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="110" t="s">
+      <c r="E2" s="111" t="s">
         <v>22</v>
       </c>
-      <c r="F2" s="113"/>
-      <c r="G2" s="110" t="s">
+      <c r="F2" s="114"/>
+      <c r="G2" s="111" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="111"/>
-      <c r="I2" s="112" t="s">
+      <c r="H2" s="112"/>
+      <c r="I2" s="113" t="s">
         <v>12</v>
       </c>
-      <c r="J2" s="113"/>
-      <c r="K2" s="110" t="s">
+      <c r="J2" s="114"/>
+      <c r="K2" s="111" t="s">
         <v>14</v>
       </c>
-      <c r="L2" s="111"/>
-      <c r="M2" s="112" t="s">
+      <c r="L2" s="112"/>
+      <c r="M2" s="113" t="s">
         <v>15</v>
       </c>
-      <c r="N2" s="113"/>
+      <c r="N2" s="114"/>
       <c r="O2" s="43" t="s">
         <v>6</v>
       </c>
@@ -1472,35 +1475,35 @@
       <c r="R2" s="15"/>
     </row>
     <row r="3" spans="2:18" x14ac:dyDescent="0.35">
-      <c r="B3" s="115"/>
-      <c r="C3" s="117"/>
-      <c r="D3" s="118"/>
-      <c r="E3" s="117" t="s">
+      <c r="B3" s="116"/>
+      <c r="C3" s="118"/>
+      <c r="D3" s="119"/>
+      <c r="E3" s="118" t="s">
         <v>23</v>
       </c>
-      <c r="F3" s="119"/>
-      <c r="G3" s="117" t="s">
+      <c r="F3" s="120"/>
+      <c r="G3" s="118" t="s">
         <v>23</v>
       </c>
-      <c r="H3" s="118"/>
+      <c r="H3" s="119"/>
       <c r="I3" s="41"/>
       <c r="J3" s="40"/>
-      <c r="K3" s="117" t="s">
+      <c r="K3" s="118" t="s">
         <v>23</v>
       </c>
-      <c r="L3" s="118"/>
-      <c r="M3" s="119" t="s">
+      <c r="L3" s="119"/>
+      <c r="M3" s="120" t="s">
         <v>23</v>
       </c>
-      <c r="N3" s="119"/>
+      <c r="N3" s="120"/>
       <c r="O3" s="42"/>
       <c r="P3" s="24"/>
       <c r="R3" s="15"/>
     </row>
     <row r="4" spans="2:18" x14ac:dyDescent="0.35">
-      <c r="B4" s="115"/>
-      <c r="C4" s="117"/>
-      <c r="D4" s="118"/>
+      <c r="B4" s="116"/>
+      <c r="C4" s="118"/>
+      <c r="D4" s="119"/>
       <c r="E4" s="21" t="s">
         <v>0</v>
       </c>
@@ -2891,7 +2894,7 @@
     </row>
     <row r="66" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B66" s="106" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C66" s="96">
         <f t="shared" si="20"/>
@@ -2903,8 +2906,8 @@
       <c r="F66" s="48"/>
     </row>
     <row r="67" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B67" s="105" t="s">
-        <v>96</v>
+      <c r="B67" s="105">
+        <v>4113</v>
       </c>
       <c r="C67" s="96">
         <f t="shared" si="20"/>
@@ -2921,7 +2924,7 @@
       </c>
       <c r="C68" s="96">
         <f t="shared" si="20"/>
-        <v>1765</v>
+        <v>1741</v>
       </c>
       <c r="D68" s="97" t="s">
         <v>85</v>
@@ -2930,7 +2933,7 @@
     </row>
     <row r="69" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B69" s="105">
-        <v>5678</v>
+        <v>5660</v>
       </c>
       <c r="C69" s="96">
         <f t="shared" si="20"/>
@@ -2947,7 +2950,7 @@
       </c>
       <c r="C70" s="96">
         <f t="shared" si="20"/>
-        <v>2657</v>
+        <v>2637</v>
       </c>
       <c r="D70" s="102" t="s">
         <v>93</v>
@@ -2955,8 +2958,8 @@
       <c r="F70" s="48"/>
     </row>
     <row r="71" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B71" s="105">
-        <v>6125</v>
+      <c r="B71" s="105" t="s">
+        <v>99</v>
       </c>
       <c r="C71" s="96">
         <f t="shared" si="20"/>
@@ -2973,21 +2976,21 @@
       </c>
       <c r="C72" s="103">
         <f t="shared" si="20"/>
-        <v>50</v>
+        <v>209</v>
       </c>
       <c r="D72" s="104" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E72" s="88"/>
       <c r="F72" s="79"/>
     </row>
     <row r="73" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B73" s="106" t="s">
-        <v>99</v>
+      <c r="B73" s="110" t="s">
+        <v>95</v>
       </c>
       <c r="C73" s="96">
         <f t="shared" si="20"/>
-        <v>3341</v>
+        <v>3226</v>
       </c>
       <c r="D73" s="97" t="s">
         <v>92</v>

</xml_diff>

<commit_message>
Changes to enable the K9 samples to be played in level 4, the Weeping Angels level.  The sampling code was refactored to acquire and release tone generator 3.
</commit_message>
<xml_diff>
--- a/docs/Memory.xlsx
+++ b/docs/Memory.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\Beeb\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CE1A301-3054-4F50-8ED3-AA33F6301278}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CACFC71B-9793-43CE-9F6F-AED72F2FF867}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-90" yWindow="0" windowWidth="19380" windowHeight="20970" xr2:uid="{C0DF3A0D-E6A9-4F13-8EDD-5DE46AD6E0DB}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="99">
   <si>
     <t>Quantity</t>
   </si>
@@ -191,18 +191,6 @@
     <t>Other Data</t>
   </si>
   <si>
-    <t>game object order</t>
-  </si>
-  <si>
-    <t>10 game objects array</t>
-  </si>
-  <si>
-    <t>Game object order array</t>
-  </si>
-  <si>
-    <t>1 K9 sprites</t>
-  </si>
-  <si>
     <t>MOS ROM workspace</t>
   </si>
   <si>
@@ -332,20 +320,26 @@
     <t>4F93</t>
   </si>
   <si>
-    <t>56AC</t>
-  </si>
-  <si>
-    <t>60F9</t>
-  </si>
-  <si>
-    <t>6D95</t>
+    <t>9 game objects array</t>
+  </si>
+  <si>
+    <t>2 K9 sprites</t>
+  </si>
+  <si>
+    <t>561C</t>
+  </si>
+  <si>
+    <t>60B5</t>
+  </si>
+  <si>
+    <t>6D3A</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -381,6 +375,20 @@
       <name val="Aptos"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -797,7 +805,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="121">
+  <cellXfs count="123">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1049,12 +1057,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1090,6 +1092,18 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1426,7 +1440,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10CD322F-64B0-476A-AEFE-F468CB566666}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="B1:R101"/>
+  <dimension ref="B1:R97"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="2.81640625" customWidth="1"/>
@@ -1436,74 +1450,74 @@
   <sheetData>
     <row r="1" spans="2:18" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="2" spans="2:18" x14ac:dyDescent="0.35">
-      <c r="B2" s="115" t="s">
+      <c r="B2" s="113" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="117" t="s">
-        <v>0</v>
-      </c>
-      <c r="D2" s="112" t="s">
+      <c r="C2" s="115" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" s="110" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="111" t="s">
+      <c r="E2" s="109" t="s">
         <v>22</v>
       </c>
-      <c r="F2" s="114"/>
-      <c r="G2" s="111" t="s">
+      <c r="F2" s="112"/>
+      <c r="G2" s="109" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="112"/>
-      <c r="I2" s="113" t="s">
+      <c r="H2" s="110"/>
+      <c r="I2" s="111" t="s">
         <v>12</v>
       </c>
-      <c r="J2" s="114"/>
-      <c r="K2" s="111" t="s">
+      <c r="J2" s="112"/>
+      <c r="K2" s="109" t="s">
         <v>14</v>
       </c>
-      <c r="L2" s="112"/>
-      <c r="M2" s="113" t="s">
+      <c r="L2" s="110"/>
+      <c r="M2" s="111" t="s">
         <v>15</v>
       </c>
-      <c r="N2" s="114"/>
+      <c r="N2" s="112"/>
       <c r="O2" s="43" t="s">
         <v>6</v>
       </c>
       <c r="P2" s="14" t="str">
-        <f>DEC2HEX(HEX2DEC(3130)-P15)</f>
-        <v>2C30</v>
+        <f>DEC2HEX(HEX2DEC(3130)-P14)</f>
+        <v>2C90</v>
       </c>
       <c r="R2" s="15"/>
     </row>
     <row r="3" spans="2:18" x14ac:dyDescent="0.35">
-      <c r="B3" s="116"/>
-      <c r="C3" s="118"/>
-      <c r="D3" s="119"/>
-      <c r="E3" s="118" t="s">
+      <c r="B3" s="114"/>
+      <c r="C3" s="116"/>
+      <c r="D3" s="117"/>
+      <c r="E3" s="116" t="s">
         <v>23</v>
       </c>
-      <c r="F3" s="120"/>
-      <c r="G3" s="118" t="s">
+      <c r="F3" s="118"/>
+      <c r="G3" s="116" t="s">
         <v>23</v>
       </c>
-      <c r="H3" s="119"/>
+      <c r="H3" s="117"/>
       <c r="I3" s="41"/>
       <c r="J3" s="40"/>
-      <c r="K3" s="118" t="s">
+      <c r="K3" s="116" t="s">
         <v>23</v>
       </c>
-      <c r="L3" s="119"/>
-      <c r="M3" s="120" t="s">
+      <c r="L3" s="117"/>
+      <c r="M3" s="118" t="s">
         <v>23</v>
       </c>
-      <c r="N3" s="120"/>
+      <c r="N3" s="118"/>
       <c r="O3" s="42"/>
       <c r="P3" s="24"/>
       <c r="R3" s="15"/>
     </row>
     <row r="4" spans="2:18" x14ac:dyDescent="0.35">
-      <c r="B4" s="116"/>
-      <c r="C4" s="118"/>
-      <c r="D4" s="119"/>
+      <c r="B4" s="114"/>
+      <c r="C4" s="116"/>
+      <c r="D4" s="117"/>
       <c r="E4" s="21" t="s">
         <v>0</v>
       </c>
@@ -1546,7 +1560,7 @@
         <v>33</v>
       </c>
       <c r="C5" s="9">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D5" s="32">
         <v>48</v>
@@ -1566,11 +1580,11 @@
         <v>0</v>
       </c>
       <c r="I5" s="31">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="J5" s="31">
         <f>I5*$D5</f>
-        <v>480</v>
+        <v>432</v>
       </c>
       <c r="K5" s="35">
         <v>0</v>
@@ -1596,222 +1610,223 @@
     </row>
     <row r="6" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B6" s="1" t="s">
-        <v>51</v>
+        <v>35</v>
       </c>
       <c r="C6" s="19">
+        <v>11</v>
+      </c>
+      <c r="D6" s="5">
+        <f>(24*32/4)</f>
+        <v>192</v>
+      </c>
+      <c r="E6" s="30">
         <v>1</v>
       </c>
-      <c r="D6" s="5">
-        <v>48</v>
-      </c>
-      <c r="E6" s="30">
-        <v>0</v>
-      </c>
       <c r="F6" s="30">
-        <f>E6*$D6</f>
-        <v>0</v>
+        <f t="shared" ref="F6" si="0">E6*$D6</f>
+        <v>192</v>
       </c>
       <c r="G6" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H6" s="5">
-        <f>G6*$D6</f>
-        <v>0</v>
+        <f t="shared" ref="H6:H7" si="1">G6*$D6</f>
+        <v>192</v>
       </c>
       <c r="I6" s="30">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J6" s="30">
-        <f>I6*$D6</f>
-        <v>48</v>
+        <f t="shared" ref="J6" si="2">I6*$D6</f>
+        <v>384</v>
       </c>
       <c r="K6" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L6" s="5">
-        <f>K6*$D6</f>
-        <v>0</v>
+        <f t="shared" ref="L6:L7" si="3">K6*$D6</f>
+        <v>960</v>
       </c>
       <c r="M6" s="30">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N6" s="30">
-        <f>M6*$D6</f>
-        <v>0</v>
+        <f t="shared" ref="N6" si="4">M6*$D6</f>
+        <v>384</v>
       </c>
       <c r="O6" s="4">
         <v>0</v>
       </c>
       <c r="P6" s="6">
-        <f>O6*$D6</f>
+        <f t="shared" ref="P6" si="5">O6*$D6</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B7" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C7" s="19">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="D7" s="5">
-        <f>(24*32/4)</f>
-        <v>192</v>
+        <f>32*4/4</f>
+        <v>32</v>
       </c>
       <c r="E7" s="30">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F7" s="30">
-        <f t="shared" ref="F7" si="0">E7*$D7</f>
-        <v>192</v>
+        <f t="shared" ref="F7:F11" si="6">E7*$D7</f>
+        <v>0</v>
       </c>
       <c r="G7" s="4">
         <v>1</v>
       </c>
       <c r="H7" s="5">
-        <f t="shared" ref="H7:H8" si="1">G7*$D7</f>
-        <v>192</v>
+        <f t="shared" si="1"/>
+        <v>32</v>
       </c>
       <c r="I7" s="30">
+        <v>0</v>
+      </c>
+      <c r="J7" s="30">
+        <f t="shared" ref="J7:J11" si="7">I7*$D7</f>
+        <v>0</v>
+      </c>
+      <c r="K7" s="4">
         <v>2</v>
       </c>
-      <c r="J7" s="30">
-        <f t="shared" ref="J7" si="2">I7*$D7</f>
-        <v>384</v>
-      </c>
-      <c r="K7" s="4">
-        <v>5</v>
-      </c>
       <c r="L7" s="5">
-        <f t="shared" ref="L7:L8" si="3">K7*$D7</f>
-        <v>960</v>
+        <f t="shared" si="3"/>
+        <v>64</v>
       </c>
       <c r="M7" s="30">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N7" s="30">
-        <f t="shared" ref="N7" si="4">M7*$D7</f>
-        <v>384</v>
+        <f t="shared" ref="N7:N11" si="8">M7*$D7</f>
+        <v>32</v>
       </c>
       <c r="O7" s="4">
         <v>0</v>
       </c>
       <c r="P7" s="6">
-        <f t="shared" ref="P7" si="5">O7*$D7</f>
+        <f t="shared" ref="P7:P11" si="9">O7*$D7</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B8" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C8" s="19">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="D8" s="5">
-        <f>32*4/4</f>
-        <v>32</v>
+        <f>(24*16/4)</f>
+        <v>96</v>
       </c>
       <c r="E8" s="30">
         <v>0</v>
       </c>
       <c r="F8" s="30">
-        <f t="shared" ref="F8:F12" si="6">E8*$D8</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="G8" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H8" s="5">
-        <f t="shared" si="1"/>
-        <v>32</v>
+        <f t="shared" ref="H8:H11" si="10">G8*$D8</f>
+        <v>0</v>
       </c>
       <c r="I8" s="30">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J8" s="30">
-        <f t="shared" ref="J8:J12" si="7">I8*$D8</f>
-        <v>0</v>
+        <f t="shared" si="7"/>
+        <v>192</v>
       </c>
       <c r="K8" s="4">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L8" s="5">
-        <f t="shared" si="3"/>
-        <v>64</v>
+        <f t="shared" ref="L8:L11" si="11">K8*$D8</f>
+        <v>0</v>
       </c>
       <c r="M8" s="30">
         <v>1</v>
       </c>
       <c r="N8" s="30">
-        <f t="shared" ref="N8:N12" si="8">M8*$D8</f>
-        <v>32</v>
+        <f t="shared" si="8"/>
+        <v>96</v>
       </c>
       <c r="O8" s="4">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="P8" s="6">
-        <f t="shared" ref="P8:P12" si="9">O8*$D8</f>
-        <v>0</v>
+        <f t="shared" si="9"/>
+        <v>768</v>
       </c>
     </row>
     <row r="9" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B9" s="1" t="s">
-        <v>36</v>
+        <v>55</v>
       </c>
       <c r="C9" s="19">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="D9" s="5">
-        <f>(24*16/4)</f>
+        <f>32*3/4</f>
+        <v>24</v>
+      </c>
+      <c r="E9" s="30">
+        <v>0</v>
+      </c>
+      <c r="F9" s="30">
+        <f>E9*$D9</f>
+        <v>0</v>
+      </c>
+      <c r="G9" s="4">
+        <v>0</v>
+      </c>
+      <c r="H9" s="5">
+        <f>G9*$D9</f>
+        <v>0</v>
+      </c>
+      <c r="I9" s="30">
+        <v>0</v>
+      </c>
+      <c r="J9" s="30">
+        <f>I9*$D9</f>
+        <v>0</v>
+      </c>
+      <c r="K9" s="4">
+        <v>0</v>
+      </c>
+      <c r="L9" s="5">
+        <f>K9*$D9</f>
+        <v>0</v>
+      </c>
+      <c r="M9" s="30">
+        <v>0</v>
+      </c>
+      <c r="N9" s="30">
+        <f>M9*$D9</f>
+        <v>0</v>
+      </c>
+      <c r="O9" s="4">
+        <v>4</v>
+      </c>
+      <c r="P9" s="6">
+        <f>O9*$D9</f>
         <v>96</v>
-      </c>
-      <c r="E9" s="30">
-        <v>0</v>
-      </c>
-      <c r="F9" s="30">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="G9" s="4">
-        <v>0</v>
-      </c>
-      <c r="H9" s="5">
-        <f t="shared" ref="H9:H12" si="10">G9*$D9</f>
-        <v>0</v>
-      </c>
-      <c r="I9" s="30">
-        <v>1</v>
-      </c>
-      <c r="J9" s="30">
-        <f t="shared" si="7"/>
-        <v>96</v>
-      </c>
-      <c r="K9" s="4">
-        <v>0</v>
-      </c>
-      <c r="L9" s="5">
-        <f t="shared" ref="L9:L12" si="11">K9*$D9</f>
-        <v>0</v>
-      </c>
-      <c r="M9" s="30">
-        <v>1</v>
-      </c>
-      <c r="N9" s="30">
-        <f t="shared" si="8"/>
-        <v>96</v>
-      </c>
-      <c r="O9" s="4">
-        <v>9</v>
-      </c>
-      <c r="P9" s="6">
-        <f t="shared" si="9"/>
-        <v>864</v>
       </c>
     </row>
     <row r="10" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B10" s="1" t="s">
-        <v>59</v>
+        <v>70</v>
       </c>
       <c r="C10" s="19">
         <v>4</v>
@@ -1865,1014 +1880,991 @@
     </row>
     <row r="11" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B11" s="1" t="s">
-        <v>74</v>
+        <v>37</v>
       </c>
       <c r="C11" s="19">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D11" s="5">
-        <f>32*3/4</f>
-        <v>24</v>
+        <v>224</v>
       </c>
       <c r="E11" s="30">
         <v>0</v>
       </c>
       <c r="F11" s="30">
-        <f>E11*$D11</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="G11" s="4">
         <v>0</v>
       </c>
       <c r="H11" s="5">
-        <f>G11*$D11</f>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="I11" s="30">
         <v>0</v>
       </c>
       <c r="J11" s="30">
-        <f>I11*$D11</f>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="K11" s="4">
         <v>0</v>
       </c>
       <c r="L11" s="5">
-        <f>K11*$D11</f>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="M11" s="30">
         <v>0</v>
       </c>
       <c r="N11" s="30">
-        <f>M11*$D11</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="O11" s="4">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="P11" s="6">
-        <f>O11*$D11</f>
-        <v>96</v>
+        <f t="shared" si="9"/>
+        <v>224</v>
       </c>
     </row>
     <row r="12" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B12" s="1" t="s">
-        <v>37</v>
+        <v>11</v>
       </c>
       <c r="C12" s="19">
         <v>1</v>
       </c>
       <c r="D12" s="5">
-        <v>224</v>
+        <v>32</v>
       </c>
       <c r="E12" s="30">
         <v>0</v>
       </c>
       <c r="F12" s="30">
-        <f t="shared" si="6"/>
+        <f>E12*$D12</f>
         <v>0</v>
       </c>
       <c r="G12" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H12" s="5">
-        <f t="shared" si="10"/>
-        <v>0</v>
+        <f>G12*$D12</f>
+        <v>32</v>
       </c>
       <c r="I12" s="30">
         <v>0</v>
       </c>
       <c r="J12" s="30">
-        <f t="shared" si="7"/>
+        <f>I12*$D12</f>
         <v>0</v>
       </c>
       <c r="K12" s="4">
         <v>0</v>
       </c>
       <c r="L12" s="5">
-        <f t="shared" si="11"/>
+        <f>K12*$D12</f>
         <v>0</v>
       </c>
       <c r="M12" s="30">
         <v>0</v>
       </c>
       <c r="N12" s="30">
-        <f t="shared" si="8"/>
+        <f>M12*$D12</f>
         <v>0</v>
       </c>
       <c r="O12" s="4">
+        <v>0</v>
+      </c>
+      <c r="P12" s="6">
+        <f>O12*$D12</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="2:18" x14ac:dyDescent="0.35">
+      <c r="B13" s="38" t="s">
+        <v>65</v>
+      </c>
+      <c r="C13" s="34">
         <v>1</v>
       </c>
-      <c r="P12" s="6">
-        <f t="shared" si="9"/>
-        <v>224</v>
-      </c>
-    </row>
-    <row r="13" spans="2:18" x14ac:dyDescent="0.35">
-      <c r="B13" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C13" s="19">
+      <c r="D13" s="8">
+        <v>16</v>
+      </c>
+      <c r="E13" s="33">
+        <v>0</v>
+      </c>
+      <c r="F13" s="33">
+        <f t="shared" ref="F13" si="12">E13*$D13</f>
+        <v>0</v>
+      </c>
+      <c r="G13" s="7">
+        <v>0</v>
+      </c>
+      <c r="H13" s="8">
+        <f t="shared" ref="H13" si="13">G13*$D13</f>
+        <v>0</v>
+      </c>
+      <c r="I13" s="33">
         <v>1</v>
       </c>
-      <c r="D13" s="5">
-        <v>32</v>
-      </c>
-      <c r="E13" s="30">
-        <v>0</v>
-      </c>
-      <c r="F13" s="30">
-        <f>E13*$D13</f>
-        <v>0</v>
-      </c>
-      <c r="G13" s="4">
+      <c r="J13" s="33">
+        <f>I13*$D13</f>
+        <v>16</v>
+      </c>
+      <c r="K13" s="7">
+        <v>0</v>
+      </c>
+      <c r="L13" s="8">
+        <f t="shared" ref="L13" si="14">K13*$D13</f>
+        <v>0</v>
+      </c>
+      <c r="M13" s="33">
+        <v>0</v>
+      </c>
+      <c r="N13" s="33">
+        <f t="shared" ref="N13" si="15">M13*$D13</f>
+        <v>0</v>
+      </c>
+      <c r="O13" s="7">
+        <v>0</v>
+      </c>
+      <c r="P13" s="39">
+        <f t="shared" ref="P13" si="16">O13*$D13</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="2:18" x14ac:dyDescent="0.35">
+      <c r="B14" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="H13" s="5">
-        <f>G13*$D13</f>
-        <v>32</v>
-      </c>
-      <c r="I13" s="30">
-        <v>0</v>
-      </c>
-      <c r="J13" s="30">
-        <f>I13*$D13</f>
-        <v>0</v>
-      </c>
-      <c r="K13" s="4">
-        <v>0</v>
-      </c>
-      <c r="L13" s="5">
-        <f>K13*$D13</f>
-        <v>0</v>
-      </c>
-      <c r="M13" s="30">
-        <v>0</v>
-      </c>
-      <c r="N13" s="30">
-        <f>M13*$D13</f>
-        <v>0</v>
-      </c>
-      <c r="O13" s="4">
-        <v>0</v>
-      </c>
-      <c r="P13" s="6">
-        <f>O13*$D13</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="2:18" x14ac:dyDescent="0.35">
-      <c r="B14" s="38" t="s">
-        <v>69</v>
-      </c>
-      <c r="C14" s="34">
-        <v>1</v>
-      </c>
-      <c r="D14" s="8">
-        <v>16</v>
-      </c>
-      <c r="E14" s="33">
-        <v>0</v>
-      </c>
-      <c r="F14" s="33">
-        <f t="shared" ref="F14" si="12">E14*$D14</f>
-        <v>0</v>
-      </c>
-      <c r="G14" s="7">
-        <v>0</v>
-      </c>
-      <c r="H14" s="8">
-        <f t="shared" ref="H14" si="13">G14*$D14</f>
-        <v>0</v>
-      </c>
-      <c r="I14" s="33">
-        <v>1</v>
-      </c>
-      <c r="J14" s="33">
-        <f>I14*$D14</f>
-        <v>16</v>
-      </c>
-      <c r="K14" s="7">
-        <v>0</v>
-      </c>
-      <c r="L14" s="8">
-        <f t="shared" ref="L14" si="14">K14*$D14</f>
-        <v>0</v>
-      </c>
-      <c r="M14" s="33">
-        <v>0</v>
-      </c>
-      <c r="N14" s="33">
-        <f t="shared" ref="N14" si="15">M14*$D14</f>
-        <v>0</v>
-      </c>
-      <c r="O14" s="7">
-        <v>0</v>
-      </c>
-      <c r="P14" s="39">
-        <f t="shared" ref="P14" si="16">O14*$D14</f>
-        <v>0</v>
+      <c r="C14" s="19"/>
+      <c r="D14" s="20"/>
+      <c r="E14" s="28"/>
+      <c r="F14" s="28">
+        <f>SUM(F5:F13)</f>
+        <v>192</v>
+      </c>
+      <c r="G14" s="19"/>
+      <c r="H14" s="20">
+        <f>SUM(H5:H13)</f>
+        <v>256</v>
+      </c>
+      <c r="I14" s="28"/>
+      <c r="J14" s="28">
+        <f>SUM(J5:J13)</f>
+        <v>1024</v>
+      </c>
+      <c r="K14" s="19"/>
+      <c r="L14" s="20">
+        <f>SUM(L5:L13)</f>
+        <v>1024</v>
+      </c>
+      <c r="M14" s="28"/>
+      <c r="N14" s="28">
+        <f>SUM(N5:N13)</f>
+        <v>512</v>
+      </c>
+      <c r="O14" s="19"/>
+      <c r="P14" s="29">
+        <f>SUM(P5:P13)</f>
+        <v>1184</v>
       </c>
     </row>
     <row r="15" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B15" s="18" t="s">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="C15" s="19"/>
       <c r="D15" s="20"/>
       <c r="E15" s="28"/>
-      <c r="F15" s="28">
-        <f>SUM(F5:F14)</f>
+      <c r="F15" s="30">
         <v>192</v>
       </c>
-      <c r="G15" s="19"/>
-      <c r="H15" s="20">
-        <f>SUM(H5:H14)</f>
+      <c r="G15" s="4"/>
+      <c r="H15" s="5">
         <v>256</v>
       </c>
-      <c r="I15" s="28"/>
-      <c r="J15" s="28">
-        <f>SUM(J5:J14)</f>
+      <c r="I15" s="30"/>
+      <c r="J15" s="30">
         <v>1024</v>
       </c>
-      <c r="K15" s="19"/>
-      <c r="L15" s="20">
-        <f>SUM(L5:L14)</f>
+      <c r="K15" s="4"/>
+      <c r="L15" s="5">
         <v>1024</v>
       </c>
-      <c r="M15" s="28"/>
-      <c r="N15" s="28">
-        <f>SUM(N5:N14)</f>
+      <c r="M15" s="30"/>
+      <c r="N15" s="30">
         <v>512</v>
       </c>
-      <c r="O15" s="19"/>
-      <c r="P15" s="29">
-        <f>SUM(P5:P14)</f>
-        <v>1280</v>
-      </c>
-    </row>
-    <row r="16" spans="2:18" x14ac:dyDescent="0.35">
-      <c r="B16" s="18" t="s">
-        <v>16</v>
-      </c>
-      <c r="C16" s="19"/>
-      <c r="D16" s="20"/>
-      <c r="E16" s="28"/>
-      <c r="F16" s="30">
+      <c r="O15" s="4"/>
+      <c r="P15" s="6"/>
+    </row>
+    <row r="16" spans="2:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B16" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C16" s="10"/>
+      <c r="D16" s="11"/>
+      <c r="E16" s="16" t="s">
+        <v>5</v>
+      </c>
+      <c r="F16" s="16">
+        <f>256-F14</f>
+        <v>64</v>
+      </c>
+      <c r="G16" s="10"/>
+      <c r="H16" s="44">
+        <f>H15-H14</f>
+        <v>0</v>
+      </c>
+      <c r="I16" s="12"/>
+      <c r="J16" s="16">
+        <f>J15-J14</f>
+        <v>0</v>
+      </c>
+      <c r="K16" s="10"/>
+      <c r="L16" s="44">
+        <f>L15-L14</f>
+        <v>0</v>
+      </c>
+      <c r="M16" s="12"/>
+      <c r="N16" s="16">
+        <f>N15-N14</f>
+        <v>0</v>
+      </c>
+      <c r="O16" s="10"/>
+      <c r="P16" s="13"/>
+    </row>
+    <row r="17" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="P17" s="3"/>
+    </row>
+    <row r="18" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B18" s="63" t="s">
+        <v>7</v>
+      </c>
+      <c r="C18" s="57" t="s">
+        <v>20</v>
+      </c>
+      <c r="D18" s="64" t="s">
+        <v>8</v>
+      </c>
+      <c r="E18" s="56"/>
+      <c r="F18" s="58"/>
+      <c r="H18" s="59" t="s">
+        <v>50</v>
+      </c>
+      <c r="I18" s="53"/>
+      <c r="J18" s="53"/>
+      <c r="K18" s="60" t="s">
+        <v>7</v>
+      </c>
+      <c r="L18" s="61" t="s">
+        <v>2</v>
+      </c>
+      <c r="M18" s="60" t="s">
+        <v>39</v>
+      </c>
+      <c r="N18" s="53"/>
+      <c r="O18" s="54"/>
+    </row>
+    <row r="19" spans="2:16" x14ac:dyDescent="0.35">
+      <c r="B19" s="62">
+        <v>0</v>
+      </c>
+      <c r="C19" s="65">
+        <v>144</v>
+      </c>
+      <c r="D19" s="56" t="s">
+        <v>66</v>
+      </c>
+      <c r="E19" s="56"/>
+      <c r="F19" s="58"/>
+      <c r="H19" s="47" t="s">
+        <v>38</v>
+      </c>
+      <c r="I19" s="17"/>
+      <c r="K19" t="s">
+        <v>40</v>
+      </c>
+      <c r="L19" s="30">
+        <v>30</v>
+      </c>
+      <c r="M19" t="s">
+        <v>42</v>
+      </c>
+      <c r="O19" s="48"/>
+    </row>
+    <row r="20" spans="2:16" x14ac:dyDescent="0.35">
+      <c r="B20" s="82">
+        <v>90</v>
+      </c>
+      <c r="C20" s="84">
+        <v>112</v>
+      </c>
+      <c r="D20" s="85" t="s">
+        <v>67</v>
+      </c>
+      <c r="E20" s="85"/>
+      <c r="F20" s="83"/>
+      <c r="H20" s="47" t="s">
+        <v>68</v>
+      </c>
+      <c r="I20" s="17"/>
+      <c r="K20" t="s">
+        <v>41</v>
+      </c>
+      <c r="L20" s="30">
+        <v>64</v>
+      </c>
+      <c r="M20" t="s">
+        <v>42</v>
+      </c>
+      <c r="O20" s="48"/>
+    </row>
+    <row r="21" spans="2:16" x14ac:dyDescent="0.35">
+      <c r="B21" s="73">
+        <v>100</v>
+      </c>
+      <c r="C21" s="31">
+        <f>(24*32/4)</f>
         <v>192</v>
       </c>
-      <c r="G16" s="4"/>
-      <c r="H16" s="5">
-        <v>256</v>
-      </c>
-      <c r="I16" s="30"/>
-      <c r="J16" s="30">
-        <v>1024</v>
-      </c>
-      <c r="K16" s="4"/>
-      <c r="L16" s="5">
-        <v>1024</v>
-      </c>
-      <c r="M16" s="30"/>
-      <c r="N16" s="30">
-        <v>512</v>
-      </c>
-      <c r="O16" s="4"/>
-      <c r="P16" s="6"/>
-    </row>
-    <row r="17" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B17" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C17" s="10"/>
-      <c r="D17" s="11"/>
-      <c r="E17" s="16" t="s">
-        <v>5</v>
-      </c>
-      <c r="F17" s="16">
-        <f>256-F15</f>
-        <v>64</v>
-      </c>
-      <c r="G17" s="10"/>
-      <c r="H17" s="44">
-        <f>H16-H15</f>
-        <v>0</v>
-      </c>
-      <c r="I17" s="12"/>
-      <c r="J17" s="16">
-        <f>J16-J15</f>
-        <v>0</v>
-      </c>
-      <c r="K17" s="10"/>
-      <c r="L17" s="44">
-        <f>L16-L15</f>
-        <v>0</v>
-      </c>
-      <c r="M17" s="12"/>
-      <c r="N17" s="16">
-        <f>N16-N15</f>
-        <v>0</v>
-      </c>
-      <c r="O17" s="10"/>
-      <c r="P17" s="13"/>
-    </row>
-    <row r="18" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="P18" s="3"/>
-    </row>
-    <row r="19" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="P19" s="3"/>
-    </row>
-    <row r="20" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B20" s="63" t="s">
-        <v>7</v>
-      </c>
-      <c r="C20" s="57" t="s">
-        <v>20</v>
-      </c>
-      <c r="D20" s="64" t="s">
-        <v>8</v>
-      </c>
-      <c r="E20" s="56"/>
-      <c r="F20" s="58"/>
-      <c r="H20" s="59" t="s">
-        <v>50</v>
-      </c>
-      <c r="I20" s="53"/>
-      <c r="J20" s="53"/>
-      <c r="K20" s="60" t="s">
-        <v>7</v>
-      </c>
-      <c r="L20" s="61" t="s">
-        <v>2</v>
-      </c>
-      <c r="M20" s="60" t="s">
-        <v>39</v>
-      </c>
-      <c r="N20" s="53"/>
-      <c r="O20" s="54"/>
-    </row>
-    <row r="21" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B21" s="62">
-        <v>0</v>
-      </c>
-      <c r="C21" s="65">
-        <v>144</v>
-      </c>
-      <c r="D21" s="56" t="s">
-        <v>70</v>
-      </c>
-      <c r="E21" s="56"/>
-      <c r="F21" s="58"/>
+      <c r="D21" s="80" t="s">
+        <v>24</v>
+      </c>
+      <c r="E21" s="80"/>
+      <c r="F21" s="81"/>
       <c r="H21" s="47" t="s">
-        <v>38</v>
+        <v>69</v>
       </c>
       <c r="I21" s="17"/>
       <c r="K21" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="L21" s="30">
-        <v>30</v>
+        <v>64</v>
       </c>
       <c r="M21" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="O21" s="48"/>
     </row>
     <row r="22" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B22" s="82">
-        <v>90</v>
-      </c>
-      <c r="C22" s="84">
-        <v>112</v>
-      </c>
-      <c r="D22" s="85" t="s">
-        <v>71</v>
-      </c>
-      <c r="E22" s="85"/>
-      <c r="F22" s="83"/>
+      <c r="B22" s="66" t="str">
+        <f t="shared" ref="B22:B47" si="17">DEC2HEX(HEX2DEC(B21)+C21)</f>
+        <v>1C0</v>
+      </c>
+      <c r="C22" s="33">
+        <v>64</v>
+      </c>
+      <c r="D22" s="67" t="s">
+        <v>31</v>
+      </c>
+      <c r="E22" s="68"/>
+      <c r="F22" s="69"/>
       <c r="H22" s="47" t="s">
-        <v>72</v>
+        <v>32</v>
       </c>
       <c r="I22" s="17"/>
       <c r="K22" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="L22" s="30">
-        <v>64</v>
+        <v>44</v>
       </c>
       <c r="M22" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="O22" s="48"/>
     </row>
     <row r="23" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B23" s="73">
-        <v>100</v>
-      </c>
-      <c r="C23" s="31">
-        <f>(24*32/4)</f>
-        <v>192</v>
-      </c>
-      <c r="D23" s="80" t="s">
-        <v>24</v>
-      </c>
-      <c r="E23" s="80"/>
-      <c r="F23" s="81"/>
+      <c r="B23" s="74" t="str">
+        <f t="shared" si="17"/>
+        <v>200</v>
+      </c>
+      <c r="C23" s="75">
+        <v>256</v>
+      </c>
+      <c r="D23" s="76" t="s">
+        <v>9</v>
+      </c>
+      <c r="E23" s="76"/>
+      <c r="F23" s="77"/>
       <c r="H23" s="47" t="s">
-        <v>73</v>
+        <v>45</v>
       </c>
       <c r="I23" s="17"/>
       <c r="K23" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="L23" s="30">
-        <v>64</v>
+        <v>12</v>
       </c>
       <c r="M23" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="O23" s="48"/>
     </row>
-    <row r="24" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B24" s="66" t="str">
-        <f t="shared" ref="B24:B50" si="17">DEC2HEX(HEX2DEC(B23)+C23)</f>
-        <v>1C0</v>
-      </c>
-      <c r="C24" s="33">
-        <v>64</v>
-      </c>
-      <c r="D24" s="67" t="s">
-        <v>31</v>
-      </c>
-      <c r="E24" s="68"/>
-      <c r="F24" s="69"/>
-      <c r="H24" s="47" t="s">
-        <v>32</v>
-      </c>
-      <c r="I24" s="17"/>
-      <c r="K24" t="s">
-        <v>46</v>
-      </c>
-      <c r="L24" s="30">
-        <v>44</v>
-      </c>
-      <c r="M24" t="s">
-        <v>48</v>
-      </c>
-      <c r="O24" s="48"/>
-    </row>
-    <row r="25" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B25" s="74" t="str">
-        <f t="shared" si="17"/>
-        <v>200</v>
-      </c>
-      <c r="C25" s="75">
-        <v>256</v>
-      </c>
-      <c r="D25" s="76" t="s">
-        <v>9</v>
-      </c>
-      <c r="E25" s="76"/>
-      <c r="F25" s="77"/>
-      <c r="H25" s="47" t="s">
-        <v>45</v>
-      </c>
-      <c r="I25" s="17"/>
-      <c r="K25" t="s">
-        <v>47</v>
-      </c>
-      <c r="L25" s="30">
-        <v>12</v>
-      </c>
-      <c r="M25" t="s">
-        <v>49</v>
-      </c>
-      <c r="O25" s="48"/>
-    </row>
-    <row r="26" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B26" s="47" t="str">
+    <row r="24" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B24" s="47" t="str">
         <f t="shared" si="17"/>
         <v>300</v>
       </c>
-      <c r="C26" s="30">
+      <c r="C24" s="30">
         <v>192</v>
       </c>
-      <c r="D26" t="s">
+      <c r="D24" t="s">
         <v>24</v>
       </c>
-      <c r="F26" s="48"/>
-      <c r="H26" s="49" t="s">
+      <c r="F24" s="48"/>
+      <c r="H24" s="49" t="s">
+        <v>57</v>
+      </c>
+      <c r="I24" s="50"/>
+      <c r="J24" s="51"/>
+      <c r="K24" s="50" t="s">
+        <v>58</v>
+      </c>
+      <c r="L24" s="16">
+        <v>20</v>
+      </c>
+      <c r="M24" s="51" t="s">
+        <v>49</v>
+      </c>
+      <c r="N24" s="51"/>
+      <c r="O24" s="52"/>
+    </row>
+    <row r="25" spans="2:16" x14ac:dyDescent="0.35">
+      <c r="B25" s="47" t="str">
+        <f t="shared" si="17"/>
+        <v>3C0</v>
+      </c>
+      <c r="C25" s="30">
+        <f>$D$7</f>
+        <v>32</v>
+      </c>
+      <c r="D25" s="86" t="s">
+        <v>25</v>
+      </c>
+      <c r="F25" s="48"/>
+      <c r="H25" s="17"/>
+      <c r="I25" s="17"/>
+      <c r="K25" s="30"/>
+    </row>
+    <row r="26" spans="2:16" x14ac:dyDescent="0.35">
+      <c r="B26" s="66" t="str">
+        <f t="shared" si="17"/>
+        <v>3E0</v>
+      </c>
+      <c r="C26" s="33">
+        <v>32</v>
+      </c>
+      <c r="D26" s="68" t="s">
         <v>61</v>
       </c>
-      <c r="I26" s="50"/>
-      <c r="J26" s="51"/>
-      <c r="K26" s="50" t="s">
-        <v>62</v>
-      </c>
-      <c r="L26" s="16">
-        <v>20</v>
-      </c>
-      <c r="M26" s="51" t="s">
-        <v>49</v>
-      </c>
-      <c r="N26" s="51"/>
-      <c r="O26" s="52"/>
+      <c r="E26" s="68"/>
+      <c r="F26" s="69"/>
+      <c r="H26" s="17"/>
     </row>
     <row r="27" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B27" s="47" t="str">
         <f t="shared" si="17"/>
-        <v>3C0</v>
+        <v>400</v>
       </c>
       <c r="C27" s="30">
-        <f>$D$8</f>
-        <v>32</v>
-      </c>
-      <c r="D27" s="86" t="s">
-        <v>25</v>
+        <v>432</v>
+      </c>
+      <c r="D27" t="s">
+        <v>94</v>
       </c>
       <c r="F27" s="48"/>
       <c r="H27" s="17"/>
-      <c r="I27" s="17"/>
-      <c r="K27" s="30"/>
+      <c r="I27" s="55"/>
     </row>
     <row r="28" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B28" s="66" t="str">
+      <c r="B28" s="47" t="str">
         <f t="shared" si="17"/>
-        <v>3E0</v>
-      </c>
-      <c r="C28" s="33">
-        <v>32</v>
-      </c>
-      <c r="D28" s="68" t="s">
-        <v>65</v>
-      </c>
-      <c r="E28" s="68"/>
-      <c r="F28" s="69"/>
-      <c r="H28" s="17"/>
+        <v>5B0</v>
+      </c>
+      <c r="C28" s="30">
+        <v>384</v>
+      </c>
+      <c r="D28" t="s">
+        <v>18</v>
+      </c>
+      <c r="F28" s="48"/>
     </row>
     <row r="29" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B29" s="47" t="str">
         <f t="shared" si="17"/>
-        <v>400</v>
+        <v>730</v>
       </c>
       <c r="C29" s="30">
-        <v>480</v>
+        <v>192</v>
       </c>
       <c r="D29" t="s">
-        <v>52</v>
+        <v>95</v>
       </c>
       <c r="F29" s="48"/>
-      <c r="H29" s="17"/>
-      <c r="I29" s="55"/>
     </row>
     <row r="30" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B30" s="47" t="str">
+      <c r="B30" s="66" t="str">
         <f t="shared" si="17"/>
-        <v>5E0</v>
-      </c>
-      <c r="C30" s="30">
-        <v>48</v>
-      </c>
-      <c r="D30" t="s">
-        <v>53</v>
-      </c>
-      <c r="F30" s="48"/>
+        <v>7F0</v>
+      </c>
+      <c r="C30" s="33">
+        <v>16</v>
+      </c>
+      <c r="D30" s="67" t="s">
+        <v>64</v>
+      </c>
+      <c r="E30" s="68"/>
+      <c r="F30" s="69"/>
     </row>
     <row r="31" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B31" s="47" t="str">
+      <c r="B31" s="78" t="str">
         <f t="shared" si="17"/>
-        <v>610</v>
-      </c>
-      <c r="C31" s="30">
-        <v>384</v>
-      </c>
-      <c r="D31" t="s">
-        <v>18</v>
-      </c>
-      <c r="F31" s="48"/>
+        <v>800</v>
+      </c>
+      <c r="C31" s="87">
+        <v>128</v>
+      </c>
+      <c r="D31" s="88" t="s">
+        <v>27</v>
+      </c>
+      <c r="E31" s="88"/>
+      <c r="F31" s="79"/>
     </row>
     <row r="32" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B32" s="47" t="str">
         <f t="shared" si="17"/>
-        <v>790</v>
+        <v>880</v>
       </c>
       <c r="C32" s="30">
-        <v>96</v>
-      </c>
-      <c r="D32" t="s">
-        <v>54</v>
+        <v>64</v>
+      </c>
+      <c r="D32" s="86" t="s">
+        <v>72</v>
       </c>
       <c r="F32" s="48"/>
     </row>
     <row r="33" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B33" s="66" t="str">
-        <f t="shared" si="17"/>
-        <v>7F0</v>
-      </c>
-      <c r="C33" s="33">
-        <v>16</v>
-      </c>
-      <c r="D33" s="67" t="s">
-        <v>68</v>
-      </c>
-      <c r="E33" s="68"/>
-      <c r="F33" s="69"/>
-    </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B34" s="78" t="str">
-        <f t="shared" si="17"/>
-        <v>800</v>
-      </c>
-      <c r="C34" s="87">
-        <v>128</v>
-      </c>
-      <c r="D34" s="88" t="s">
-        <v>27</v>
-      </c>
-      <c r="E34" s="88"/>
-      <c r="F34" s="79"/>
-    </row>
-    <row r="35" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B35" s="47" t="str">
-        <f t="shared" si="17"/>
-        <v>880</v>
-      </c>
-      <c r="C35" s="30">
-        <v>64</v>
-      </c>
-      <c r="D35" s="86" t="s">
-        <v>76</v>
-      </c>
-      <c r="F35" s="48"/>
-    </row>
-    <row r="36" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B36" s="74" t="str">
+      <c r="B33" s="74" t="str">
         <f t="shared" si="17"/>
         <v>8C0</v>
       </c>
-      <c r="C36" s="75">
-        <f>2*$D$8</f>
+      <c r="C33" s="75">
+        <f>2*$D$7</f>
         <v>64</v>
       </c>
-      <c r="D36" s="76" t="s">
+      <c r="D33" s="76" t="s">
         <v>27</v>
       </c>
-      <c r="E36" s="76"/>
-      <c r="F36" s="77"/>
+      <c r="E33" s="76"/>
+      <c r="F33" s="77"/>
+    </row>
+    <row r="34" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B34" s="47" t="str">
+        <f t="shared" si="17"/>
+        <v>900</v>
+      </c>
+      <c r="C34" s="30">
+        <v>960</v>
+      </c>
+      <c r="D34" t="s">
+        <v>17</v>
+      </c>
+      <c r="F34" s="48"/>
+    </row>
+    <row r="35" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B35" s="66" t="str">
+        <f t="shared" si="17"/>
+        <v>CC0</v>
+      </c>
+      <c r="C35" s="33">
+        <v>64</v>
+      </c>
+      <c r="D35" s="68" t="s">
+        <v>26</v>
+      </c>
+      <c r="E35" s="68"/>
+      <c r="F35" s="69"/>
+    </row>
+    <row r="36" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B36" s="47" t="str">
+        <f t="shared" si="17"/>
+        <v>D00</v>
+      </c>
+      <c r="C36" s="30">
+        <v>32</v>
+      </c>
+      <c r="D36" s="86" t="s">
+        <v>60</v>
+      </c>
+      <c r="F36" s="48"/>
     </row>
     <row r="37" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B37" s="47" t="str">
+        <f>DEC2HEX(HEX2DEC(B36)+C36)</f>
+        <v>D20</v>
+      </c>
+      <c r="C37" s="30">
+        <v>64</v>
+      </c>
+      <c r="D37" s="86" t="s">
+        <v>73</v>
+      </c>
+      <c r="F37" s="48"/>
+    </row>
+    <row r="38" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B38" s="74" t="str">
         <f t="shared" si="17"/>
-        <v>900</v>
-      </c>
-      <c r="C37" s="30">
-        <v>960</v>
-      </c>
-      <c r="D37" t="s">
-        <v>17</v>
-      </c>
-      <c r="F37" s="48"/>
-    </row>
-    <row r="38" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B38" s="66" t="str">
-        <f t="shared" si="17"/>
-        <v>CC0</v>
-      </c>
-      <c r="C38" s="33">
-        <v>64</v>
-      </c>
-      <c r="D38" s="68" t="s">
-        <v>26</v>
-      </c>
-      <c r="E38" s="68"/>
-      <c r="F38" s="69"/>
+        <v>D60</v>
+      </c>
+      <c r="C38" s="75">
+        <v>160</v>
+      </c>
+      <c r="D38" s="76" t="s">
+        <v>51</v>
+      </c>
+      <c r="E38" s="76"/>
+      <c r="F38" s="77"/>
     </row>
     <row r="39" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B39" s="47" t="str">
         <f t="shared" si="17"/>
-        <v>D00</v>
+        <v>E00</v>
       </c>
       <c r="C39" s="30">
-        <v>32</v>
+        <v>384</v>
       </c>
       <c r="D39" s="86" t="s">
-        <v>64</v>
+        <v>18</v>
       </c>
       <c r="F39" s="48"/>
     </row>
     <row r="40" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B40" s="47" t="str">
-        <f>DEC2HEX(HEX2DEC(B39)+C39)</f>
-        <v>D20</v>
+        <f t="shared" si="17"/>
+        <v>F80</v>
       </c>
       <c r="C40" s="30">
-        <v>64</v>
+        <v>32</v>
       </c>
       <c r="D40" s="86" t="s">
-        <v>77</v>
+        <v>25</v>
       </c>
       <c r="F40" s="48"/>
     </row>
     <row r="41" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B41" s="74" t="str">
+      <c r="B41" s="66" t="str">
         <f t="shared" si="17"/>
-        <v>D60</v>
-      </c>
-      <c r="C41" s="75">
-        <v>160</v>
-      </c>
-      <c r="D41" s="76" t="s">
-        <v>55</v>
-      </c>
-      <c r="E41" s="76"/>
-      <c r="F41" s="77"/>
+        <v>FA0</v>
+      </c>
+      <c r="C41" s="33">
+        <v>96</v>
+      </c>
+      <c r="D41" s="67" t="s">
+        <v>52</v>
+      </c>
+      <c r="E41" s="68"/>
+      <c r="F41" s="69"/>
     </row>
     <row r="42" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B42" s="47" t="str">
+      <c r="B42" s="78" t="str">
         <f t="shared" si="17"/>
-        <v>E00</v>
-      </c>
-      <c r="C42" s="30">
-        <v>384</v>
-      </c>
-      <c r="D42" s="86" t="s">
-        <v>18</v>
-      </c>
-      <c r="F42" s="48"/>
+        <v>1000</v>
+      </c>
+      <c r="C42" s="87">
+        <v>144</v>
+      </c>
+      <c r="D42" s="89" t="s">
+        <v>21</v>
+      </c>
+      <c r="E42" s="88"/>
+      <c r="F42" s="79"/>
     </row>
     <row r="43" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B43" s="47" t="str">
         <f t="shared" si="17"/>
-        <v>F80</v>
+        <v>1090</v>
       </c>
       <c r="C43" s="30">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="D43" s="86" t="s">
-        <v>25</v>
+        <v>53</v>
       </c>
       <c r="F43" s="48"/>
     </row>
     <row r="44" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B44" s="66" t="str">
-        <f t="shared" si="17"/>
-        <v>FA0</v>
-      </c>
-      <c r="C44" s="33">
-        <v>96</v>
-      </c>
-      <c r="D44" s="67" t="s">
-        <v>56</v>
-      </c>
-      <c r="E44" s="68"/>
-      <c r="F44" s="69"/>
-    </row>
-    <row r="45" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B45" s="78" t="str">
-        <f t="shared" si="17"/>
-        <v>1000</v>
-      </c>
-      <c r="C45" s="87">
-        <v>144</v>
-      </c>
-      <c r="D45" s="89" t="s">
-        <v>21</v>
-      </c>
-      <c r="E45" s="88"/>
-      <c r="F45" s="79"/>
-    </row>
-    <row r="46" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B46" s="47" t="str">
-        <f t="shared" si="17"/>
-        <v>1090</v>
-      </c>
-      <c r="C46" s="30">
-        <v>48</v>
-      </c>
-      <c r="D46" s="86" t="s">
-        <v>57</v>
-      </c>
-      <c r="F46" s="48"/>
-    </row>
-    <row r="47" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B47" s="47" t="str">
+      <c r="B44" s="47" t="str">
         <f t="shared" si="17"/>
         <v>10C0</v>
       </c>
-      <c r="C47" s="30">
+      <c r="C44" s="30">
         <v>32</v>
       </c>
-      <c r="D47" s="86" t="s">
+      <c r="D44" s="86" t="s">
         <v>21</v>
       </c>
-      <c r="F47" s="48"/>
-    </row>
-    <row r="48" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B48" s="47" t="str">
+      <c r="F44" s="48"/>
+    </row>
+    <row r="45" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B45" s="47" t="str">
         <f t="shared" si="17"/>
         <v>10E0</v>
       </c>
-      <c r="C48" s="30">
+      <c r="C45" s="30">
         <v>12</v>
       </c>
-      <c r="D48" s="86" t="s">
-        <v>63</v>
-      </c>
-      <c r="F48" s="48"/>
-    </row>
-    <row r="49" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B49" s="66" t="str">
+      <c r="D45" s="86" t="s">
+        <v>59</v>
+      </c>
+      <c r="F45" s="48"/>
+    </row>
+    <row r="46" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B46" s="66" t="str">
         <f t="shared" si="17"/>
         <v>10EC</v>
       </c>
-      <c r="C49" s="33">
+      <c r="C46" s="33">
         <v>20</v>
       </c>
-      <c r="D49" s="67" t="s">
-        <v>66</v>
-      </c>
-      <c r="E49" s="68"/>
-      <c r="F49" s="69"/>
-    </row>
-    <row r="50" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B50" s="90" t="str">
+      <c r="D46" s="67" t="s">
+        <v>62</v>
+      </c>
+      <c r="E46" s="68"/>
+      <c r="F46" s="69"/>
+    </row>
+    <row r="47" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B47" s="90" t="str">
         <f t="shared" si="17"/>
         <v>1100</v>
       </c>
-      <c r="C50" s="70">
-        <f>HEX2DEC(B51)-HEX2DEC(B50)</f>
-        <v>6960</v>
-      </c>
-      <c r="D50" s="71" t="s">
+      <c r="C47" s="70">
+        <f>HEX2DEC(B48)-HEX2DEC(B47)</f>
+        <v>7056</v>
+      </c>
+      <c r="D47" s="71" t="s">
         <v>10</v>
       </c>
-      <c r="E50" s="71"/>
-      <c r="F50" s="72"/>
+      <c r="E47" s="71"/>
+      <c r="F47" s="72"/>
+    </row>
+    <row r="48" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B48" s="73" t="str">
+        <f t="shared" ref="B48:B52" si="18">DEC2HEX(HEX2DEC(B49)-C48)</f>
+        <v>2C90</v>
+      </c>
+      <c r="C48" s="31">
+        <v>768</v>
+      </c>
+      <c r="D48" s="80" t="s">
+        <v>54</v>
+      </c>
+      <c r="E48" s="80"/>
+      <c r="F48" s="81"/>
+    </row>
+    <row r="49" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B49" s="47" t="str">
+        <f t="shared" si="18"/>
+        <v>2F90</v>
+      </c>
+      <c r="C49" s="30">
+        <v>96</v>
+      </c>
+      <c r="D49" t="s">
+        <v>56</v>
+      </c>
+      <c r="F49" s="48"/>
+    </row>
+    <row r="50" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B50" s="47" t="str">
+        <f t="shared" si="18"/>
+        <v>2FF0</v>
+      </c>
+      <c r="C50" s="30">
+        <v>96</v>
+      </c>
+      <c r="D50" t="s">
+        <v>71</v>
+      </c>
+      <c r="F50" s="48"/>
     </row>
     <row r="51" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B51" s="73" t="str">
-        <f t="shared" ref="B51:B55" si="18">DEC2HEX(HEX2DEC(B52)-C51)</f>
-        <v>2C30</v>
-      </c>
-      <c r="C51" s="31">
-        <v>864</v>
-      </c>
-      <c r="D51" s="80" t="s">
-        <v>58</v>
-      </c>
-      <c r="E51" s="80"/>
-      <c r="F51" s="81"/>
+      <c r="B51" s="66" t="str">
+        <f t="shared" si="18"/>
+        <v>3050</v>
+      </c>
+      <c r="C51" s="33">
+        <f>$D$11</f>
+        <v>224</v>
+      </c>
+      <c r="D51" s="68" t="s">
+        <v>28</v>
+      </c>
+      <c r="E51" s="68"/>
+      <c r="F51" s="69"/>
     </row>
     <row r="52" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B52" s="47" t="str">
         <f t="shared" si="18"/>
-        <v>2F90</v>
+        <v>3130</v>
       </c>
       <c r="C52" s="30">
-        <v>96</v>
+        <v>16</v>
       </c>
       <c r="D52" t="s">
-        <v>60</v>
+        <v>29</v>
       </c>
       <c r="F52" s="48"/>
     </row>
     <row r="53" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B53" s="47" t="str">
-        <f t="shared" si="18"/>
-        <v>2FF0</v>
+        <f>DEC2HEX(HEX2DEC(B54)-C53)</f>
+        <v>3140</v>
       </c>
       <c r="C53" s="30">
-        <v>96</v>
-      </c>
-      <c r="D53" t="s">
-        <v>75</v>
+        <v>1728</v>
+      </c>
+      <c r="D53" s="17" t="s">
+        <v>63</v>
       </c>
       <c r="F53" s="48"/>
     </row>
     <row r="54" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B54" s="66" t="str">
-        <f t="shared" si="18"/>
-        <v>3050</v>
-      </c>
-      <c r="C54" s="33">
-        <f>$D$12</f>
-        <v>224</v>
-      </c>
-      <c r="D54" s="68" t="s">
-        <v>28</v>
-      </c>
-      <c r="E54" s="68"/>
-      <c r="F54" s="69"/>
-    </row>
-    <row r="55" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B55" s="47" t="str">
-        <f t="shared" si="18"/>
-        <v>3130</v>
-      </c>
-      <c r="C55" s="30">
-        <v>16</v>
-      </c>
-      <c r="D55" t="s">
-        <v>29</v>
-      </c>
-      <c r="F55" s="48"/>
-    </row>
-    <row r="56" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B56" s="47" t="str">
-        <f>DEC2HEX(HEX2DEC(B57)-C56)</f>
-        <v>3140</v>
-      </c>
-      <c r="C56" s="30">
-        <v>1728</v>
-      </c>
-      <c r="D56" s="17" t="s">
-        <v>67</v>
-      </c>
-      <c r="F56" s="48"/>
-    </row>
-    <row r="57" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B57" s="47" t="str">
-        <f t="shared" ref="B57" si="19">DEC2HEX(HEX2DEC(B58)-C57)</f>
+      <c r="B54" s="47" t="str">
+        <f t="shared" ref="B54" si="19">DEC2HEX(HEX2DEC(B55)-C54)</f>
         <v>3800</v>
       </c>
-      <c r="C57" s="30">
+      <c r="C54" s="30">
         <f>2048</f>
         <v>2048</v>
       </c>
-      <c r="D57" s="17" t="s">
+      <c r="D54" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="F57" s="48"/>
-    </row>
-    <row r="58" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B58" s="91">
+      <c r="F54" s="48"/>
+    </row>
+    <row r="55" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B55" s="91">
         <v>4000</v>
       </c>
-      <c r="C58" s="92"/>
-      <c r="D58" s="93" t="s">
+      <c r="C55" s="92"/>
+      <c r="D55" s="93" t="s">
         <v>19</v>
       </c>
-      <c r="E58" s="94"/>
-      <c r="F58" s="95"/>
+      <c r="E55" s="94"/>
+      <c r="F55" s="95"/>
+    </row>
+    <row r="56" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B56" s="17"/>
+      <c r="C56" s="17"/>
+      <c r="D56" s="17"/>
+    </row>
+    <row r="57" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B57" s="100" t="s">
+        <v>7</v>
+      </c>
+      <c r="C57" s="61" t="s">
+        <v>20</v>
+      </c>
+      <c r="D57" s="101" t="s">
+        <v>8</v>
+      </c>
+      <c r="E57" s="53"/>
+      <c r="F57" s="54"/>
+    </row>
+    <row r="58" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B58" s="105">
+        <v>4000</v>
+      </c>
+      <c r="C58" s="96">
+        <f>HEX2DEC(B59)-HEX2DEC(B58)</f>
+        <v>2</v>
+      </c>
+      <c r="D58" s="97" t="s">
+        <v>74</v>
+      </c>
+      <c r="F58" s="48"/>
     </row>
     <row r="59" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B59" s="17"/>
-      <c r="C59" s="17"/>
-      <c r="D59" s="17"/>
-    </row>
-    <row r="60" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B60" s="17"/>
-      <c r="C60" s="17"/>
-      <c r="D60" s="17"/>
-    </row>
-    <row r="61" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B61" s="100" t="s">
-        <v>7</v>
-      </c>
-      <c r="C61" s="61" t="s">
-        <v>20</v>
-      </c>
-      <c r="D61" s="101" t="s">
-        <v>8</v>
-      </c>
-      <c r="E61" s="53"/>
-      <c r="F61" s="54"/>
+      <c r="B59" s="105">
+        <v>4002</v>
+      </c>
+      <c r="C59" s="96">
+        <f>HEX2DEC(B60)-HEX2DEC(B59)</f>
+        <v>28</v>
+      </c>
+      <c r="D59" s="97" t="s">
+        <v>75</v>
+      </c>
+      <c r="F59" s="48"/>
+    </row>
+    <row r="60" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B60" s="105" t="s">
+        <v>76</v>
+      </c>
+      <c r="C60" s="96">
+        <f t="shared" ref="C60:C70" si="20">HEX2DEC(B61)-HEX2DEC(B60)</f>
+        <v>5</v>
+      </c>
+      <c r="D60" s="97" t="s">
+        <v>77</v>
+      </c>
+      <c r="F60" s="48"/>
+    </row>
+    <row r="61" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B61" s="105">
+        <v>4023</v>
+      </c>
+      <c r="C61" s="96">
+        <f t="shared" si="20"/>
+        <v>192</v>
+      </c>
+      <c r="D61" s="97" t="s">
+        <v>78</v>
+      </c>
+      <c r="F61" s="48"/>
     </row>
     <row r="62" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B62" s="105">
-        <v>4000</v>
+      <c r="B62" s="106" t="s">
+        <v>92</v>
       </c>
       <c r="C62" s="96">
-        <f>HEX2DEC(B63)-HEX2DEC(B62)</f>
-        <v>2</v>
+        <f t="shared" si="20"/>
+        <v>48</v>
       </c>
       <c r="D62" s="97" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F62" s="48"/>
     </row>
     <row r="63" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B63" s="105">
-        <v>4002</v>
+        <v>4113</v>
       </c>
       <c r="C63" s="96">
-        <f>HEX2DEC(B64)-HEX2DEC(B63)</f>
-        <v>28</v>
+        <f t="shared" si="20"/>
+        <v>3712</v>
       </c>
       <c r="D63" s="97" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F63" s="48"/>
     </row>
     <row r="64" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B64" s="105" t="s">
-        <v>80</v>
-      </c>
-      <c r="C64" s="96">
-        <f t="shared" ref="C64:C74" si="20">HEX2DEC(B65)-HEX2DEC(B64)</f>
-        <v>5</v>
+        <v>93</v>
+      </c>
+      <c r="C64" s="120">
+        <f t="shared" si="20"/>
+        <v>1673</v>
       </c>
       <c r="D64" s="97" t="s">
         <v>81</v>
@@ -2880,12 +2872,12 @@
       <c r="F64" s="48"/>
     </row>
     <row r="65" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B65" s="105">
-        <v>4023</v>
+      <c r="B65" s="119" t="s">
+        <v>96</v>
       </c>
       <c r="C65" s="96">
         <f t="shared" si="20"/>
-        <v>192</v>
+        <v>76</v>
       </c>
       <c r="D65" s="97" t="s">
         <v>82</v>
@@ -2893,139 +2885,99 @@
       <c r="F65" s="48"/>
     </row>
     <row r="66" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B66" s="106" t="s">
-        <v>96</v>
-      </c>
-      <c r="C66" s="96">
+      <c r="B66" s="121">
+        <v>5668</v>
+      </c>
+      <c r="C66" s="120">
         <f t="shared" si="20"/>
-        <v>48</v>
-      </c>
-      <c r="D66" s="97" t="s">
+        <v>2637</v>
+      </c>
+      <c r="D66" s="102" t="s">
+        <v>89</v>
+      </c>
+      <c r="F66" s="48"/>
+    </row>
+    <row r="67" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B67" s="119" t="s">
+        <v>97</v>
+      </c>
+      <c r="C67" s="120">
+        <f t="shared" si="20"/>
+        <v>3205</v>
+      </c>
+      <c r="D67" s="97" t="s">
         <v>83</v>
       </c>
-      <c r="F66" s="48"/>
-    </row>
-    <row r="67" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B67" s="105">
-        <v>4113</v>
-      </c>
-      <c r="C67" s="96">
+      <c r="F67" s="48"/>
+    </row>
+    <row r="68" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B68" s="122" t="s">
+        <v>98</v>
+      </c>
+      <c r="C68" s="103">
         <f t="shared" si="20"/>
-        <v>3712</v>
-      </c>
-      <c r="D67" s="97" t="s">
-        <v>84</v>
-      </c>
-      <c r="F67" s="48"/>
-    </row>
-    <row r="68" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B68" s="105" t="s">
-        <v>97</v>
-      </c>
-      <c r="C68" s="96">
-        <f t="shared" si="20"/>
-        <v>1741</v>
-      </c>
-      <c r="D68" s="97" t="s">
-        <v>85</v>
-      </c>
-      <c r="F68" s="48"/>
+        <v>300</v>
+      </c>
+      <c r="D68" s="104" t="s">
+        <v>90</v>
+      </c>
+      <c r="E68" s="88"/>
+      <c r="F68" s="79"/>
     </row>
     <row r="69" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B69" s="105">
-        <v>5660</v>
+      <c r="B69" s="108" t="s">
+        <v>91</v>
       </c>
       <c r="C69" s="96">
         <f t="shared" si="20"/>
-        <v>76</v>
+        <v>3226</v>
       </c>
       <c r="D69" s="97" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="F69" s="48"/>
     </row>
     <row r="70" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B70" s="107" t="s">
-        <v>98</v>
+      <c r="B70" s="105" t="s">
+        <v>84</v>
       </c>
       <c r="C70" s="96">
         <f t="shared" si="20"/>
-        <v>2637</v>
-      </c>
-      <c r="D70" s="102" t="s">
-        <v>93</v>
+        <v>256</v>
+      </c>
+      <c r="D70" s="97" t="s">
+        <v>85</v>
       </c>
       <c r="F70" s="48"/>
     </row>
-    <row r="71" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B71" s="105" t="s">
-        <v>99</v>
-      </c>
-      <c r="C71" s="96">
-        <f t="shared" si="20"/>
-        <v>3228</v>
-      </c>
-      <c r="D71" s="97" t="s">
+    <row r="71" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B71" s="107" t="s">
+        <v>86</v>
+      </c>
+      <c r="C71" s="98">
+        <v>1024</v>
+      </c>
+      <c r="D71" s="99" t="s">
         <v>87</v>
       </c>
-      <c r="F71" s="48"/>
+      <c r="E71" s="51"/>
+      <c r="F71" s="52"/>
     </row>
     <row r="72" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B72" s="108" t="s">
-        <v>100</v>
-      </c>
-      <c r="C72" s="103">
-        <f t="shared" si="20"/>
-        <v>209</v>
-      </c>
-      <c r="D72" s="104" t="s">
-        <v>94</v>
-      </c>
-      <c r="E72" s="88"/>
-      <c r="F72" s="79"/>
+      <c r="B72" s="46"/>
+      <c r="C72" s="96"/>
     </row>
     <row r="73" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B73" s="110" t="s">
-        <v>95</v>
-      </c>
-      <c r="C73" s="96">
-        <f t="shared" si="20"/>
-        <v>3226</v>
-      </c>
-      <c r="D73" s="97" t="s">
-        <v>92</v>
-      </c>
-      <c r="F73" s="48"/>
+      <c r="B73" s="46"/>
     </row>
     <row r="74" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B74" s="105" t="s">
-        <v>88</v>
-      </c>
-      <c r="C74" s="96">
-        <f t="shared" si="20"/>
-        <v>256</v>
-      </c>
-      <c r="D74" s="97" t="s">
-        <v>89</v>
-      </c>
-      <c r="F74" s="48"/>
-    </row>
-    <row r="75" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B75" s="109" t="s">
-        <v>90</v>
-      </c>
-      <c r="C75" s="98">
-        <v>1024</v>
-      </c>
-      <c r="D75" s="99" t="s">
-        <v>91</v>
-      </c>
-      <c r="E75" s="51"/>
-      <c r="F75" s="52"/>
+      <c r="B74" s="46"/>
+    </row>
+    <row r="75" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B75" s="46"/>
     </row>
     <row r="76" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B76" s="46"/>
-      <c r="C76" s="96"/>
     </row>
     <row r="77" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B77" s="46"/>
@@ -3088,19 +3040,7 @@
       <c r="B96" s="46"/>
     </row>
     <row r="97" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B97" s="46"/>
-    </row>
-    <row r="98" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B98" s="46"/>
-    </row>
-    <row r="99" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B99" s="46"/>
-    </row>
-    <row r="100" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B100" s="46"/>
-    </row>
-    <row r="101" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B101" s="45"/>
+      <c r="B97" s="45"/>
     </row>
   </sheetData>
   <mergeCells count="12">

</xml_diff>

<commit_message>
Updated documentation with build smoke tests, which I used to catch two regression on the Model B+.  Also brought forward the battery flat sound effect so that it plays at the end of the screen transition.
</commit_message>
<xml_diff>
--- a/docs/Memory.xlsx
+++ b/docs/Memory.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\Beeb\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CACFC71B-9793-43CE-9F6F-AED72F2FF867}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{954BA03F-DB52-4008-8571-C8DEE52D16F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="19380" windowHeight="20970" xr2:uid="{C0DF3A0D-E6A9-4F13-8EDD-5DE46AD6E0DB}"/>
+    <workbookView xWindow="14540" yWindow="650" windowWidth="21080" windowHeight="19990" xr2:uid="{C0DF3A0D-E6A9-4F13-8EDD-5DE46AD6E0DB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -339,7 +339,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -375,20 +375,6 @@
       <name val="Aptos"/>
       <family val="2"/>
     </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Aptos"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos"/>
-      <family val="2"/>
-    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -805,7 +791,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="123">
+  <cellXfs count="121">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1093,16 +1079,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2862,7 +2842,7 @@
       <c r="B64" s="105" t="s">
         <v>93</v>
       </c>
-      <c r="C64" s="120">
+      <c r="C64" s="96">
         <f t="shared" si="20"/>
         <v>1673</v>
       </c>
@@ -2872,7 +2852,7 @@
       <c r="F64" s="48"/>
     </row>
     <row r="65" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B65" s="119" t="s">
+      <c r="B65" s="105" t="s">
         <v>96</v>
       </c>
       <c r="C65" s="96">
@@ -2885,10 +2865,10 @@
       <c r="F65" s="48"/>
     </row>
     <row r="66" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B66" s="121">
+      <c r="B66" s="119">
         <v>5668</v>
       </c>
-      <c r="C66" s="120">
+      <c r="C66" s="96">
         <f t="shared" si="20"/>
         <v>2637</v>
       </c>
@@ -2898,10 +2878,10 @@
       <c r="F66" s="48"/>
     </row>
     <row r="67" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B67" s="119" t="s">
+      <c r="B67" s="105" t="s">
         <v>97</v>
       </c>
-      <c r="C67" s="120">
+      <c r="C67" s="96">
         <f t="shared" si="20"/>
         <v>3205</v>
       </c>
@@ -2911,7 +2891,7 @@
       <c r="F67" s="48"/>
     </row>
     <row r="68" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B68" s="122" t="s">
+      <c r="B68" s="120" t="s">
         <v>98</v>
       </c>
       <c r="C68" s="103">

</xml_diff>

<commit_message>
Renames and documentation updates (no binary changes)
</commit_message>
<xml_diff>
--- a/docs/Memory.xlsx
+++ b/docs/Memory.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\Beeb\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\Beeb\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{954BA03F-DB52-4008-8571-C8DEE52D16F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB38BD7B-C08D-4A76-A07C-0F4BA4769C8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14540" yWindow="650" windowWidth="21080" windowHeight="19990" xr2:uid="{C0DF3A0D-E6A9-4F13-8EDD-5DE46AD6E0DB}"/>
+    <workbookView xWindow="12390" yWindow="0" windowWidth="12660" windowHeight="16010" xr2:uid="{C0DF3A0D-E6A9-4F13-8EDD-5DE46AD6E0DB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="100">
   <si>
     <t>Quantity</t>
   </si>
@@ -200,9 +200,6 @@
     <t>Sound effects</t>
   </si>
   <si>
-    <t>9 K9 sprites</t>
-  </si>
-  <si>
     <t>elevator sprite</t>
   </si>
   <si>
@@ -333,6 +330,12 @@
   </si>
   <si>
     <t>6D3A</t>
+  </si>
+  <si>
+    <t>16K</t>
+  </si>
+  <si>
+    <t>8 K9 sprites</t>
   </si>
 </sst>
 </file>
@@ -1049,6 +1052,12 @@
     <xf numFmtId="11" fontId="3" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1078,12 +1087,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1430,35 +1433,35 @@
   <sheetData>
     <row r="1" spans="2:18" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="2" spans="2:18" x14ac:dyDescent="0.35">
-      <c r="B2" s="113" t="s">
+      <c r="B2" s="115" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="115" t="s">
-        <v>0</v>
-      </c>
-      <c r="D2" s="110" t="s">
+      <c r="C2" s="117" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" s="112" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="109" t="s">
+      <c r="E2" s="111" t="s">
         <v>22</v>
       </c>
-      <c r="F2" s="112"/>
-      <c r="G2" s="109" t="s">
+      <c r="F2" s="114"/>
+      <c r="G2" s="111" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="110"/>
-      <c r="I2" s="111" t="s">
+      <c r="H2" s="112"/>
+      <c r="I2" s="113" t="s">
         <v>12</v>
       </c>
-      <c r="J2" s="112"/>
-      <c r="K2" s="109" t="s">
+      <c r="J2" s="114"/>
+      <c r="K2" s="111" t="s">
         <v>14</v>
       </c>
-      <c r="L2" s="110"/>
-      <c r="M2" s="111" t="s">
+      <c r="L2" s="112"/>
+      <c r="M2" s="113" t="s">
         <v>15</v>
       </c>
-      <c r="N2" s="112"/>
+      <c r="N2" s="114"/>
       <c r="O2" s="43" t="s">
         <v>6</v>
       </c>
@@ -1469,35 +1472,35 @@
       <c r="R2" s="15"/>
     </row>
     <row r="3" spans="2:18" x14ac:dyDescent="0.35">
-      <c r="B3" s="114"/>
-      <c r="C3" s="116"/>
-      <c r="D3" s="117"/>
-      <c r="E3" s="116" t="s">
+      <c r="B3" s="116"/>
+      <c r="C3" s="118"/>
+      <c r="D3" s="119"/>
+      <c r="E3" s="118" t="s">
         <v>23</v>
       </c>
-      <c r="F3" s="118"/>
-      <c r="G3" s="116" t="s">
+      <c r="F3" s="120"/>
+      <c r="G3" s="118" t="s">
         <v>23</v>
       </c>
-      <c r="H3" s="117"/>
+      <c r="H3" s="119"/>
       <c r="I3" s="41"/>
       <c r="J3" s="40"/>
-      <c r="K3" s="116" t="s">
+      <c r="K3" s="118" t="s">
         <v>23</v>
       </c>
-      <c r="L3" s="117"/>
-      <c r="M3" s="118" t="s">
+      <c r="L3" s="119"/>
+      <c r="M3" s="120" t="s">
         <v>23</v>
       </c>
-      <c r="N3" s="118"/>
+      <c r="N3" s="120"/>
       <c r="O3" s="42"/>
       <c r="P3" s="24"/>
       <c r="R3" s="15"/>
     </row>
     <row r="4" spans="2:18" x14ac:dyDescent="0.35">
-      <c r="B4" s="114"/>
-      <c r="C4" s="116"/>
-      <c r="D4" s="117"/>
+      <c r="B4" s="116"/>
+      <c r="C4" s="118"/>
+      <c r="D4" s="119"/>
       <c r="E4" s="21" t="s">
         <v>0</v>
       </c>
@@ -1752,7 +1755,7 @@
     </row>
     <row r="9" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B9" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C9" s="19">
         <v>4</v>
@@ -1806,7 +1809,7 @@
     </row>
     <row r="10" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B10" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C10" s="19">
         <v>4</v>
@@ -1966,7 +1969,7 @@
     </row>
     <row r="13" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B13" s="38" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C13" s="34">
         <v>1</v>
@@ -2159,7 +2162,7 @@
         <v>144</v>
       </c>
       <c r="D19" s="56" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E19" s="56"/>
       <c r="F19" s="58"/>
@@ -2186,12 +2189,12 @@
         <v>112</v>
       </c>
       <c r="D20" s="85" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E20" s="85"/>
       <c r="F20" s="83"/>
       <c r="H20" s="47" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="I20" s="17"/>
       <c r="K20" t="s">
@@ -2219,7 +2222,7 @@
       <c r="E21" s="80"/>
       <c r="F21" s="81"/>
       <c r="H21" s="47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I21" s="17"/>
       <c r="K21" t="s">
@@ -2302,12 +2305,12 @@
       </c>
       <c r="F24" s="48"/>
       <c r="H24" s="49" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="I24" s="50"/>
       <c r="J24" s="51"/>
       <c r="K24" s="50" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="L24" s="16">
         <v>20</v>
@@ -2344,7 +2347,7 @@
         <v>32</v>
       </c>
       <c r="D26" s="68" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E26" s="68"/>
       <c r="F26" s="69"/>
@@ -2359,7 +2362,7 @@
         <v>432</v>
       </c>
       <c r="D27" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F27" s="48"/>
       <c r="H27" s="17"/>
@@ -2387,7 +2390,7 @@
         <v>192</v>
       </c>
       <c r="D29" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F29" s="48"/>
     </row>
@@ -2400,7 +2403,7 @@
         <v>16</v>
       </c>
       <c r="D30" s="67" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E30" s="68"/>
       <c r="F30" s="69"/>
@@ -2428,7 +2431,7 @@
         <v>64</v>
       </c>
       <c r="D32" s="86" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F32" s="48"/>
     </row>
@@ -2483,7 +2486,7 @@
         <v>32</v>
       </c>
       <c r="D36" s="86" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F36" s="48"/>
     </row>
@@ -2496,7 +2499,7 @@
         <v>64</v>
       </c>
       <c r="D37" s="86" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F37" s="48"/>
     </row>
@@ -2603,7 +2606,7 @@
         <v>12</v>
       </c>
       <c r="D45" s="86" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F45" s="48"/>
     </row>
@@ -2616,7 +2619,7 @@
         <v>20</v>
       </c>
       <c r="D46" s="67" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E46" s="68"/>
       <c r="F46" s="69"/>
@@ -2645,7 +2648,7 @@
         <v>768</v>
       </c>
       <c r="D48" s="80" t="s">
-        <v>54</v>
+        <v>99</v>
       </c>
       <c r="E48" s="80"/>
       <c r="F48" s="81"/>
@@ -2659,7 +2662,7 @@
         <v>96</v>
       </c>
       <c r="D49" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F49" s="48"/>
     </row>
@@ -2672,7 +2675,7 @@
         <v>96</v>
       </c>
       <c r="D50" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F50" s="48"/>
     </row>
@@ -2713,7 +2716,7 @@
         <v>1728</v>
       </c>
       <c r="D53" s="17" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F53" s="48"/>
     </row>
@@ -2735,7 +2738,9 @@
       <c r="B55" s="91">
         <v>4000</v>
       </c>
-      <c r="C55" s="92"/>
+      <c r="C55" s="92" t="s">
+        <v>98</v>
+      </c>
       <c r="D55" s="93" t="s">
         <v>19</v>
       </c>
@@ -2769,7 +2774,7 @@
         <v>2</v>
       </c>
       <c r="D58" s="97" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F58" s="48"/>
     </row>
@@ -2782,20 +2787,20 @@
         <v>28</v>
       </c>
       <c r="D59" s="97" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F59" s="48"/>
     </row>
     <row r="60" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B60" s="105" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C60" s="96">
         <f t="shared" ref="C60:C70" si="20">HEX2DEC(B61)-HEX2DEC(B60)</f>
         <v>5</v>
       </c>
       <c r="D60" s="97" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F60" s="48"/>
     </row>
@@ -2808,20 +2813,20 @@
         <v>192</v>
       </c>
       <c r="D61" s="97" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F61" s="48"/>
     </row>
     <row r="62" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B62" s="106" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C62" s="96">
         <f t="shared" si="20"/>
         <v>48</v>
       </c>
       <c r="D62" s="97" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F62" s="48"/>
     </row>
@@ -2834,38 +2839,38 @@
         <v>3712</v>
       </c>
       <c r="D63" s="97" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F63" s="48"/>
     </row>
     <row r="64" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B64" s="105" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C64" s="96">
         <f t="shared" si="20"/>
         <v>1673</v>
       </c>
       <c r="D64" s="97" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F64" s="48"/>
     </row>
     <row r="65" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B65" s="105" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C65" s="96">
         <f t="shared" si="20"/>
         <v>76</v>
       </c>
       <c r="D65" s="97" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F65" s="48"/>
     </row>
     <row r="66" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B66" s="119">
+      <c r="B66" s="109">
         <v>5668</v>
       </c>
       <c r="C66" s="96">
@@ -2873,72 +2878,72 @@
         <v>2637</v>
       </c>
       <c r="D66" s="102" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F66" s="48"/>
     </row>
     <row r="67" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B67" s="105" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C67" s="96">
         <f t="shared" si="20"/>
         <v>3205</v>
       </c>
       <c r="D67" s="97" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F67" s="48"/>
     </row>
     <row r="68" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B68" s="120" t="s">
-        <v>98</v>
+      <c r="B68" s="110" t="s">
+        <v>97</v>
       </c>
       <c r="C68" s="103">
         <f t="shared" si="20"/>
         <v>300</v>
       </c>
       <c r="D68" s="104" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E68" s="88"/>
       <c r="F68" s="79"/>
     </row>
     <row r="69" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B69" s="108" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C69" s="96">
         <f t="shared" si="20"/>
         <v>3226</v>
       </c>
       <c r="D69" s="97" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F69" s="48"/>
     </row>
     <row r="70" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B70" s="105" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C70" s="96">
         <f t="shared" si="20"/>
         <v>256</v>
       </c>
       <c r="D70" s="97" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F70" s="48"/>
     </row>
     <row r="71" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B71" s="107" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C71" s="98">
         <v>1024</v>
       </c>
       <c r="D71" s="99" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E71" s="51"/>
       <c r="F71" s="52"/>

</xml_diff>

<commit_message>
Updated God mode to help players experience more of the game.  God mode is revised so that: - K9's laser operates at double the standard strength, while enemy weapons function at half their usual power. - An arbitrary level can be loaded by pressing the associated number key. E.g. '1' to '6'. - The level can be scrolled using the arrow keys, independent of K9’s position. - The mode is activated by pressing the ‘G’, ‘O’, and ‘D’ keys together. A sound effect will play and the top-right screen pixel will be painted black to help distinguish it from normal play. Bug fixes:  - Fixed bug where movement sound effect tone could change near the beginning of a level  - Fixed a bug where the tile grid flags were not always set correctly when an enemy turns, and moves.  - A number of code size optimizations were made to facilitate the changes.  - Corrected Weeping Angel move right sprites  - Made all game bar backgrounds blue
</commit_message>
<xml_diff>
--- a/docs/Memory.xlsx
+++ b/docs/Memory.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\Beeb\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\Beeb\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB38BD7B-C08D-4A76-A07C-0F4BA4769C8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC2A5183-8E6E-404F-9500-3B038BBD59F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12390" yWindow="0" windowWidth="12660" windowHeight="16010" xr2:uid="{C0DF3A0D-E6A9-4F13-8EDD-5DE46AD6E0DB}"/>
+    <workbookView xWindow="19110" yWindow="0" windowWidth="19380" windowHeight="20970" xr2:uid="{C0DF3A0D-E6A9-4F13-8EDD-5DE46AD6E0DB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="99">
   <si>
     <t>Quantity</t>
   </si>
@@ -323,19 +323,16 @@
     <t>2 K9 sprites</t>
   </si>
   <si>
-    <t>561C</t>
-  </si>
-  <si>
-    <t>60B5</t>
-  </si>
-  <si>
-    <t>6D3A</t>
-  </si>
-  <si>
     <t>16K</t>
   </si>
   <si>
     <t>8 K9 sprites</t>
+  </si>
+  <si>
+    <t>60E2</t>
+  </si>
+  <si>
+    <t>6D67</t>
   </si>
 </sst>
 </file>
@@ -1055,7 +1052,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="11" fontId="3" fillId="2" borderId="7" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2648,7 +2645,7 @@
         <v>768</v>
       </c>
       <c r="D48" s="80" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="E48" s="80"/>
       <c r="F48" s="81"/>
@@ -2739,7 +2736,7 @@
         <v>4000</v>
       </c>
       <c r="C55" s="92" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="D55" s="93" t="s">
         <v>19</v>
@@ -2849,7 +2846,7 @@
       </c>
       <c r="C64" s="96">
         <f t="shared" si="20"/>
-        <v>1673</v>
+        <v>1714</v>
       </c>
       <c r="D64" s="97" t="s">
         <v>80</v>
@@ -2857,8 +2854,8 @@
       <c r="F64" s="48"/>
     </row>
     <row r="65" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B65" s="105" t="s">
-        <v>95</v>
+      <c r="B65" s="105">
+        <v>5645</v>
       </c>
       <c r="C65" s="96">
         <f t="shared" si="20"/>
@@ -2871,11 +2868,11 @@
     </row>
     <row r="66" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B66" s="109">
-        <v>5668</v>
+        <v>5691</v>
       </c>
       <c r="C66" s="96">
         <f t="shared" si="20"/>
-        <v>2637</v>
+        <v>2641</v>
       </c>
       <c r="D66" s="102" t="s">
         <v>88</v>
@@ -2883,8 +2880,8 @@
       <c r="F66" s="48"/>
     </row>
     <row r="67" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B67" s="105" t="s">
-        <v>96</v>
+      <c r="B67" s="108" t="s">
+        <v>97</v>
       </c>
       <c r="C67" s="96">
         <f t="shared" si="20"/>
@@ -2897,11 +2894,11 @@
     </row>
     <row r="68" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B68" s="110" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C68" s="103">
         <f t="shared" si="20"/>
-        <v>300</v>
+        <v>255</v>
       </c>
       <c r="D68" s="104" t="s">
         <v>89</v>

</xml_diff>

<commit_message>
Added palette inversion effect. Also:  - Corrected typos in comments  - Updated documentation.  - Fixed usage of waitForVSync
</commit_message>
<xml_diff>
--- a/docs/Memory.xlsx
+++ b/docs/Memory.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\Beeb\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC2A5183-8E6E-404F-9500-3B038BBD59F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB2F8A52-861A-46C3-ADD1-370A73AF6027}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19110" yWindow="0" windowWidth="19380" windowHeight="20970" xr2:uid="{C0DF3A0D-E6A9-4F13-8EDD-5DE46AD6E0DB}"/>
+    <workbookView xWindow="9810" yWindow="870" windowWidth="26580" windowHeight="19990" xr2:uid="{C0DF3A0D-E6A9-4F13-8EDD-5DE46AD6E0DB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="101">
   <si>
     <t>Quantity</t>
   </si>
@@ -224,15 +224,9 @@
     <t>Draw object jump tables</t>
   </si>
   <si>
-    <t>29 level tiles</t>
-  </si>
-  <si>
     <t>Black palette</t>
   </si>
   <si>
-    <t>black palette</t>
-  </si>
-  <si>
     <t>zero-page game variables</t>
   </si>
   <si>
@@ -263,76 +257,88 @@
     <t>Level tile types</t>
   </si>
   <si>
+    <t>Level settings</t>
+  </si>
+  <si>
+    <t>Level object descriptors (48)</t>
+  </si>
+  <si>
+    <t>Level switch pairings</t>
+  </si>
+  <si>
+    <t>Level sprite data</t>
+  </si>
+  <si>
+    <t>Level initialization code</t>
+  </si>
+  <si>
+    <t>Mode 7 routines</t>
+  </si>
+  <si>
+    <t>Music data and code</t>
+  </si>
+  <si>
+    <t>7B00</t>
+  </si>
+  <si>
+    <t>DFS command page backup</t>
+  </si>
+  <si>
+    <t>7C00</t>
+  </si>
+  <si>
+    <t>Mode 7 screen</t>
+  </si>
+  <si>
+    <t>PCM load buffer</t>
+  </si>
+  <si>
+    <t>Titles, interstitial, or finale</t>
+  </si>
+  <si>
+    <t>Unused memory</t>
+  </si>
+  <si>
+    <t>6E66</t>
+  </si>
+  <si>
+    <t>9 game objects array</t>
+  </si>
+  <si>
+    <t>2 K9 sprites</t>
+  </si>
+  <si>
+    <t>16K</t>
+  </si>
+  <si>
+    <t>8 K9 sprites</t>
+  </si>
+  <si>
+    <t>level palette</t>
+  </si>
+  <si>
+    <t>402E</t>
+  </si>
+  <si>
+    <t>40F3</t>
+  </si>
+  <si>
+    <t>4FA3</t>
+  </si>
+  <si>
     <t>401E</t>
   </si>
   <si>
-    <t>Level settings</t>
-  </si>
-  <si>
-    <t>Level object descriptors (48)</t>
-  </si>
-  <si>
-    <t>Level switch pairings</t>
-  </si>
-  <si>
-    <t>Level sprite data</t>
-  </si>
-  <si>
-    <t>Level initialization code</t>
-  </si>
-  <si>
-    <t>Mode 7 routines</t>
-  </si>
-  <si>
-    <t>Music data and code</t>
-  </si>
-  <si>
-    <t>7B00</t>
-  </si>
-  <si>
-    <t>DFS command page backup</t>
-  </si>
-  <si>
-    <t>7C00</t>
-  </si>
-  <si>
-    <t>Mode 7 screen</t>
-  </si>
-  <si>
-    <t>PCM load buffer</t>
-  </si>
-  <si>
-    <t>Titles, interstitial, or finale</t>
-  </si>
-  <si>
-    <t>Unused memory</t>
-  </si>
-  <si>
-    <t>6E66</t>
-  </si>
-  <si>
-    <t>40E3</t>
-  </si>
-  <si>
-    <t>4F93</t>
-  </si>
-  <si>
-    <t>9 game objects array</t>
-  </si>
-  <si>
-    <t>2 K9 sprites</t>
-  </si>
-  <si>
-    <t>16K</t>
-  </si>
-  <si>
-    <t>8 K9 sprites</t>
-  </si>
-  <si>
-    <t>60E2</t>
-  </si>
-  <si>
-    <t>6D67</t>
+    <t>27 level tiles</t>
+  </si>
+  <si>
+    <t>56CC</t>
+  </si>
+  <si>
+    <t>60F4</t>
+  </si>
+  <si>
+    <t>6D79</t>
   </si>
 </sst>
 </file>
@@ -791,7 +797,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="121">
+  <cellXfs count="122">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1043,47 +1049,50 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="11" fontId="3" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="11" fontId="3" fillId="2" borderId="7" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="11" fontId="3" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="11" fontId="3" fillId="2" borderId="7" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1430,74 +1439,74 @@
   <sheetData>
     <row r="1" spans="2:18" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="2" spans="2:18" x14ac:dyDescent="0.35">
-      <c r="B2" s="115" t="s">
+      <c r="B2" s="112" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="117" t="s">
-        <v>0</v>
-      </c>
-      <c r="D2" s="112" t="s">
+      <c r="C2" s="114" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" s="109" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="111" t="s">
+      <c r="E2" s="108" t="s">
         <v>22</v>
       </c>
-      <c r="F2" s="114"/>
-      <c r="G2" s="111" t="s">
+      <c r="F2" s="111"/>
+      <c r="G2" s="108" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="112"/>
-      <c r="I2" s="113" t="s">
+      <c r="H2" s="109"/>
+      <c r="I2" s="110" t="s">
         <v>12</v>
       </c>
-      <c r="J2" s="114"/>
-      <c r="K2" s="111" t="s">
+      <c r="J2" s="111"/>
+      <c r="K2" s="108" t="s">
         <v>14</v>
       </c>
-      <c r="L2" s="112"/>
-      <c r="M2" s="113" t="s">
+      <c r="L2" s="109"/>
+      <c r="M2" s="110" t="s">
         <v>15</v>
       </c>
-      <c r="N2" s="114"/>
+      <c r="N2" s="111"/>
       <c r="O2" s="43" t="s">
         <v>6</v>
       </c>
       <c r="P2" s="14" t="str">
-        <f>DEC2HEX(HEX2DEC(3130)-P14)</f>
-        <v>2C90</v>
+        <f>DEC2HEX(HEX2DEC(3140)-P14)</f>
+        <v>2CA0</v>
       </c>
       <c r="R2" s="15"/>
     </row>
     <row r="3" spans="2:18" x14ac:dyDescent="0.35">
-      <c r="B3" s="116"/>
-      <c r="C3" s="118"/>
-      <c r="D3" s="119"/>
-      <c r="E3" s="118" t="s">
+      <c r="B3" s="113"/>
+      <c r="C3" s="115"/>
+      <c r="D3" s="116"/>
+      <c r="E3" s="115" t="s">
         <v>23</v>
       </c>
-      <c r="F3" s="120"/>
-      <c r="G3" s="118" t="s">
+      <c r="F3" s="117"/>
+      <c r="G3" s="115" t="s">
         <v>23</v>
       </c>
-      <c r="H3" s="119"/>
+      <c r="H3" s="116"/>
       <c r="I3" s="41"/>
       <c r="J3" s="40"/>
-      <c r="K3" s="118" t="s">
+      <c r="K3" s="115" t="s">
         <v>23</v>
       </c>
-      <c r="L3" s="119"/>
-      <c r="M3" s="120" t="s">
+      <c r="L3" s="116"/>
+      <c r="M3" s="117" t="s">
         <v>23</v>
       </c>
-      <c r="N3" s="120"/>
+      <c r="N3" s="117"/>
       <c r="O3" s="42"/>
       <c r="P3" s="24"/>
       <c r="R3" s="15"/>
     </row>
     <row r="4" spans="2:18" x14ac:dyDescent="0.35">
-      <c r="B4" s="116"/>
-      <c r="C4" s="118"/>
-      <c r="D4" s="119"/>
+      <c r="B4" s="113"/>
+      <c r="C4" s="115"/>
+      <c r="D4" s="116"/>
       <c r="E4" s="21" t="s">
         <v>0</v>
       </c>
@@ -1806,7 +1815,7 @@
     </row>
     <row r="10" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B10" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C10" s="19">
         <v>4</v>
@@ -1966,7 +1975,7 @@
     </row>
     <row r="13" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B13" s="38" t="s">
-        <v>64</v>
+        <v>92</v>
       </c>
       <c r="C13" s="34">
         <v>1</v>
@@ -2159,7 +2168,7 @@
         <v>144</v>
       </c>
       <c r="D19" s="56" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E19" s="56"/>
       <c r="F19" s="58"/>
@@ -2186,12 +2195,12 @@
         <v>112</v>
       </c>
       <c r="D20" s="85" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="E20" s="85"/>
       <c r="F20" s="83"/>
       <c r="H20" s="47" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="I20" s="17"/>
       <c r="K20" t="s">
@@ -2219,7 +2228,7 @@
       <c r="E21" s="80"/>
       <c r="F21" s="81"/>
       <c r="H21" s="47" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="I21" s="17"/>
       <c r="K21" t="s">
@@ -2359,7 +2368,7 @@
         <v>432</v>
       </c>
       <c r="D27" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F27" s="48"/>
       <c r="H27" s="17"/>
@@ -2387,7 +2396,7 @@
         <v>192</v>
       </c>
       <c r="D29" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="F29" s="48"/>
     </row>
@@ -2400,7 +2409,7 @@
         <v>16</v>
       </c>
       <c r="D30" s="67" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E30" s="68"/>
       <c r="F30" s="69"/>
@@ -2428,7 +2437,7 @@
         <v>64</v>
       </c>
       <c r="D32" s="86" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F32" s="48"/>
     </row>
@@ -2496,7 +2505,7 @@
         <v>64</v>
       </c>
       <c r="D37" s="86" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F37" s="48"/>
     </row>
@@ -2628,7 +2637,7 @@
       </c>
       <c r="C47" s="70">
         <f>HEX2DEC(B48)-HEX2DEC(B47)</f>
-        <v>7056</v>
+        <v>7072</v>
       </c>
       <c r="D47" s="71" t="s">
         <v>10</v>
@@ -2638,14 +2647,14 @@
     </row>
     <row r="48" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B48" s="73" t="str">
-        <f t="shared" ref="B48:B52" si="18">DEC2HEX(HEX2DEC(B49)-C48)</f>
-        <v>2C90</v>
+        <f t="shared" ref="B48:B50" si="18">DEC2HEX(HEX2DEC(B49)-C48)</f>
+        <v>2CA0</v>
       </c>
       <c r="C48" s="31">
         <v>768</v>
       </c>
       <c r="D48" s="80" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="E48" s="80"/>
       <c r="F48" s="81"/>
@@ -2653,7 +2662,7 @@
     <row r="49" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B49" s="47" t="str">
         <f t="shared" si="18"/>
-        <v>2F90</v>
+        <v>2FA0</v>
       </c>
       <c r="C49" s="30">
         <v>96</v>
@@ -2666,281 +2675,281 @@
     <row r="50" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B50" s="47" t="str">
         <f t="shared" si="18"/>
-        <v>2FF0</v>
+        <v>3000</v>
       </c>
       <c r="C50" s="30">
         <v>96</v>
       </c>
       <c r="D50" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F50" s="48"/>
     </row>
     <row r="51" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B51" s="66" t="str">
-        <f t="shared" si="18"/>
-        <v>3050</v>
-      </c>
-      <c r="C51" s="33">
+      <c r="B51" s="47" t="str">
+        <f>DEC2HEX(HEX2DEC(B52)-C51)</f>
+        <v>3060</v>
+      </c>
+      <c r="C51" s="30">
         <f>$D$11</f>
         <v>224</v>
       </c>
-      <c r="D51" s="68" t="s">
+      <c r="D51" t="s">
         <v>28</v>
       </c>
-      <c r="E51" s="68"/>
-      <c r="F51" s="69"/>
+      <c r="F51" s="48"/>
     </row>
     <row r="52" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B52" s="47" t="str">
-        <f t="shared" si="18"/>
-        <v>3130</v>
-      </c>
-      <c r="C52" s="30">
-        <v>16</v>
-      </c>
-      <c r="D52" t="s">
-        <v>29</v>
-      </c>
-      <c r="F52" s="48"/>
+      <c r="B52" s="73" t="str">
+        <f>DEC2HEX(HEX2DEC(B53)-C52)</f>
+        <v>3140</v>
+      </c>
+      <c r="C52" s="31">
+        <v>1728</v>
+      </c>
+      <c r="D52" s="107" t="s">
+        <v>97</v>
+      </c>
+      <c r="E52" s="80"/>
+      <c r="F52" s="81"/>
     </row>
     <row r="53" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B53" s="47" t="str">
-        <f>DEC2HEX(HEX2DEC(B54)-C53)</f>
-        <v>3140</v>
+        <f t="shared" ref="B53" si="19">DEC2HEX(HEX2DEC(B54)-C53)</f>
+        <v>3800</v>
       </c>
       <c r="C53" s="30">
-        <v>1728</v>
-      </c>
-      <c r="D53" s="17" t="s">
-        <v>62</v>
-      </c>
-      <c r="F53" s="48"/>
-    </row>
-    <row r="54" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B54" s="47" t="str">
-        <f t="shared" ref="B54" si="19">DEC2HEX(HEX2DEC(B55)-C54)</f>
-        <v>3800</v>
-      </c>
-      <c r="C54" s="30">
         <f>2048</f>
         <v>2048</v>
       </c>
-      <c r="D54" s="17" t="s">
+      <c r="D53" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="F54" s="48"/>
+      <c r="F53" s="48"/>
+    </row>
+    <row r="54" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B54" s="91">
+        <v>4000</v>
+      </c>
+      <c r="C54" s="92" t="s">
+        <v>90</v>
+      </c>
+      <c r="D54" s="93" t="s">
+        <v>19</v>
+      </c>
+      <c r="E54" s="94"/>
+      <c r="F54" s="95"/>
     </row>
     <row r="55" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B55" s="91">
+      <c r="B55" s="17"/>
+      <c r="C55" s="17"/>
+      <c r="D55" s="17"/>
+    </row>
+    <row r="56" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B56" s="100" t="s">
+        <v>7</v>
+      </c>
+      <c r="C56" s="61" t="s">
+        <v>20</v>
+      </c>
+      <c r="D56" s="101" t="s">
+        <v>8</v>
+      </c>
+      <c r="E56" s="53"/>
+      <c r="F56" s="54"/>
+    </row>
+    <row r="57" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B57" s="105">
         <v>4000</v>
       </c>
-      <c r="C55" s="92" t="s">
-        <v>95</v>
-      </c>
-      <c r="D55" s="93" t="s">
-        <v>19</v>
-      </c>
-      <c r="E55" s="94"/>
-      <c r="F55" s="95"/>
-    </row>
-    <row r="56" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B56" s="17"/>
-      <c r="C56" s="17"/>
-      <c r="D56" s="17"/>
-    </row>
-    <row r="57" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B57" s="100" t="s">
-        <v>7</v>
-      </c>
-      <c r="C57" s="61" t="s">
-        <v>20</v>
-      </c>
-      <c r="D57" s="101" t="s">
-        <v>8</v>
-      </c>
-      <c r="E57" s="53"/>
-      <c r="F57" s="54"/>
+      <c r="C57" s="96">
+        <f>HEX2DEC(B58)-HEX2DEC(B57)</f>
+        <v>2</v>
+      </c>
+      <c r="D57" s="97" t="s">
+        <v>71</v>
+      </c>
+      <c r="F57" s="48"/>
     </row>
     <row r="58" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B58" s="105">
-        <v>4000</v>
+        <v>4002</v>
       </c>
       <c r="C58" s="96">
         <f>HEX2DEC(B59)-HEX2DEC(B58)</f>
-        <v>2</v>
+        <v>28</v>
       </c>
       <c r="D58" s="97" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F58" s="48"/>
     </row>
     <row r="59" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B59" s="105">
-        <v>4002</v>
+      <c r="B59" s="105" t="s">
+        <v>96</v>
       </c>
       <c r="C59" s="96">
-        <f>HEX2DEC(B60)-HEX2DEC(B59)</f>
-        <v>28</v>
+        <f t="shared" ref="C59:C61" si="20">HEX2DEC(B60)-HEX2DEC(B59)</f>
+        <v>16</v>
       </c>
       <c r="D59" s="97" t="s">
-        <v>74</v>
+        <v>29</v>
       </c>
       <c r="F59" s="48"/>
     </row>
     <row r="60" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B60" s="105" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="C60" s="96">
-        <f t="shared" ref="C60:C70" si="20">HEX2DEC(B61)-HEX2DEC(B60)</f>
+        <f t="shared" si="20"/>
         <v>5</v>
       </c>
       <c r="D60" s="97" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="F60" s="48"/>
     </row>
     <row r="61" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B61" s="105">
-        <v>4023</v>
+        <v>4033</v>
       </c>
       <c r="C61" s="96">
         <f t="shared" si="20"/>
         <v>192</v>
       </c>
       <c r="D61" s="97" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="F61" s="48"/>
     </row>
     <row r="62" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B62" s="106" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="C62" s="96">
-        <f t="shared" si="20"/>
+        <f t="shared" ref="C62:C70" si="21">HEX2DEC(B63)-HEX2DEC(B62)</f>
         <v>48</v>
       </c>
       <c r="D62" s="97" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="F62" s="48"/>
     </row>
     <row r="63" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B63" s="105">
-        <v>4113</v>
+        <v>4123</v>
       </c>
       <c r="C63" s="96">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>3712</v>
       </c>
       <c r="D63" s="97" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="F63" s="48"/>
     </row>
     <row r="64" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B64" s="105" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="C64" s="96">
-        <f t="shared" si="20"/>
-        <v>1714</v>
+        <f t="shared" si="21"/>
+        <v>1757</v>
       </c>
       <c r="D64" s="97" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="F64" s="48"/>
     </row>
     <row r="65" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B65" s="105">
-        <v>5645</v>
+        <v>5680</v>
       </c>
       <c r="C65" s="96">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>76</v>
       </c>
       <c r="D65" s="97" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="F65" s="48"/>
     </row>
     <row r="66" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B66" s="109">
-        <v>5691</v>
+      <c r="B66" s="118" t="s">
+        <v>98</v>
       </c>
       <c r="C66" s="96">
-        <f t="shared" si="20"/>
-        <v>2641</v>
+        <f t="shared" si="21"/>
+        <v>2600</v>
       </c>
       <c r="D66" s="102" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="F66" s="48"/>
     </row>
     <row r="67" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B67" s="108" t="s">
-        <v>97</v>
+      <c r="B67" s="119" t="s">
+        <v>99</v>
       </c>
       <c r="C67" s="96">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>3205</v>
       </c>
       <c r="D67" s="97" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="F67" s="48"/>
     </row>
     <row r="68" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B68" s="110" t="s">
-        <v>98</v>
+      <c r="B68" s="120" t="s">
+        <v>100</v>
       </c>
       <c r="C68" s="103">
-        <f t="shared" si="20"/>
-        <v>255</v>
+        <f t="shared" si="21"/>
+        <v>237</v>
       </c>
       <c r="D68" s="104" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="E68" s="88"/>
       <c r="F68" s="79"/>
     </row>
     <row r="69" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B69" s="108" t="s">
-        <v>90</v>
+      <c r="B69" s="119" t="s">
+        <v>87</v>
       </c>
       <c r="C69" s="96">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>3226</v>
       </c>
       <c r="D69" s="97" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="F69" s="48"/>
     </row>
     <row r="70" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B70" s="105" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C70" s="96">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>256</v>
       </c>
       <c r="D70" s="97" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="F70" s="48"/>
     </row>
     <row r="71" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B71" s="107" t="s">
-        <v>85</v>
+      <c r="B71" s="121" t="s">
+        <v>82</v>
       </c>
       <c r="C71" s="98">
         <v>1024</v>
       </c>
       <c r="D71" s="99" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="E71" s="51"/>
       <c r="F71" s="52"/>

</xml_diff>

<commit_message>
Changes:  - Improved teleport sound effect, adding new white noise sound effect.  - Removed transition callback which was not needed.  - Optimized drawObject, removing routine call in outer-loop  - Fixed clipping regression in drawObject  - Various code size optimizations  - Update documentation
</commit_message>
<xml_diff>
--- a/docs/Memory.xlsx
+++ b/docs/Memory.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\Beeb\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB2F8A52-861A-46C3-ADD1-370A73AF6027}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC0A388A-BE0A-48F5-A784-4014B9BF170B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9810" yWindow="870" windowWidth="26580" windowHeight="19990" xr2:uid="{C0DF3A0D-E6A9-4F13-8EDD-5DE46AD6E0DB}"/>
+    <workbookView xWindow="11820" yWindow="360" windowWidth="26580" windowHeight="19990" xr2:uid="{C0DF3A0D-E6A9-4F13-8EDD-5DE46AD6E0DB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -206,12 +206,6 @@
     <t>4 elevator sprites</t>
   </si>
   <si>
-    <t>drawObject jump tables</t>
-  </si>
-  <si>
-    <t>&amp;10EB</t>
-  </si>
-  <si>
     <t>Sprite health bar table</t>
   </si>
   <si>
@@ -332,13 +326,19 @@
     <t>27 level tiles</t>
   </si>
   <si>
-    <t>56CC</t>
-  </si>
-  <si>
-    <t>60F4</t>
-  </si>
-  <si>
-    <t>6D79</t>
+    <t>drawObject jump table</t>
+  </si>
+  <si>
+    <t>&amp;10EC</t>
+  </si>
+  <si>
+    <t>56AE</t>
+  </si>
+  <si>
+    <t>60D6</t>
+  </si>
+  <si>
+    <t>6D5B</t>
   </si>
 </sst>
 </file>
@@ -1052,6 +1052,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="11" fontId="3" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="11" fontId="3" fillId="2" borderId="7" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1081,18 +1093,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="11" fontId="3" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="11" fontId="3" fillId="2" borderId="7" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1439,35 +1439,35 @@
   <sheetData>
     <row r="1" spans="2:18" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="2" spans="2:18" x14ac:dyDescent="0.35">
-      <c r="B2" s="112" t="s">
+      <c r="B2" s="116" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="114" t="s">
-        <v>0</v>
-      </c>
-      <c r="D2" s="109" t="s">
+      <c r="C2" s="118" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" s="113" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="108" t="s">
+      <c r="E2" s="112" t="s">
         <v>22</v>
       </c>
-      <c r="F2" s="111"/>
-      <c r="G2" s="108" t="s">
+      <c r="F2" s="115"/>
+      <c r="G2" s="112" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="109"/>
-      <c r="I2" s="110" t="s">
+      <c r="H2" s="113"/>
+      <c r="I2" s="114" t="s">
         <v>12</v>
       </c>
-      <c r="J2" s="111"/>
-      <c r="K2" s="108" t="s">
+      <c r="J2" s="115"/>
+      <c r="K2" s="112" t="s">
         <v>14</v>
       </c>
-      <c r="L2" s="109"/>
-      <c r="M2" s="110" t="s">
+      <c r="L2" s="113"/>
+      <c r="M2" s="114" t="s">
         <v>15</v>
       </c>
-      <c r="N2" s="111"/>
+      <c r="N2" s="115"/>
       <c r="O2" s="43" t="s">
         <v>6</v>
       </c>
@@ -1478,35 +1478,35 @@
       <c r="R2" s="15"/>
     </row>
     <row r="3" spans="2:18" x14ac:dyDescent="0.35">
-      <c r="B3" s="113"/>
-      <c r="C3" s="115"/>
-      <c r="D3" s="116"/>
-      <c r="E3" s="115" t="s">
+      <c r="B3" s="117"/>
+      <c r="C3" s="119"/>
+      <c r="D3" s="120"/>
+      <c r="E3" s="119" t="s">
         <v>23</v>
       </c>
-      <c r="F3" s="117"/>
-      <c r="G3" s="115" t="s">
+      <c r="F3" s="121"/>
+      <c r="G3" s="119" t="s">
         <v>23</v>
       </c>
-      <c r="H3" s="116"/>
+      <c r="H3" s="120"/>
       <c r="I3" s="41"/>
       <c r="J3" s="40"/>
-      <c r="K3" s="115" t="s">
+      <c r="K3" s="119" t="s">
         <v>23</v>
       </c>
-      <c r="L3" s="116"/>
-      <c r="M3" s="117" t="s">
+      <c r="L3" s="120"/>
+      <c r="M3" s="121" t="s">
         <v>23</v>
       </c>
-      <c r="N3" s="117"/>
+      <c r="N3" s="121"/>
       <c r="O3" s="42"/>
       <c r="P3" s="24"/>
       <c r="R3" s="15"/>
     </row>
     <row r="4" spans="2:18" x14ac:dyDescent="0.35">
-      <c r="B4" s="113"/>
-      <c r="C4" s="115"/>
-      <c r="D4" s="116"/>
+      <c r="B4" s="117"/>
+      <c r="C4" s="119"/>
+      <c r="D4" s="120"/>
       <c r="E4" s="21" t="s">
         <v>0</v>
       </c>
@@ -1815,7 +1815,7 @@
     </row>
     <row r="10" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B10" s="1" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C10" s="19">
         <v>4</v>
@@ -1975,7 +1975,7 @@
     </row>
     <row r="13" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B13" s="38" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C13" s="34">
         <v>1</v>
@@ -2168,7 +2168,7 @@
         <v>144</v>
       </c>
       <c r="D19" s="56" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E19" s="56"/>
       <c r="F19" s="58"/>
@@ -2195,12 +2195,12 @@
         <v>112</v>
       </c>
       <c r="D20" s="85" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E20" s="85"/>
       <c r="F20" s="83"/>
       <c r="H20" s="47" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="I20" s="17"/>
       <c r="K20" t="s">
@@ -2228,7 +2228,7 @@
       <c r="E21" s="80"/>
       <c r="F21" s="81"/>
       <c r="H21" s="47" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I21" s="17"/>
       <c r="K21" t="s">
@@ -2263,7 +2263,7 @@
         <v>46</v>
       </c>
       <c r="L22" s="30">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="M22" t="s">
         <v>48</v>
@@ -2311,15 +2311,15 @@
       </c>
       <c r="F24" s="48"/>
       <c r="H24" s="49" t="s">
-        <v>56</v>
+        <v>96</v>
       </c>
       <c r="I24" s="50"/>
       <c r="J24" s="51"/>
       <c r="K24" s="50" t="s">
-        <v>57</v>
+        <v>97</v>
       </c>
       <c r="L24" s="16">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="M24" s="51" t="s">
         <v>49</v>
@@ -2353,7 +2353,7 @@
         <v>32</v>
       </c>
       <c r="D26" s="68" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E26" s="68"/>
       <c r="F26" s="69"/>
@@ -2368,7 +2368,7 @@
         <v>432</v>
       </c>
       <c r="D27" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="F27" s="48"/>
       <c r="H27" s="17"/>
@@ -2396,7 +2396,7 @@
         <v>192</v>
       </c>
       <c r="D29" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="F29" s="48"/>
     </row>
@@ -2409,7 +2409,7 @@
         <v>16</v>
       </c>
       <c r="D30" s="67" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E30" s="68"/>
       <c r="F30" s="69"/>
@@ -2437,7 +2437,7 @@
         <v>64</v>
       </c>
       <c r="D32" s="86" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="F32" s="48"/>
     </row>
@@ -2492,7 +2492,7 @@
         <v>32</v>
       </c>
       <c r="D36" s="86" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F36" s="48"/>
     </row>
@@ -2505,7 +2505,7 @@
         <v>64</v>
       </c>
       <c r="D37" s="86" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F37" s="48"/>
     </row>
@@ -2612,7 +2612,7 @@
         <v>12</v>
       </c>
       <c r="D45" s="86" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="F45" s="48"/>
     </row>
@@ -2625,7 +2625,7 @@
         <v>20</v>
       </c>
       <c r="D46" s="67" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E46" s="68"/>
       <c r="F46" s="69"/>
@@ -2654,7 +2654,7 @@
         <v>768</v>
       </c>
       <c r="D48" s="80" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E48" s="80"/>
       <c r="F48" s="81"/>
@@ -2681,7 +2681,7 @@
         <v>96</v>
       </c>
       <c r="D50" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="F50" s="48"/>
     </row>
@@ -2708,7 +2708,7 @@
         <v>1728</v>
       </c>
       <c r="D52" s="107" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="E52" s="80"/>
       <c r="F52" s="81"/>
@@ -2732,7 +2732,7 @@
         <v>4000</v>
       </c>
       <c r="C54" s="92" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D54" s="93" t="s">
         <v>19</v>
@@ -2767,7 +2767,7 @@
         <v>2</v>
       </c>
       <c r="D57" s="97" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F57" s="48"/>
     </row>
@@ -2780,13 +2780,13 @@
         <v>28</v>
       </c>
       <c r="D58" s="97" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F58" s="48"/>
     </row>
     <row r="59" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B59" s="105" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C59" s="96">
         <f t="shared" ref="C59:C61" si="20">HEX2DEC(B60)-HEX2DEC(B59)</f>
@@ -2799,14 +2799,14 @@
     </row>
     <row r="60" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B60" s="105" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C60" s="96">
         <f t="shared" si="20"/>
         <v>5</v>
       </c>
       <c r="D60" s="97" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F60" s="48"/>
     </row>
@@ -2819,20 +2819,20 @@
         <v>192</v>
       </c>
       <c r="D61" s="97" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="F61" s="48"/>
     </row>
     <row r="62" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B62" s="106" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C62" s="96">
         <f t="shared" ref="C62:C70" si="21">HEX2DEC(B63)-HEX2DEC(B62)</f>
         <v>48</v>
       </c>
       <c r="D62" s="97" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="F62" s="48"/>
     </row>
@@ -2845,38 +2845,38 @@
         <v>3712</v>
       </c>
       <c r="D63" s="97" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="F63" s="48"/>
     </row>
     <row r="64" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B64" s="105" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C64" s="96">
         <f t="shared" si="21"/>
-        <v>1757</v>
+        <v>1727</v>
       </c>
       <c r="D64" s="97" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F64" s="48"/>
     </row>
     <row r="65" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B65" s="105">
-        <v>5680</v>
+        <v>5662</v>
       </c>
       <c r="C65" s="96">
         <f t="shared" si="21"/>
         <v>76</v>
       </c>
       <c r="D65" s="97" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="F65" s="48"/>
     </row>
     <row r="66" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B66" s="118" t="s">
+      <c r="B66" s="108" t="s">
         <v>98</v>
       </c>
       <c r="C66" s="96">
@@ -2884,12 +2884,12 @@
         <v>2600</v>
       </c>
       <c r="D66" s="102" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="F66" s="48"/>
     </row>
     <row r="67" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B67" s="119" t="s">
+      <c r="B67" s="109" t="s">
         <v>99</v>
       </c>
       <c r="C67" s="96">
@@ -2897,59 +2897,59 @@
         <v>3205</v>
       </c>
       <c r="D67" s="97" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="F67" s="48"/>
     </row>
     <row r="68" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B68" s="120" t="s">
+      <c r="B68" s="110" t="s">
         <v>100</v>
       </c>
       <c r="C68" s="103">
         <f t="shared" si="21"/>
-        <v>237</v>
+        <v>267</v>
       </c>
       <c r="D68" s="104" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E68" s="88"/>
       <c r="F68" s="79"/>
     </row>
     <row r="69" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B69" s="119" t="s">
-        <v>87</v>
+      <c r="B69" s="109" t="s">
+        <v>85</v>
       </c>
       <c r="C69" s="96">
         <f t="shared" si="21"/>
         <v>3226</v>
       </c>
       <c r="D69" s="97" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F69" s="48"/>
     </row>
     <row r="70" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B70" s="105" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C70" s="96">
         <f t="shared" si="21"/>
         <v>256</v>
       </c>
       <c r="D70" s="97" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="F70" s="48"/>
     </row>
     <row r="71" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B71" s="121" t="s">
-        <v>82</v>
+      <c r="B71" s="111" t="s">
+        <v>80</v>
       </c>
       <c r="C71" s="98">
         <v>1024</v>
       </c>
       <c r="D71" s="99" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="E71" s="51"/>
       <c r="F71" s="52"/>

</xml_diff>

<commit_message>
Minor change to not update the game-bar when samples are played.  Also updated documentation adding a section on the profiler-based optimization made.  Also updated the memory maps (appendix).
</commit_message>
<xml_diff>
--- a/docs/Memory.xlsx
+++ b/docs/Memory.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\Beeb\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09CB818F-0584-4982-96EA-42E8EB7C1039}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2678569-AA9D-492B-B13B-6833C80C52A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16140" xr2:uid="{C0DF3A0D-E6A9-4F13-8EDD-5DE46AD6E0DB}"/>
   </bookViews>
@@ -854,7 +854,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="144">
+  <cellXfs count="138">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1097,36 +1097,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1181,20 +1151,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="34" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="35" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1204,7 +1160,37 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1550,35 +1536,35 @@
   <sheetData>
     <row r="1" spans="2:18" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="2" spans="2:18" x14ac:dyDescent="0.35">
-      <c r="B2" s="106" t="s">
+      <c r="B2" s="132" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="108" t="s">
-        <v>0</v>
-      </c>
-      <c r="D2" s="103" t="s">
+      <c r="C2" s="134" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" s="129" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="102" t="s">
+      <c r="E2" s="128" t="s">
         <v>22</v>
       </c>
-      <c r="F2" s="105"/>
-      <c r="G2" s="102" t="s">
+      <c r="F2" s="131"/>
+      <c r="G2" s="128" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="103"/>
-      <c r="I2" s="104" t="s">
+      <c r="H2" s="129"/>
+      <c r="I2" s="130" t="s">
         <v>12</v>
       </c>
-      <c r="J2" s="105"/>
-      <c r="K2" s="102" t="s">
+      <c r="J2" s="131"/>
+      <c r="K2" s="128" t="s">
         <v>14</v>
       </c>
-      <c r="L2" s="103"/>
-      <c r="M2" s="104" t="s">
+      <c r="L2" s="129"/>
+      <c r="M2" s="130" t="s">
         <v>15</v>
       </c>
-      <c r="N2" s="105"/>
+      <c r="N2" s="131"/>
       <c r="O2" s="43" t="s">
         <v>6</v>
       </c>
@@ -1589,35 +1575,35 @@
       <c r="R2" s="15"/>
     </row>
     <row r="3" spans="2:18" x14ac:dyDescent="0.35">
-      <c r="B3" s="107"/>
-      <c r="C3" s="109"/>
-      <c r="D3" s="110"/>
-      <c r="E3" s="109" t="s">
+      <c r="B3" s="133"/>
+      <c r="C3" s="135"/>
+      <c r="D3" s="136"/>
+      <c r="E3" s="135" t="s">
         <v>23</v>
       </c>
-      <c r="F3" s="111"/>
-      <c r="G3" s="109" t="s">
+      <c r="F3" s="137"/>
+      <c r="G3" s="135" t="s">
         <v>23</v>
       </c>
-      <c r="H3" s="110"/>
+      <c r="H3" s="136"/>
       <c r="I3" s="41"/>
       <c r="J3" s="40"/>
-      <c r="K3" s="109" t="s">
+      <c r="K3" s="135" t="s">
         <v>23</v>
       </c>
-      <c r="L3" s="110"/>
-      <c r="M3" s="111" t="s">
+      <c r="L3" s="136"/>
+      <c r="M3" s="137" t="s">
         <v>23</v>
       </c>
-      <c r="N3" s="111"/>
+      <c r="N3" s="137"/>
       <c r="O3" s="42"/>
       <c r="P3" s="24"/>
       <c r="R3" s="15"/>
     </row>
     <row r="4" spans="2:18" x14ac:dyDescent="0.35">
-      <c r="B4" s="107"/>
-      <c r="C4" s="109"/>
-      <c r="D4" s="110"/>
+      <c r="B4" s="133"/>
+      <c r="C4" s="135"/>
+      <c r="D4" s="136"/>
       <c r="E4" s="21" t="s">
         <v>0</v>
       </c>
@@ -2243,7 +2229,7 @@
       <c r="P17" s="3"/>
     </row>
     <row r="18" spans="2:16" ht="19" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B18" s="143" t="s">
+      <c r="B18" s="127" t="s">
         <v>109</v>
       </c>
       <c r="P18" s="3"/>
@@ -2762,7 +2748,7 @@
       <c r="E48" s="70"/>
       <c r="F48" s="71"/>
     </row>
-    <row r="49" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="49" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B49" s="72" t="str">
         <f t="shared" ref="B49:B51" si="18">DEC2HEX(HEX2DEC(B50)-C49)</f>
         <v>2CA0</v>
@@ -2776,7 +2762,7 @@
       <c r="E49" s="79"/>
       <c r="F49" s="80"/>
     </row>
-    <row r="50" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="50" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B50" s="46" t="str">
         <f t="shared" si="18"/>
         <v>2FA0</v>
@@ -2789,7 +2775,7 @@
       </c>
       <c r="F50" s="47"/>
     </row>
-    <row r="51" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="51" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B51" s="46" t="str">
         <f t="shared" si="18"/>
         <v>3000</v>
@@ -2802,7 +2788,7 @@
       </c>
       <c r="F51" s="47"/>
     </row>
-    <row r="52" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="52" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B52" s="46" t="str">
         <f>DEC2HEX(HEX2DEC(B53)-C52)</f>
         <v>3060</v>
@@ -2816,61 +2802,61 @@
       </c>
       <c r="F52" s="47"/>
     </row>
-    <row r="53" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B53" s="121" t="str">
+    <row r="53" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B53" s="111" t="str">
         <f>DEC2HEX(HEX2DEC(B54)-C53)</f>
         <v>3140</v>
       </c>
-      <c r="C53" s="122">
+      <c r="C53" s="112">
         <v>1728</v>
       </c>
-      <c r="D53" s="123" t="s">
+      <c r="D53" s="113" t="s">
         <v>92</v>
       </c>
-      <c r="E53" s="124"/>
-      <c r="F53" s="125"/>
-    </row>
-    <row r="54" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B54" s="126" t="str">
+      <c r="E53" s="114"/>
+      <c r="F53" s="115"/>
+    </row>
+    <row r="54" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B54" s="116" t="str">
         <f>DEC2HEX(HEX2DEC(B55)-C54)</f>
         <v>3800</v>
       </c>
-      <c r="C54" s="127">
+      <c r="C54" s="117">
         <f>2048</f>
         <v>2048</v>
       </c>
-      <c r="D54" s="128" t="s">
+      <c r="D54" s="118" t="s">
         <v>30</v>
       </c>
-      <c r="E54" s="115"/>
-      <c r="F54" s="116"/>
-    </row>
-    <row r="55" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B55" s="129">
+      <c r="E54" s="105"/>
+      <c r="F54" s="106"/>
+    </row>
+    <row r="55" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B55" s="119">
         <v>4000</v>
       </c>
-      <c r="C55" s="130" t="s">
+      <c r="C55" s="120" t="s">
         <v>85</v>
       </c>
-      <c r="D55" s="131" t="s">
+      <c r="D55" s="121" t="s">
         <v>19</v>
       </c>
-      <c r="E55" s="132"/>
-      <c r="F55" s="133"/>
-    </row>
-    <row r="56" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="E55" s="122"/>
+      <c r="F55" s="123"/>
+    </row>
+    <row r="56" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B56" s="17"/>
       <c r="C56" s="17"/>
       <c r="D56" s="17"/>
     </row>
-    <row r="57" spans="2:7" ht="19" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B57" s="142" t="s">
+    <row r="57" spans="2:10" ht="19" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B57" s="126" t="s">
         <v>108</v>
       </c>
       <c r="C57" s="17"/>
       <c r="D57" s="17"/>
     </row>
-    <row r="58" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="58" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B58" s="94" t="s">
         <v>7</v>
       </c>
@@ -2883,179 +2869,185 @@
       <c r="E58" s="52"/>
       <c r="F58" s="53"/>
     </row>
-    <row r="59" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B59" s="120">
+    <row r="59" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B59" s="110">
         <v>4000</v>
       </c>
-      <c r="C59" s="113">
+      <c r="C59" s="103">
         <f>HEX2DEC(B60)-HEX2DEC(B59)</f>
         <v>2</v>
       </c>
-      <c r="D59" s="114" t="s">
+      <c r="D59" s="104" t="s">
         <v>69</v>
       </c>
-      <c r="E59" s="115"/>
-      <c r="F59" s="116"/>
-    </row>
-    <row r="60" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B60" s="120">
+      <c r="E59" s="105"/>
+      <c r="F59" s="106"/>
+      <c r="J59">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="60" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B60" s="110">
         <v>4002</v>
       </c>
-      <c r="C60" s="113">
+      <c r="C60" s="103">
         <f>HEX2DEC(B61)-HEX2DEC(B60)</f>
         <v>28</v>
       </c>
-      <c r="D60" s="114" t="s">
+      <c r="D60" s="104" t="s">
         <v>70</v>
       </c>
-      <c r="E60" s="115"/>
-      <c r="F60" s="116"/>
-    </row>
-    <row r="61" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B61" s="112" t="s">
+      <c r="E60" s="105"/>
+      <c r="F60" s="106"/>
+      <c r="J60">
+        <v>59344</v>
+      </c>
+    </row>
+    <row r="61" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B61" s="102" t="s">
         <v>91</v>
       </c>
-      <c r="C61" s="113">
+      <c r="C61" s="103">
         <f t="shared" ref="C61:C65" si="19">HEX2DEC(B62)-HEX2DEC(B61)</f>
         <v>16</v>
       </c>
-      <c r="D61" s="114" t="s">
+      <c r="D61" s="104" t="s">
         <v>29</v>
       </c>
-      <c r="E61" s="115"/>
-      <c r="F61" s="116"/>
-    </row>
-    <row r="62" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B62" s="112" t="s">
+      <c r="E61" s="105"/>
+      <c r="F61" s="106"/>
+    </row>
+    <row r="62" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B62" s="102" t="s">
         <v>88</v>
       </c>
-      <c r="C62" s="113">
+      <c r="C62" s="103">
         <f t="shared" si="19"/>
         <v>5</v>
       </c>
-      <c r="D62" s="114" t="s">
+      <c r="D62" s="104" t="s">
         <v>71</v>
       </c>
-      <c r="E62" s="115"/>
-      <c r="F62" s="116"/>
-    </row>
-    <row r="63" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B63" s="112">
+      <c r="E62" s="105"/>
+      <c r="F62" s="106"/>
+    </row>
+    <row r="63" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B63" s="102">
         <v>4033</v>
       </c>
-      <c r="C63" s="113">
+      <c r="C63" s="103">
         <f t="shared" si="19"/>
         <v>192</v>
       </c>
-      <c r="D63" s="114" t="s">
+      <c r="D63" s="104" t="s">
         <v>72</v>
       </c>
-      <c r="E63" s="115"/>
-      <c r="F63" s="116"/>
-    </row>
-    <row r="64" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B64" s="112" t="s">
+      <c r="E63" s="105"/>
+      <c r="F63" s="106"/>
+    </row>
+    <row r="64" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B64" s="102" t="s">
         <v>89</v>
       </c>
-      <c r="C64" s="113">
+      <c r="C64" s="103">
         <f t="shared" si="19"/>
         <v>48</v>
       </c>
-      <c r="D64" s="114" t="s">
+      <c r="D64" s="104" t="s">
         <v>73</v>
       </c>
-      <c r="E64" s="115"/>
-      <c r="F64" s="116"/>
+      <c r="E64" s="105"/>
+      <c r="F64" s="106"/>
       <c r="G64" s="97"/>
     </row>
     <row r="65" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B65" s="112">
+      <c r="B65" s="102">
         <v>4123</v>
       </c>
-      <c r="C65" s="113">
+      <c r="C65" s="103">
         <f t="shared" si="19"/>
         <v>3712</v>
       </c>
-      <c r="D65" s="114" t="s">
+      <c r="D65" s="104" t="s">
         <v>74</v>
       </c>
-      <c r="E65" s="115"/>
-      <c r="F65" s="116"/>
+      <c r="E65" s="105"/>
+      <c r="F65" s="106"/>
       <c r="G65" s="96"/>
     </row>
     <row r="66" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B66" s="112" t="s">
+      <c r="B66" s="102" t="s">
         <v>90</v>
       </c>
-      <c r="C66" s="113">
+      <c r="C66" s="103">
         <f t="shared" ref="C66:C72" si="20">HEX2DEC(B67)-HEX2DEC(B66)</f>
         <v>2304</v>
       </c>
-      <c r="D66" s="114" t="s">
+      <c r="D66" s="104" t="s">
         <v>96</v>
       </c>
-      <c r="E66" s="115"/>
-      <c r="F66" s="116"/>
+      <c r="E66" s="105"/>
+      <c r="F66" s="106"/>
       <c r="G66" s="96"/>
     </row>
     <row r="67" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B67" s="112" t="s">
+      <c r="B67" s="102" t="s">
         <v>95</v>
       </c>
-      <c r="C67" s="113">
+      <c r="C67" s="103">
         <f t="shared" si="20"/>
         <v>1995</v>
       </c>
-      <c r="D67" s="114" t="s">
+      <c r="D67" s="104" t="s">
         <v>75</v>
       </c>
-      <c r="E67" s="115"/>
-      <c r="F67" s="116"/>
+      <c r="E67" s="105"/>
+      <c r="F67" s="106"/>
       <c r="G67" s="96"/>
     </row>
     <row r="68" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B68" s="112" t="s">
+      <c r="B68" s="102" t="s">
         <v>97</v>
       </c>
-      <c r="C68" s="113">
+      <c r="C68" s="103">
         <f t="shared" si="20"/>
         <v>84</v>
       </c>
-      <c r="D68" s="114" t="s">
+      <c r="D68" s="104" t="s">
         <v>76</v>
       </c>
-      <c r="E68" s="115"/>
-      <c r="F68" s="116"/>
+      <c r="E68" s="105"/>
+      <c r="F68" s="106"/>
       <c r="G68" s="96"/>
     </row>
     <row r="69" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B69" s="117" t="s">
+      <c r="B69" s="107" t="s">
         <v>98</v>
       </c>
-      <c r="C69" s="113">
+      <c r="C69" s="103">
         <f t="shared" si="20"/>
         <v>2634</v>
       </c>
-      <c r="D69" s="118" t="s">
+      <c r="D69" s="108" t="s">
         <v>101</v>
       </c>
-      <c r="E69" s="115"/>
-      <c r="F69" s="116"/>
+      <c r="E69" s="105"/>
+      <c r="F69" s="106"/>
       <c r="G69" s="98"/>
     </row>
     <row r="70" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B70" s="119" t="s">
+      <c r="B70" s="109" t="s">
         <v>99</v>
       </c>
-      <c r="C70" s="113">
+      <c r="C70" s="103">
         <f t="shared" si="20"/>
         <v>3203</v>
       </c>
-      <c r="D70" s="114" t="s">
+      <c r="D70" s="104" t="s">
         <v>77</v>
       </c>
-      <c r="E70" s="115"/>
-      <c r="F70" s="116"/>
+      <c r="E70" s="105"/>
+      <c r="F70" s="106"/>
       <c r="G70" s="99"/>
     </row>
     <row r="71" spans="2:7" x14ac:dyDescent="0.35">
@@ -3103,7 +3095,7 @@
       <c r="C74" s="90"/>
     </row>
     <row r="75" spans="2:7" ht="19" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B75" s="141" t="s">
+      <c r="B75" s="125" t="s">
         <v>106</v>
       </c>
       <c r="C75" s="90"/>
@@ -3122,187 +3114,187 @@
       <c r="F76" s="53"/>
     </row>
     <row r="77" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B77" s="121" t="str">
+      <c r="B77" s="111" t="str">
         <f>DEC2HEX(HEX2DEC(B78)-C77)</f>
         <v>3140</v>
       </c>
-      <c r="C77" s="122">
+      <c r="C77" s="112">
         <v>1728</v>
       </c>
-      <c r="D77" s="123" t="s">
+      <c r="D77" s="113" t="s">
         <v>92</v>
       </c>
-      <c r="E77" s="124"/>
-      <c r="F77" s="125"/>
+      <c r="E77" s="114"/>
+      <c r="F77" s="115"/>
     </row>
     <row r="78" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B78" s="126" t="str">
+      <c r="B78" s="116" t="str">
         <f>DEC2HEX(HEX2DEC(B79)-C78)</f>
         <v>3800</v>
       </c>
-      <c r="C78" s="127">
+      <c r="C78" s="117">
         <f>2048</f>
         <v>2048</v>
       </c>
-      <c r="D78" s="128" t="s">
+      <c r="D78" s="118" t="s">
         <v>30</v>
       </c>
-      <c r="E78" s="115"/>
-      <c r="F78" s="116"/>
+      <c r="E78" s="105"/>
+      <c r="F78" s="106"/>
     </row>
     <row r="79" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B79" s="120">
+      <c r="B79" s="110">
         <v>4000</v>
       </c>
-      <c r="C79" s="113">
+      <c r="C79" s="103">
         <f>HEX2DEC(B80)-HEX2DEC(B79)</f>
         <v>2</v>
       </c>
-      <c r="D79" s="114" t="s">
+      <c r="D79" s="104" t="s">
         <v>69</v>
       </c>
-      <c r="E79" s="115"/>
-      <c r="F79" s="116"/>
+      <c r="E79" s="105"/>
+      <c r="F79" s="106"/>
     </row>
     <row r="80" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B80" s="120">
+      <c r="B80" s="110">
         <v>4002</v>
       </c>
-      <c r="C80" s="113">
+      <c r="C80" s="103">
         <f>HEX2DEC(B81)-HEX2DEC(B80)</f>
         <v>28</v>
       </c>
-      <c r="D80" s="114" t="s">
+      <c r="D80" s="104" t="s">
         <v>70</v>
       </c>
-      <c r="E80" s="115"/>
-      <c r="F80" s="116"/>
+      <c r="E80" s="105"/>
+      <c r="F80" s="106"/>
     </row>
     <row r="81" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B81" s="112" t="s">
+      <c r="B81" s="102" t="s">
         <v>91</v>
       </c>
-      <c r="C81" s="113">
+      <c r="C81" s="103">
         <f t="shared" ref="C81:C91" si="21">HEX2DEC(B82)-HEX2DEC(B81)</f>
         <v>16</v>
       </c>
-      <c r="D81" s="114" t="s">
+      <c r="D81" s="104" t="s">
         <v>29</v>
       </c>
-      <c r="E81" s="115"/>
-      <c r="F81" s="116"/>
+      <c r="E81" s="105"/>
+      <c r="F81" s="106"/>
     </row>
     <row r="82" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B82" s="112" t="s">
+      <c r="B82" s="102" t="s">
         <v>88</v>
       </c>
-      <c r="C82" s="113">
+      <c r="C82" s="103">
         <f t="shared" si="21"/>
         <v>5</v>
       </c>
-      <c r="D82" s="114" t="s">
+      <c r="D82" s="104" t="s">
         <v>71</v>
       </c>
-      <c r="E82" s="115"/>
-      <c r="F82" s="116"/>
+      <c r="E82" s="105"/>
+      <c r="F82" s="106"/>
     </row>
     <row r="83" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B83" s="112">
+      <c r="B83" s="102">
         <v>4033</v>
       </c>
-      <c r="C83" s="113">
+      <c r="C83" s="103">
         <f t="shared" si="21"/>
         <v>192</v>
       </c>
-      <c r="D83" s="114" t="s">
+      <c r="D83" s="104" t="s">
         <v>72</v>
       </c>
-      <c r="E83" s="115"/>
-      <c r="F83" s="116"/>
+      <c r="E83" s="105"/>
+      <c r="F83" s="106"/>
     </row>
     <row r="84" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B84" s="112" t="s">
+      <c r="B84" s="102" t="s">
         <v>89</v>
       </c>
-      <c r="C84" s="113">
+      <c r="C84" s="103">
         <f t="shared" si="21"/>
         <v>48</v>
       </c>
-      <c r="D84" s="114" t="s">
+      <c r="D84" s="104" t="s">
         <v>73</v>
       </c>
-      <c r="E84" s="115"/>
-      <c r="F84" s="116"/>
+      <c r="E84" s="105"/>
+      <c r="F84" s="106"/>
     </row>
     <row r="85" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B85" s="112">
+      <c r="B85" s="102">
         <v>4123</v>
       </c>
-      <c r="C85" s="113">
+      <c r="C85" s="103">
         <f t="shared" si="21"/>
         <v>3712</v>
       </c>
-      <c r="D85" s="114" t="s">
+      <c r="D85" s="104" t="s">
         <v>74</v>
       </c>
-      <c r="E85" s="115"/>
-      <c r="F85" s="116"/>
+      <c r="E85" s="105"/>
+      <c r="F85" s="106"/>
     </row>
     <row r="86" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B86" s="112" t="s">
+      <c r="B86" s="102" t="s">
         <v>90</v>
       </c>
-      <c r="C86" s="113">
+      <c r="C86" s="103">
         <f t="shared" si="21"/>
         <v>2304</v>
       </c>
-      <c r="D86" s="114" t="s">
+      <c r="D86" s="104" t="s">
         <v>96</v>
       </c>
-      <c r="E86" s="115"/>
-      <c r="F86" s="116"/>
+      <c r="E86" s="105"/>
+      <c r="F86" s="106"/>
     </row>
     <row r="87" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B87" s="112" t="s">
+      <c r="B87" s="102" t="s">
         <v>95</v>
       </c>
-      <c r="C87" s="113">
+      <c r="C87" s="103">
         <f t="shared" si="21"/>
         <v>1995</v>
       </c>
-      <c r="D87" s="114" t="s">
+      <c r="D87" s="104" t="s">
         <v>75</v>
       </c>
-      <c r="E87" s="115"/>
-      <c r="F87" s="116"/>
+      <c r="E87" s="105"/>
+      <c r="F87" s="106"/>
     </row>
     <row r="88" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B88" s="112" t="s">
+      <c r="B88" s="102" t="s">
         <v>97</v>
       </c>
-      <c r="C88" s="113">
+      <c r="C88" s="103">
         <f t="shared" si="21"/>
         <v>84</v>
       </c>
-      <c r="D88" s="114" t="s">
+      <c r="D88" s="104" t="s">
         <v>76</v>
       </c>
-      <c r="E88" s="115"/>
-      <c r="F88" s="116"/>
+      <c r="E88" s="105"/>
+      <c r="F88" s="106"/>
     </row>
     <row r="89" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B89" s="117" t="s">
+      <c r="B89" s="107" t="s">
         <v>98</v>
       </c>
-      <c r="C89" s="113">
+      <c r="C89" s="103">
         <f t="shared" si="21"/>
         <v>2064</v>
       </c>
-      <c r="D89" s="118" t="s">
+      <c r="D89" s="108" t="s">
         <v>104</v>
       </c>
-      <c r="E89" s="115"/>
-      <c r="F89" s="116"/>
+      <c r="E89" s="105"/>
+      <c r="F89" s="106"/>
     </row>
     <row r="90" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B90" s="99" t="s">
@@ -3347,7 +3339,7 @@
       <c r="B93" s="45"/>
     </row>
     <row r="94" spans="2:6" ht="19" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B94" s="141" t="s">
+      <c r="B94" s="125" t="s">
         <v>107</v>
       </c>
     </row>
@@ -3365,116 +3357,108 @@
       <c r="F95" s="53"/>
     </row>
     <row r="96" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B96" s="134">
+      <c r="B96" s="96">
         <v>4000</v>
       </c>
-      <c r="C96" s="135">
+      <c r="C96" s="90">
         <f>HEX2DEC(B97)-HEX2DEC(B96)</f>
         <v>2</v>
       </c>
-      <c r="D96" s="136" t="s">
+      <c r="D96" s="91" t="s">
         <v>69</v>
       </c>
-      <c r="E96" s="137"/>
-      <c r="F96" s="138"/>
+      <c r="F96" s="47"/>
     </row>
     <row r="97" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B97" s="134">
+      <c r="B97" s="96">
         <v>4002</v>
       </c>
-      <c r="C97" s="135">
+      <c r="C97" s="90">
         <f>HEX2DEC(B98)-HEX2DEC(B97)</f>
         <v>28</v>
       </c>
-      <c r="D97" s="136" t="s">
+      <c r="D97" s="91" t="s">
         <v>70</v>
       </c>
-      <c r="E97" s="137"/>
-      <c r="F97" s="138"/>
+      <c r="F97" s="47"/>
     </row>
     <row r="98" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B98" s="139" t="s">
+      <c r="B98" s="97" t="s">
         <v>91</v>
       </c>
-      <c r="C98" s="135">
+      <c r="C98" s="90">
         <f t="shared" ref="C98:C110" si="22">HEX2DEC(B99)-HEX2DEC(B98)</f>
         <v>16</v>
       </c>
-      <c r="D98" s="136" t="s">
+      <c r="D98" s="91" t="s">
         <v>29</v>
       </c>
-      <c r="E98" s="137"/>
-      <c r="F98" s="138"/>
+      <c r="F98" s="47"/>
     </row>
     <row r="99" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B99" s="139" t="s">
+      <c r="B99" s="97" t="s">
         <v>88</v>
       </c>
-      <c r="C99" s="135">
+      <c r="C99" s="90">
         <f t="shared" si="22"/>
         <v>5</v>
       </c>
-      <c r="D99" s="136" t="s">
+      <c r="D99" s="91" t="s">
         <v>71</v>
       </c>
-      <c r="E99" s="137"/>
-      <c r="F99" s="138"/>
+      <c r="F99" s="47"/>
     </row>
     <row r="100" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B100" s="139">
+      <c r="B100" s="97">
         <v>4033</v>
       </c>
-      <c r="C100" s="135">
+      <c r="C100" s="90">
         <f t="shared" si="22"/>
         <v>192</v>
       </c>
-      <c r="D100" s="136" t="s">
+      <c r="D100" s="91" t="s">
         <v>72</v>
       </c>
-      <c r="E100" s="137"/>
-      <c r="F100" s="138"/>
+      <c r="F100" s="47"/>
     </row>
     <row r="101" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B101" s="139" t="s">
+      <c r="B101" s="97" t="s">
         <v>89</v>
       </c>
-      <c r="C101" s="135">
+      <c r="C101" s="90">
         <f t="shared" si="22"/>
         <v>48</v>
       </c>
-      <c r="D101" s="136" t="s">
+      <c r="D101" s="91" t="s">
         <v>73</v>
       </c>
-      <c r="E101" s="137"/>
-      <c r="F101" s="138"/>
+      <c r="F101" s="47"/>
     </row>
     <row r="102" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B102" s="139">
+      <c r="B102" s="97">
         <v>4123</v>
       </c>
-      <c r="C102" s="135">
+      <c r="C102" s="90">
         <f t="shared" si="22"/>
         <v>3712</v>
       </c>
-      <c r="D102" s="136" t="s">
+      <c r="D102" s="91" t="s">
         <v>74</v>
       </c>
-      <c r="E102" s="137"/>
-      <c r="F102" s="138"/>
+      <c r="F102" s="47"/>
     </row>
     <row r="103" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B103" s="139" t="s">
+      <c r="B103" s="97" t="s">
         <v>90</v>
       </c>
-      <c r="C103" s="135">
+      <c r="C103" s="90">
         <f t="shared" si="22"/>
         <v>2304</v>
       </c>
-      <c r="D103" s="136" t="s">
+      <c r="D103" s="91" t="s">
         <v>96</v>
       </c>
-      <c r="E103" s="137"/>
-      <c r="F103" s="138"/>
+      <c r="F103" s="47"/>
     </row>
     <row r="104" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B104" s="97" t="s">
@@ -3490,60 +3474,60 @@
       <c r="F104" s="47"/>
     </row>
     <row r="105" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B105" s="112" t="s">
+      <c r="B105" s="102" t="s">
         <v>97</v>
       </c>
-      <c r="C105" s="113">
+      <c r="C105" s="103">
         <f t="shared" si="22"/>
         <v>84</v>
       </c>
-      <c r="D105" s="114" t="s">
+      <c r="D105" s="104" t="s">
         <v>76</v>
       </c>
-      <c r="E105" s="115"/>
-      <c r="F105" s="116"/>
+      <c r="E105" s="105"/>
+      <c r="F105" s="106"/>
     </row>
     <row r="106" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B106" s="117" t="s">
+      <c r="B106" s="107" t="s">
         <v>98</v>
       </c>
-      <c r="C106" s="113">
+      <c r="C106" s="103">
         <f t="shared" si="22"/>
         <v>2047</v>
       </c>
-      <c r="D106" s="118" t="s">
+      <c r="D106" s="108" t="s">
         <v>105</v>
       </c>
-      <c r="E106" s="115"/>
-      <c r="F106" s="116"/>
+      <c r="E106" s="105"/>
+      <c r="F106" s="106"/>
     </row>
     <row r="107" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B107" s="117" t="s">
+      <c r="B107" s="107" t="s">
         <v>102</v>
       </c>
-      <c r="C107" s="113">
+      <c r="C107" s="103">
         <f t="shared" si="22"/>
         <v>587</v>
       </c>
-      <c r="D107" s="140" t="s">
+      <c r="D107" s="124" t="s">
         <v>82</v>
       </c>
-      <c r="E107" s="115"/>
-      <c r="F107" s="116"/>
+      <c r="E107" s="105"/>
+      <c r="F107" s="106"/>
     </row>
     <row r="108" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B108" s="119" t="s">
+      <c r="B108" s="109" t="s">
         <v>99</v>
       </c>
-      <c r="C108" s="113">
+      <c r="C108" s="103">
         <f t="shared" si="22"/>
         <v>3203</v>
       </c>
-      <c r="D108" s="114" t="s">
+      <c r="D108" s="104" t="s">
         <v>77</v>
       </c>
-      <c r="E108" s="115"/>
-      <c r="F108" s="116"/>
+      <c r="E108" s="105"/>
+      <c r="F108" s="106"/>
     </row>
     <row r="109" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B109" s="99" t="s">

</xml_diff>

<commit_message>
drawObject common case optimizations. Plus code size optimizations.
</commit_message>
<xml_diff>
--- a/docs/Memory.xlsx
+++ b/docs/Memory.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\Beeb\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2678569-AA9D-492B-B13B-6833C80C52A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8582F92E-0FE5-425A-B2A4-F3EBF4D747EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16140" xr2:uid="{C0DF3A0D-E6A9-4F13-8EDD-5DE46AD6E0DB}"/>
+    <workbookView xWindow="380" yWindow="380" windowWidth="21950" windowHeight="14140" xr2:uid="{C0DF3A0D-E6A9-4F13-8EDD-5DE46AD6E0DB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="116">
   <si>
     <t>Quantity</t>
   </si>
@@ -203,9 +203,6 @@
     <t>elevator sprite</t>
   </si>
   <si>
-    <t>4 elevator sprites</t>
-  </si>
-  <si>
     <t>Sprite health bar table</t>
   </si>
   <si>
@@ -366,6 +363,27 @@
   </si>
   <si>
     <t>Gameplay</t>
+  </si>
+  <si>
+    <t>…</t>
+  </si>
+  <si>
+    <t>object extents</t>
+  </si>
+  <si>
+    <t>Object extents</t>
+  </si>
+  <si>
+    <t>10F5</t>
+  </si>
+  <si>
+    <t>&amp;10F5</t>
+  </si>
+  <si>
+    <t>1 elevator sprite</t>
+  </si>
+  <si>
+    <t>3 elevator sprites</t>
   </si>
 </sst>
 </file>
@@ -854,7 +872,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="138">
+  <cellXfs count="159">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
@@ -999,8 +1017,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1048,16 +1064,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1080,12 +1086,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="11" fontId="3" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1140,27 +1140,35 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="34" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="35" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1190,6 +1198,75 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="11" fontId="3" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1526,7 +1603,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10CD322F-64B0-476A-AEFE-F468CB566666}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="B1:R111"/>
+  <dimension ref="B1:R107"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="2.81640625" customWidth="1"/>
@@ -1536,74 +1613,74 @@
   <sheetData>
     <row r="1" spans="2:18" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="2" spans="2:18" x14ac:dyDescent="0.35">
-      <c r="B2" s="132" t="s">
+      <c r="B2" s="126" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="134" t="s">
-        <v>0</v>
-      </c>
-      <c r="D2" s="129" t="s">
+      <c r="C2" s="128" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" s="123" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="128" t="s">
+      <c r="E2" s="122" t="s">
         <v>22</v>
       </c>
-      <c r="F2" s="131"/>
-      <c r="G2" s="128" t="s">
+      <c r="F2" s="125"/>
+      <c r="G2" s="122" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="129"/>
-      <c r="I2" s="130" t="s">
+      <c r="H2" s="123"/>
+      <c r="I2" s="124" t="s">
         <v>12</v>
       </c>
-      <c r="J2" s="131"/>
-      <c r="K2" s="128" t="s">
+      <c r="J2" s="125"/>
+      <c r="K2" s="122" t="s">
         <v>14</v>
       </c>
-      <c r="L2" s="129"/>
-      <c r="M2" s="130" t="s">
+      <c r="L2" s="123"/>
+      <c r="M2" s="124" t="s">
         <v>15</v>
       </c>
-      <c r="N2" s="131"/>
+      <c r="N2" s="125"/>
       <c r="O2" s="43" t="s">
         <v>6</v>
       </c>
       <c r="P2" s="14" t="str">
         <f>DEC2HEX(HEX2DEC(3140)-P14)</f>
-        <v>2CA0</v>
+        <v>2CB8</v>
       </c>
       <c r="R2" s="15"/>
     </row>
     <row r="3" spans="2:18" x14ac:dyDescent="0.35">
-      <c r="B3" s="133"/>
-      <c r="C3" s="135"/>
-      <c r="D3" s="136"/>
-      <c r="E3" s="135" t="s">
+      <c r="B3" s="127"/>
+      <c r="C3" s="129"/>
+      <c r="D3" s="130"/>
+      <c r="E3" s="129" t="s">
         <v>23</v>
       </c>
-      <c r="F3" s="137"/>
-      <c r="G3" s="135" t="s">
+      <c r="F3" s="131"/>
+      <c r="G3" s="129" t="s">
         <v>23</v>
       </c>
-      <c r="H3" s="136"/>
+      <c r="H3" s="130"/>
       <c r="I3" s="41"/>
       <c r="J3" s="40"/>
-      <c r="K3" s="135" t="s">
+      <c r="K3" s="129" t="s">
         <v>23</v>
       </c>
-      <c r="L3" s="136"/>
-      <c r="M3" s="137" t="s">
+      <c r="L3" s="130"/>
+      <c r="M3" s="131" t="s">
         <v>23</v>
       </c>
-      <c r="N3" s="137"/>
+      <c r="N3" s="131"/>
       <c r="O3" s="42"/>
       <c r="P3" s="24"/>
       <c r="R3" s="15"/>
     </row>
     <row r="4" spans="2:18" x14ac:dyDescent="0.35">
-      <c r="B4" s="133"/>
-      <c r="C4" s="135"/>
-      <c r="D4" s="136"/>
+      <c r="B4" s="127"/>
+      <c r="C4" s="129"/>
+      <c r="D4" s="130"/>
       <c r="E4" s="21" t="s">
         <v>0</v>
       </c>
@@ -1868,11 +1945,11 @@
         <v>24</v>
       </c>
       <c r="E9" s="30">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F9" s="30">
         <f>E9*$D9</f>
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="G9" s="4">
         <v>0</v>
@@ -1903,16 +1980,16 @@
         <v>0</v>
       </c>
       <c r="O9" s="4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P9" s="6">
         <f>O9*$D9</f>
-        <v>96</v>
+        <v>72</v>
       </c>
     </row>
     <row r="10" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B10" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C10" s="19">
         <v>4</v>
@@ -2072,7 +2149,7 @@
     </row>
     <row r="13" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B13" s="38" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C13" s="34">
         <v>1</v>
@@ -2132,7 +2209,7 @@
       <c r="E14" s="28"/>
       <c r="F14" s="28">
         <f>SUM(F5:F13)</f>
-        <v>192</v>
+        <v>216</v>
       </c>
       <c r="G14" s="19"/>
       <c r="H14" s="20">
@@ -2157,7 +2234,7 @@
       <c r="O14" s="19"/>
       <c r="P14" s="29">
         <f>SUM(P5:P13)</f>
-        <v>1184</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="15" spans="2:18" x14ac:dyDescent="0.35">
@@ -2168,7 +2245,7 @@
       <c r="D15" s="20"/>
       <c r="E15" s="28"/>
       <c r="F15" s="30">
-        <v>192</v>
+        <v>216</v>
       </c>
       <c r="G15" s="4"/>
       <c r="H15" s="5">
@@ -2200,7 +2277,7 @@
       </c>
       <c r="F16" s="16">
         <f>256-F14</f>
-        <v>64</v>
+        <v>40</v>
       </c>
       <c r="G16" s="10"/>
       <c r="H16" s="44">
@@ -2229,81 +2306,83 @@
       <c r="P17" s="3"/>
     </row>
     <row r="18" spans="2:16" ht="19" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B18" s="127" t="s">
-        <v>109</v>
+      <c r="B18" s="111" t="s">
+        <v>108</v>
       </c>
       <c r="P18" s="3"/>
     </row>
     <row r="19" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B19" s="62" t="s">
+      <c r="B19" s="60" t="s">
         <v>7</v>
       </c>
       <c r="C19" s="56" t="s">
         <v>20</v>
       </c>
-      <c r="D19" s="63" t="s">
+      <c r="D19" s="61" t="s">
         <v>8</v>
       </c>
       <c r="E19" s="55"/>
       <c r="F19" s="57"/>
-      <c r="H19" s="58" t="s">
+      <c r="H19" s="119" t="s">
         <v>50</v>
       </c>
-      <c r="I19" s="52"/>
-      <c r="J19" s="52"/>
-      <c r="K19" s="59" t="s">
+      <c r="I19" s="55"/>
+      <c r="J19" s="55"/>
+      <c r="K19" s="120" t="s">
         <v>7</v>
       </c>
-      <c r="L19" s="60" t="s">
+      <c r="L19" s="56" t="s">
         <v>2</v>
       </c>
-      <c r="M19" s="59" t="s">
+      <c r="M19" s="120" t="s">
         <v>39</v>
       </c>
-      <c r="N19" s="52"/>
-      <c r="O19" s="53"/>
+      <c r="N19" s="55"/>
+      <c r="O19" s="57"/>
     </row>
     <row r="20" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B20" s="61">
-        <v>0</v>
-      </c>
-      <c r="C20" s="64">
+      <c r="B20" s="59">
+        <v>0</v>
+      </c>
+      <c r="C20" s="62">
         <v>144</v>
       </c>
       <c r="D20" s="55" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E20" s="55"/>
       <c r="F20" s="57"/>
-      <c r="H20" s="46" t="s">
+      <c r="H20" s="59" t="s">
         <v>38</v>
       </c>
-      <c r="I20" s="17"/>
-      <c r="K20" t="s">
+      <c r="I20" s="121"/>
+      <c r="J20" s="55"/>
+      <c r="K20" s="55" t="s">
         <v>40</v>
       </c>
-      <c r="L20" s="30">
+      <c r="L20" s="62">
         <v>30</v>
       </c>
-      <c r="M20" t="s">
+      <c r="M20" s="55" t="s">
         <v>42</v>
       </c>
-      <c r="O20" s="47"/>
+      <c r="N20" s="55"/>
+      <c r="O20" s="57"/>
     </row>
     <row r="21" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B21" s="81">
+      <c r="B21" s="79">
         <v>90</v>
       </c>
-      <c r="C21" s="83">
+      <c r="C21" s="139">
         <v>112</v>
       </c>
-      <c r="D21" s="84" t="s">
+      <c r="D21" s="140" t="s">
+        <v>61</v>
+      </c>
+      <c r="E21" s="140"/>
+      <c r="F21" s="80"/>
+      <c r="H21" s="46" t="s">
         <v>62</v>
-      </c>
-      <c r="E21" s="84"/>
-      <c r="F21" s="82"/>
-      <c r="H21" s="46" t="s">
-        <v>63</v>
       </c>
       <c r="I21" s="17"/>
       <c r="K21" t="s">
@@ -2318,20 +2397,20 @@
       <c r="O21" s="47"/>
     </row>
     <row r="22" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B22" s="72">
+      <c r="B22" s="70">
         <v>100</v>
       </c>
       <c r="C22" s="31">
         <f>(24*32/4)</f>
         <v>192</v>
       </c>
-      <c r="D22" s="79" t="s">
+      <c r="D22" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="E22" s="79"/>
-      <c r="F22" s="80"/>
+      <c r="E22" s="77"/>
+      <c r="F22" s="78"/>
       <c r="H22" s="46" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="I22" s="17"/>
       <c r="K22" t="s">
@@ -2346,18 +2425,18 @@
       <c r="O22" s="47"/>
     </row>
     <row r="23" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B23" s="65" t="str">
-        <f t="shared" ref="B23:B48" si="17">DEC2HEX(HEX2DEC(B22)+C22)</f>
+      <c r="B23" s="46" t="str">
+        <f t="shared" ref="B23:B47" si="17">DEC2HEX(HEX2DEC(B22)+C22)</f>
         <v>1C0</v>
       </c>
-      <c r="C23" s="33">
-        <v>64</v>
-      </c>
-      <c r="D23" s="66" t="s">
-        <v>31</v>
-      </c>
-      <c r="E23" s="67"/>
-      <c r="F23" s="68"/>
+      <c r="C23" s="132">
+        <v>24</v>
+      </c>
+      <c r="D23" s="133" t="s">
+        <v>114</v>
+      </c>
+      <c r="E23" s="133"/>
+      <c r="F23" s="47"/>
       <c r="H23" s="46" t="s">
         <v>32</v>
       </c>
@@ -2374,18 +2453,18 @@
       <c r="O23" s="47"/>
     </row>
     <row r="24" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B24" s="73" t="str">
+      <c r="B24" s="63" t="str">
         <f t="shared" si="17"/>
-        <v>200</v>
-      </c>
-      <c r="C24" s="74">
-        <v>256</v>
-      </c>
-      <c r="D24" s="75" t="s">
-        <v>9</v>
-      </c>
-      <c r="E24" s="75"/>
-      <c r="F24" s="76"/>
+        <v>1D8</v>
+      </c>
+      <c r="C24" s="33">
+        <v>40</v>
+      </c>
+      <c r="D24" s="64" t="s">
+        <v>31</v>
+      </c>
+      <c r="E24" s="65"/>
+      <c r="F24" s="66"/>
       <c r="H24" s="46" t="s">
         <v>45</v>
       </c>
@@ -2401,1172 +2480,1148 @@
       </c>
       <c r="O24" s="47"/>
     </row>
-    <row r="25" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B25" s="46" t="str">
+    <row r="25" spans="2:16" x14ac:dyDescent="0.35">
+      <c r="B25" s="71" t="str">
+        <f t="shared" si="17"/>
+        <v>200</v>
+      </c>
+      <c r="C25" s="72">
+        <v>256</v>
+      </c>
+      <c r="D25" s="73" t="s">
+        <v>9</v>
+      </c>
+      <c r="E25" s="73"/>
+      <c r="F25" s="74"/>
+      <c r="H25" s="46" t="s">
+        <v>92</v>
+      </c>
+      <c r="I25" s="17"/>
+      <c r="K25" s="17" t="s">
+        <v>93</v>
+      </c>
+      <c r="L25" s="30">
+        <v>9</v>
+      </c>
+      <c r="M25" t="s">
+        <v>49</v>
+      </c>
+      <c r="O25" s="47"/>
+    </row>
+    <row r="26" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B26" s="46" t="str">
         <f t="shared" si="17"/>
         <v>300</v>
       </c>
-      <c r="C25" s="30">
+      <c r="C26" s="132">
         <v>192</v>
       </c>
-      <c r="D25" t="s">
+      <c r="D26" s="133" t="s">
         <v>24</v>
       </c>
-      <c r="F25" s="47"/>
-      <c r="H25" s="48" t="s">
-        <v>93</v>
-      </c>
-      <c r="I25" s="49"/>
-      <c r="J25" s="50"/>
-      <c r="K25" s="49" t="s">
-        <v>94</v>
-      </c>
-      <c r="L25" s="16">
-        <v>9</v>
-      </c>
-      <c r="M25" s="50" t="s">
+      <c r="E26" s="133"/>
+      <c r="F26" s="47"/>
+      <c r="H26" s="48" t="s">
+        <v>110</v>
+      </c>
+      <c r="I26" s="49"/>
+      <c r="J26" s="50"/>
+      <c r="K26" s="49" t="s">
+        <v>113</v>
+      </c>
+      <c r="L26" s="16">
+        <v>8</v>
+      </c>
+      <c r="M26" s="50" t="s">
         <v>49</v>
       </c>
-      <c r="N25" s="50"/>
-      <c r="O25" s="51"/>
-    </row>
-    <row r="26" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B26" s="46" t="str">
+      <c r="N26" s="50"/>
+      <c r="O26" s="51"/>
+    </row>
+    <row r="27" spans="2:16" x14ac:dyDescent="0.35">
+      <c r="B27" s="46" t="str">
         <f t="shared" si="17"/>
         <v>3C0</v>
       </c>
-      <c r="C26" s="30">
+      <c r="C27" s="132">
         <f>$D$7</f>
         <v>32</v>
       </c>
-      <c r="D26" s="85" t="s">
+      <c r="D27" s="141" t="s">
         <v>25</v>
       </c>
-      <c r="F26" s="47"/>
-      <c r="H26" s="17"/>
-      <c r="I26" s="17"/>
-      <c r="K26" s="30"/>
-    </row>
-    <row r="27" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B27" s="65" t="str">
+      <c r="E27" s="133"/>
+      <c r="F27" s="47"/>
+      <c r="H27" s="17"/>
+    </row>
+    <row r="28" spans="2:16" x14ac:dyDescent="0.35">
+      <c r="B28" s="63" t="str">
         <f t="shared" si="17"/>
         <v>3E0</v>
       </c>
-      <c r="C27" s="33">
+      <c r="C28" s="33">
         <v>32</v>
       </c>
-      <c r="D27" s="67" t="s">
-        <v>58</v>
-      </c>
-      <c r="E27" s="67"/>
-      <c r="F27" s="68"/>
-      <c r="H27" s="17"/>
-    </row>
-    <row r="28" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B28" s="46" t="str">
-        <f t="shared" si="17"/>
-        <v>400</v>
-      </c>
-      <c r="C28" s="30">
-        <v>432</v>
-      </c>
-      <c r="D28" t="s">
-        <v>83</v>
-      </c>
-      <c r="F28" s="47"/>
+      <c r="D28" s="65" t="s">
+        <v>57</v>
+      </c>
+      <c r="E28" s="65"/>
+      <c r="F28" s="66"/>
       <c r="H28" s="17"/>
       <c r="I28" s="54"/>
     </row>
     <row r="29" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B29" s="46" t="str">
         <f t="shared" si="17"/>
-        <v>5B0</v>
-      </c>
-      <c r="C29" s="30">
-        <v>384</v>
-      </c>
-      <c r="D29" t="s">
-        <v>18</v>
-      </c>
+        <v>400</v>
+      </c>
+      <c r="C29" s="132">
+        <v>432</v>
+      </c>
+      <c r="D29" s="133" t="s">
+        <v>82</v>
+      </c>
+      <c r="E29" s="133"/>
       <c r="F29" s="47"/>
     </row>
     <row r="30" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B30" s="46" t="str">
         <f t="shared" si="17"/>
+        <v>5B0</v>
+      </c>
+      <c r="C30" s="132">
+        <v>384</v>
+      </c>
+      <c r="D30" s="133" t="s">
+        <v>18</v>
+      </c>
+      <c r="E30" s="133"/>
+      <c r="F30" s="47"/>
+    </row>
+    <row r="31" spans="2:16" x14ac:dyDescent="0.35">
+      <c r="B31" s="46" t="str">
+        <f t="shared" si="17"/>
         <v>730</v>
       </c>
-      <c r="C30" s="30">
+      <c r="C31" s="132">
         <v>192</v>
       </c>
-      <c r="D30" t="s">
-        <v>84</v>
-      </c>
-      <c r="F30" s="47"/>
-    </row>
-    <row r="31" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B31" s="65" t="str">
+      <c r="D31" s="133" t="s">
+        <v>83</v>
+      </c>
+      <c r="E31" s="133"/>
+      <c r="F31" s="47"/>
+    </row>
+    <row r="32" spans="2:16" x14ac:dyDescent="0.35">
+      <c r="B32" s="63" t="str">
         <f t="shared" si="17"/>
         <v>7F0</v>
       </c>
-      <c r="C31" s="33">
+      <c r="C32" s="33">
         <v>16</v>
       </c>
-      <c r="D31" s="66" t="s">
-        <v>60</v>
-      </c>
-      <c r="E31" s="67"/>
-      <c r="F31" s="68"/>
-    </row>
-    <row r="32" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B32" s="77" t="str">
+      <c r="D32" s="64" t="s">
+        <v>59</v>
+      </c>
+      <c r="E32" s="65"/>
+      <c r="F32" s="66"/>
+    </row>
+    <row r="33" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B33" s="75" t="str">
         <f t="shared" si="17"/>
         <v>800</v>
       </c>
-      <c r="C32" s="86">
+      <c r="C33" s="142">
         <v>128</v>
       </c>
-      <c r="D32" s="87" t="s">
+      <c r="D33" s="143" t="s">
         <v>27</v>
       </c>
-      <c r="E32" s="87"/>
-      <c r="F32" s="78"/>
-    </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B33" s="46" t="str">
+      <c r="E33" s="143"/>
+      <c r="F33" s="76"/>
+    </row>
+    <row r="34" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B34" s="46" t="str">
         <f t="shared" si="17"/>
         <v>880</v>
       </c>
-      <c r="C33" s="30">
+      <c r="C34" s="132">
         <v>64</v>
       </c>
-      <c r="D33" s="85" t="s">
-        <v>67</v>
-      </c>
-      <c r="F33" s="47"/>
-    </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B34" s="73" t="str">
+      <c r="D34" s="141" t="s">
+        <v>66</v>
+      </c>
+      <c r="E34" s="133"/>
+      <c r="F34" s="47"/>
+    </row>
+    <row r="35" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B35" s="71" t="str">
         <f t="shared" si="17"/>
         <v>8C0</v>
       </c>
-      <c r="C34" s="74">
+      <c r="C35" s="72">
         <f>2*$D$7</f>
         <v>64</v>
       </c>
-      <c r="D34" s="75" t="s">
+      <c r="D35" s="73" t="s">
         <v>27</v>
       </c>
-      <c r="E34" s="75"/>
-      <c r="F34" s="76"/>
-    </row>
-    <row r="35" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B35" s="46" t="str">
+      <c r="E35" s="73"/>
+      <c r="F35" s="74"/>
+    </row>
+    <row r="36" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B36" s="46" t="str">
         <f t="shared" si="17"/>
         <v>900</v>
       </c>
-      <c r="C35" s="30">
+      <c r="C36" s="132">
         <v>960</v>
       </c>
-      <c r="D35" t="s">
+      <c r="D36" s="133" t="s">
         <v>17</v>
       </c>
-      <c r="F35" s="47"/>
-    </row>
-    <row r="36" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B36" s="65" t="str">
+      <c r="E36" s="133"/>
+      <c r="F36" s="47"/>
+    </row>
+    <row r="37" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B37" s="63" t="str">
         <f t="shared" si="17"/>
         <v>CC0</v>
       </c>
-      <c r="C36" s="33">
+      <c r="C37" s="33">
         <v>64</v>
       </c>
-      <c r="D36" s="67" t="s">
+      <c r="D37" s="65" t="s">
         <v>26</v>
       </c>
-      <c r="E36" s="67"/>
-      <c r="F36" s="68"/>
-    </row>
-    <row r="37" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B37" s="46" t="str">
+      <c r="E37" s="65"/>
+      <c r="F37" s="66"/>
+    </row>
+    <row r="38" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B38" s="46" t="str">
         <f t="shared" si="17"/>
         <v>D00</v>
       </c>
-      <c r="C37" s="30">
+      <c r="C38" s="132">
         <v>32</v>
       </c>
-      <c r="D37" s="85" t="s">
-        <v>57</v>
-      </c>
-      <c r="F37" s="47"/>
-    </row>
-    <row r="38" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B38" s="46" t="str">
-        <f>DEC2HEX(HEX2DEC(B37)+C37)</f>
+      <c r="D38" s="141" t="s">
+        <v>56</v>
+      </c>
+      <c r="E38" s="133"/>
+      <c r="F38" s="47"/>
+    </row>
+    <row r="39" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B39" s="46" t="str">
+        <f>DEC2HEX(HEX2DEC(B38)+C38)</f>
         <v>D20</v>
       </c>
-      <c r="C38" s="30">
+      <c r="C39" s="132">
         <v>64</v>
       </c>
-      <c r="D38" s="85" t="s">
-        <v>68</v>
-      </c>
-      <c r="F38" s="47"/>
-    </row>
-    <row r="39" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B39" s="73" t="str">
+      <c r="D39" s="141" t="s">
+        <v>67</v>
+      </c>
+      <c r="E39" s="133"/>
+      <c r="F39" s="47"/>
+    </row>
+    <row r="40" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B40" s="71" t="str">
         <f t="shared" si="17"/>
         <v>D60</v>
       </c>
-      <c r="C39" s="74">
+      <c r="C40" s="72">
         <v>160</v>
       </c>
-      <c r="D39" s="75" t="s">
+      <c r="D40" s="73" t="s">
         <v>51</v>
       </c>
-      <c r="E39" s="75"/>
-      <c r="F39" s="76"/>
-    </row>
-    <row r="40" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B40" s="46" t="str">
-        <f t="shared" si="17"/>
-        <v>E00</v>
-      </c>
-      <c r="C40" s="30">
-        <v>384</v>
-      </c>
-      <c r="D40" s="85" t="s">
-        <v>18</v>
-      </c>
-      <c r="F40" s="47"/>
+      <c r="E40" s="73"/>
+      <c r="F40" s="74"/>
     </row>
     <row r="41" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B41" s="46" t="str">
         <f t="shared" si="17"/>
+        <v>E00</v>
+      </c>
+      <c r="C41" s="132">
+        <v>384</v>
+      </c>
+      <c r="D41" s="141" t="s">
+        <v>18</v>
+      </c>
+      <c r="E41" s="133"/>
+      <c r="F41" s="47"/>
+    </row>
+    <row r="42" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B42" s="46" t="str">
+        <f t="shared" si="17"/>
         <v>F80</v>
       </c>
-      <c r="C41" s="30">
+      <c r="C42" s="132">
         <v>32</v>
       </c>
-      <c r="D41" s="85" t="s">
+      <c r="D42" s="141" t="s">
         <v>25</v>
       </c>
-      <c r="F41" s="47"/>
-    </row>
-    <row r="42" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B42" s="65" t="str">
+      <c r="E42" s="133"/>
+      <c r="F42" s="47"/>
+    </row>
+    <row r="43" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B43" s="46" t="str">
         <f t="shared" si="17"/>
         <v>FA0</v>
       </c>
-      <c r="C42" s="33">
+      <c r="C43" s="132">
         <v>96</v>
       </c>
-      <c r="D42" s="66" t="s">
+      <c r="D43" s="141" t="s">
         <v>52</v>
       </c>
-      <c r="E42" s="67"/>
-      <c r="F42" s="68"/>
-    </row>
-    <row r="43" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B43" s="77" t="str">
+      <c r="E43" s="133"/>
+      <c r="F43" s="47"/>
+    </row>
+    <row r="44" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B44" s="75" t="str">
         <f t="shared" si="17"/>
         <v>1000</v>
       </c>
-      <c r="C43" s="86">
+      <c r="C44" s="142">
         <v>144</v>
       </c>
-      <c r="D43" s="88" t="s">
+      <c r="D44" s="144" t="s">
         <v>21</v>
       </c>
-      <c r="E43" s="87"/>
-      <c r="F43" s="78"/>
-    </row>
-    <row r="44" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B44" s="46" t="str">
-        <f t="shared" si="17"/>
-        <v>1090</v>
-      </c>
-      <c r="C44" s="30">
-        <v>48</v>
-      </c>
-      <c r="D44" s="85" t="s">
-        <v>53</v>
-      </c>
-      <c r="F44" s="47"/>
+      <c r="E44" s="143"/>
+      <c r="F44" s="76"/>
     </row>
     <row r="45" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B45" s="46" t="str">
         <f t="shared" si="17"/>
-        <v>10C0</v>
-      </c>
-      <c r="C45" s="30">
-        <v>32</v>
-      </c>
-      <c r="D45" s="85" t="s">
-        <v>21</v>
-      </c>
+        <v>1090</v>
+      </c>
+      <c r="C45" s="132">
+        <v>48</v>
+      </c>
+      <c r="D45" s="141" t="s">
+        <v>53</v>
+      </c>
+      <c r="E45" s="133"/>
       <c r="F45" s="47"/>
     </row>
     <row r="46" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B46" s="46" t="str">
         <f t="shared" si="17"/>
+        <v>10C0</v>
+      </c>
+      <c r="C46" s="132">
+        <v>32</v>
+      </c>
+      <c r="D46" s="141" t="s">
+        <v>21</v>
+      </c>
+      <c r="E46" s="133"/>
+      <c r="F46" s="47"/>
+    </row>
+    <row r="47" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B47" s="46" t="str">
+        <f t="shared" si="17"/>
         <v>10E0</v>
       </c>
-      <c r="C46" s="30">
+      <c r="C47" s="132">
         <v>12</v>
       </c>
-      <c r="D46" s="85" t="s">
-        <v>56</v>
-      </c>
-      <c r="F46" s="47"/>
-    </row>
-    <row r="47" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B47" s="65" t="str">
-        <f t="shared" si="17"/>
-        <v>10EC</v>
-      </c>
-      <c r="C47" s="33">
-        <v>20</v>
-      </c>
-      <c r="D47" s="66" t="s">
-        <v>59</v>
-      </c>
-      <c r="E47" s="67"/>
-      <c r="F47" s="68"/>
+      <c r="D47" s="141" t="s">
+        <v>55</v>
+      </c>
+      <c r="E47" s="133"/>
+      <c r="F47" s="47"/>
     </row>
     <row r="48" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B48" s="89" t="str">
-        <f t="shared" si="17"/>
+      <c r="B48" s="46" t="str">
+        <f>DEC2HEX(HEX2DEC(B46)+C46)</f>
+        <v>10E0</v>
+      </c>
+      <c r="C48" s="132">
+        <v>9</v>
+      </c>
+      <c r="D48" s="141" t="s">
+        <v>58</v>
+      </c>
+      <c r="E48" s="133"/>
+      <c r="F48" s="47"/>
+    </row>
+    <row r="49" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B49" s="46" t="s">
+        <v>112</v>
+      </c>
+      <c r="C49" s="132">
+        <v>8</v>
+      </c>
+      <c r="D49" s="141" t="s">
+        <v>111</v>
+      </c>
+      <c r="E49" s="133"/>
+      <c r="F49" s="47"/>
+    </row>
+    <row r="50" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B50" s="81">
         <v>1100</v>
       </c>
-      <c r="C48" s="69">
-        <f>HEX2DEC(B49)-HEX2DEC(B48)</f>
-        <v>7072</v>
-      </c>
-      <c r="D48" s="70" t="s">
+      <c r="C50" s="67">
+        <f>HEX2DEC(B51)-HEX2DEC(B50)</f>
+        <v>7096</v>
+      </c>
+      <c r="D50" s="68" t="s">
         <v>10</v>
       </c>
-      <c r="E48" s="70"/>
-      <c r="F48" s="71"/>
-    </row>
-    <row r="49" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B49" s="72" t="str">
-        <f t="shared" ref="B49:B51" si="18">DEC2HEX(HEX2DEC(B50)-C49)</f>
-        <v>2CA0</v>
-      </c>
-      <c r="C49" s="31">
+      <c r="E50" s="68"/>
+      <c r="F50" s="69"/>
+    </row>
+    <row r="51" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B51" s="157" t="str">
+        <f t="shared" ref="B51:B53" si="18">DEC2HEX(HEX2DEC(B52)-C51)</f>
+        <v>2CB8</v>
+      </c>
+      <c r="C51" s="31">
         <v>768</v>
       </c>
-      <c r="D49" s="79" t="s">
-        <v>86</v>
-      </c>
-      <c r="E49" s="79"/>
-      <c r="F49" s="80"/>
-    </row>
-    <row r="50" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B50" s="46" t="str">
+      <c r="D51" s="77" t="s">
+        <v>85</v>
+      </c>
+      <c r="E51" s="77"/>
+      <c r="F51" s="78"/>
+    </row>
+    <row r="52" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B52" s="158" t="str">
         <f t="shared" si="18"/>
-        <v>2FA0</v>
-      </c>
-      <c r="C50" s="30">
-        <v>96</v>
-      </c>
-      <c r="D50" t="s">
-        <v>55</v>
-      </c>
-      <c r="F50" s="47"/>
-    </row>
-    <row r="51" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B51" s="46" t="str">
+        <v>2FB8</v>
+      </c>
+      <c r="C52" s="132">
+        <f>24*3</f>
+        <v>72</v>
+      </c>
+      <c r="D52" s="133" t="s">
+        <v>115</v>
+      </c>
+      <c r="E52" s="133"/>
+      <c r="F52" s="47"/>
+    </row>
+    <row r="53" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B53" s="46" t="str">
         <f t="shared" si="18"/>
         <v>3000</v>
       </c>
-      <c r="C51" s="30">
+      <c r="C53" s="132">
         <v>96</v>
       </c>
-      <c r="D51" t="s">
-        <v>66</v>
-      </c>
-      <c r="F51" s="47"/>
-    </row>
-    <row r="52" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B52" s="46" t="str">
-        <f>DEC2HEX(HEX2DEC(B53)-C52)</f>
+      <c r="D53" s="133" t="s">
+        <v>65</v>
+      </c>
+      <c r="E53" s="133"/>
+      <c r="F53" s="47"/>
+    </row>
+    <row r="54" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B54" s="46" t="str">
+        <f>DEC2HEX(HEX2DEC(B55)-C54)</f>
         <v>3060</v>
       </c>
-      <c r="C52" s="30">
+      <c r="C54" s="132">
         <f>$D$11</f>
         <v>224</v>
       </c>
-      <c r="D52" t="s">
+      <c r="D54" s="133" t="s">
         <v>28</v>
       </c>
-      <c r="F52" s="47"/>
-    </row>
-    <row r="53" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B53" s="111" t="str">
-        <f>DEC2HEX(HEX2DEC(B54)-C53)</f>
+      <c r="E54" s="133"/>
+      <c r="F54" s="47"/>
+    </row>
+    <row r="55" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B55" s="70" t="str">
+        <f>DEC2HEX(HEX2DEC(B56)-C55)</f>
         <v>3140</v>
       </c>
-      <c r="C53" s="112">
+      <c r="C55" s="31">
         <v>1728</v>
       </c>
-      <c r="D53" s="113" t="s">
-        <v>92</v>
-      </c>
-      <c r="E53" s="114"/>
-      <c r="F53" s="115"/>
-    </row>
-    <row r="54" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B54" s="116" t="str">
-        <f>DEC2HEX(HEX2DEC(B55)-C54)</f>
+      <c r="D55" s="113" t="s">
+        <v>91</v>
+      </c>
+      <c r="E55" s="77"/>
+      <c r="F55" s="78"/>
+    </row>
+    <row r="56" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B56" s="46" t="str">
+        <f>DEC2HEX(HEX2DEC(B57)-C56)</f>
         <v>3800</v>
       </c>
-      <c r="C54" s="117">
+      <c r="C56" s="132">
         <f>2048</f>
         <v>2048</v>
       </c>
-      <c r="D54" s="118" t="s">
+      <c r="D56" s="134" t="s">
         <v>30</v>
       </c>
-      <c r="E54" s="105"/>
-      <c r="F54" s="106"/>
-    </row>
-    <row r="55" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B55" s="119">
+      <c r="E56" s="133"/>
+      <c r="F56" s="47"/>
+    </row>
+    <row r="57" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B57" s="114">
         <v>4000</v>
       </c>
-      <c r="C55" s="120" t="s">
-        <v>85</v>
-      </c>
-      <c r="D55" s="121" t="s">
+      <c r="C57" s="115" t="s">
+        <v>84</v>
+      </c>
+      <c r="D57" s="116" t="s">
         <v>19</v>
       </c>
-      <c r="E55" s="122"/>
-      <c r="F55" s="123"/>
-    </row>
-    <row r="56" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B56" s="17"/>
-      <c r="C56" s="17"/>
-      <c r="D56" s="17"/>
-    </row>
-    <row r="57" spans="2:10" ht="19" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B57" s="126" t="s">
-        <v>108</v>
-      </c>
-      <c r="C57" s="17"/>
-      <c r="D57" s="17"/>
-    </row>
-    <row r="58" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B58" s="94" t="s">
+      <c r="E57" s="117"/>
+      <c r="F57" s="118"/>
+    </row>
+    <row r="58" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B58" s="46"/>
+      <c r="C58" s="134"/>
+      <c r="D58" s="134"/>
+      <c r="E58" s="133"/>
+      <c r="F58" s="47"/>
+    </row>
+    <row r="59" spans="2:6" ht="19" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B59" s="145" t="s">
+        <v>107</v>
+      </c>
+      <c r="C59" s="134"/>
+      <c r="D59" s="134"/>
+      <c r="E59" s="133"/>
+      <c r="F59" s="47"/>
+    </row>
+    <row r="60" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B60" s="86" t="s">
         <v>7</v>
       </c>
-      <c r="C58" s="60" t="s">
+      <c r="C60" s="58" t="s">
         <v>20</v>
       </c>
-      <c r="D58" s="95" t="s">
+      <c r="D60" s="87" t="s">
         <v>8</v>
       </c>
-      <c r="E58" s="52"/>
-      <c r="F58" s="53"/>
-    </row>
-    <row r="59" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B59" s="110">
+      <c r="E60" s="52"/>
+      <c r="F60" s="53"/>
+    </row>
+    <row r="61" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B61" s="112" t="s">
+        <v>109</v>
+      </c>
+      <c r="C61" s="146"/>
+      <c r="D61" s="147"/>
+      <c r="E61" s="133"/>
+      <c r="F61" s="47"/>
+    </row>
+    <row r="62" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B62" s="101" t="str">
+        <f>DEC2HEX(HEX2DEC(B63)-C62)</f>
+        <v>3140</v>
+      </c>
+      <c r="C62" s="102">
+        <v>1728</v>
+      </c>
+      <c r="D62" s="103" t="s">
+        <v>91</v>
+      </c>
+      <c r="E62" s="104"/>
+      <c r="F62" s="105"/>
+    </row>
+    <row r="63" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B63" s="106" t="str">
+        <f>DEC2HEX(HEX2DEC(B64)-C63)</f>
+        <v>3800</v>
+      </c>
+      <c r="C63" s="148">
+        <f>2048</f>
+        <v>2048</v>
+      </c>
+      <c r="D63" s="149" t="s">
+        <v>30</v>
+      </c>
+      <c r="E63" s="150"/>
+      <c r="F63" s="96"/>
+    </row>
+    <row r="64" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B64" s="100">
         <v>4000</v>
       </c>
-      <c r="C59" s="103">
-        <f>HEX2DEC(B60)-HEX2DEC(B59)</f>
+      <c r="C64" s="151">
+        <f>HEX2DEC(B65)-HEX2DEC(B64)</f>
         <v>2</v>
       </c>
-      <c r="D59" s="104" t="s">
+      <c r="D64" s="152" t="s">
+        <v>68</v>
+      </c>
+      <c r="E64" s="150"/>
+      <c r="F64" s="96"/>
+    </row>
+    <row r="65" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B65" s="100">
+        <v>4002</v>
+      </c>
+      <c r="C65" s="151">
+        <f>HEX2DEC(B66)-HEX2DEC(B65)</f>
+        <v>28</v>
+      </c>
+      <c r="D65" s="152" t="s">
         <v>69</v>
       </c>
-      <c r="E59" s="105"/>
-      <c r="F59" s="106"/>
-      <c r="J59">
-        <v>40000</v>
-      </c>
-    </row>
-    <row r="60" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B60" s="110">
-        <v>4002</v>
-      </c>
-      <c r="C60" s="103">
-        <f>HEX2DEC(B61)-HEX2DEC(B60)</f>
-        <v>28</v>
-      </c>
-      <c r="D60" s="104" t="s">
-        <v>70</v>
-      </c>
-      <c r="E60" s="105"/>
-      <c r="F60" s="106"/>
-      <c r="J60">
-        <v>59344</v>
-      </c>
-    </row>
-    <row r="61" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B61" s="102" t="s">
-        <v>91</v>
-      </c>
-      <c r="C61" s="103">
-        <f t="shared" ref="C61:C65" si="19">HEX2DEC(B62)-HEX2DEC(B61)</f>
+      <c r="E65" s="150"/>
+      <c r="F65" s="96"/>
+    </row>
+    <row r="66" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B66" s="92" t="s">
+        <v>90</v>
+      </c>
+      <c r="C66" s="151">
+        <f t="shared" ref="C66:C70" si="19">HEX2DEC(B67)-HEX2DEC(B66)</f>
         <v>16</v>
       </c>
-      <c r="D61" s="104" t="s">
+      <c r="D66" s="152" t="s">
         <v>29</v>
       </c>
-      <c r="E61" s="105"/>
-      <c r="F61" s="106"/>
-    </row>
-    <row r="62" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B62" s="102" t="s">
-        <v>88</v>
-      </c>
-      <c r="C62" s="103">
+      <c r="E66" s="150"/>
+      <c r="F66" s="96"/>
+    </row>
+    <row r="67" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B67" s="92" t="s">
+        <v>87</v>
+      </c>
+      <c r="C67" s="151">
         <f t="shared" si="19"/>
         <v>5</v>
       </c>
-      <c r="D62" s="104" t="s">
-        <v>71</v>
-      </c>
-      <c r="E62" s="105"/>
-      <c r="F62" s="106"/>
-    </row>
-    <row r="63" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B63" s="102">
+      <c r="D67" s="152" t="s">
+        <v>70</v>
+      </c>
+      <c r="E67" s="150"/>
+      <c r="F67" s="96"/>
+    </row>
+    <row r="68" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B68" s="92">
         <v>4033</v>
       </c>
-      <c r="C63" s="103">
+      <c r="C68" s="151">
         <f t="shared" si="19"/>
         <v>192</v>
       </c>
-      <c r="D63" s="104" t="s">
-        <v>72</v>
-      </c>
-      <c r="E63" s="105"/>
-      <c r="F63" s="106"/>
-    </row>
-    <row r="64" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B64" s="102" t="s">
-        <v>89</v>
-      </c>
-      <c r="C64" s="103">
+      <c r="D68" s="152" t="s">
+        <v>71</v>
+      </c>
+      <c r="E68" s="150"/>
+      <c r="F68" s="96"/>
+      <c r="G68" s="135"/>
+    </row>
+    <row r="69" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B69" s="92" t="s">
+        <v>88</v>
+      </c>
+      <c r="C69" s="151">
         <f t="shared" si="19"/>
         <v>48</v>
       </c>
-      <c r="D64" s="104" t="s">
-        <v>73</v>
-      </c>
-      <c r="E64" s="105"/>
-      <c r="F64" s="106"/>
-      <c r="G64" s="97"/>
-    </row>
-    <row r="65" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B65" s="102">
+      <c r="D69" s="152" t="s">
+        <v>72</v>
+      </c>
+      <c r="E69" s="150"/>
+      <c r="F69" s="96"/>
+      <c r="G69" s="136"/>
+    </row>
+    <row r="70" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B70" s="92">
         <v>4123</v>
       </c>
-      <c r="C65" s="103">
+      <c r="C70" s="151">
         <f t="shared" si="19"/>
         <v>3712</v>
       </c>
-      <c r="D65" s="104" t="s">
-        <v>74</v>
-      </c>
-      <c r="E65" s="105"/>
-      <c r="F65" s="106"/>
-      <c r="G65" s="96"/>
-    </row>
-    <row r="66" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B66" s="102" t="s">
-        <v>90</v>
-      </c>
-      <c r="C66" s="103">
-        <f t="shared" ref="C66:C72" si="20">HEX2DEC(B67)-HEX2DEC(B66)</f>
+      <c r="D70" s="152" t="s">
+        <v>73</v>
+      </c>
+      <c r="E70" s="150"/>
+      <c r="F70" s="96"/>
+      <c r="G70" s="136"/>
+    </row>
+    <row r="71" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B71" s="92" t="s">
+        <v>89</v>
+      </c>
+      <c r="C71" s="151">
+        <f t="shared" ref="C71:C77" si="20">HEX2DEC(B72)-HEX2DEC(B71)</f>
         <v>2304</v>
       </c>
-      <c r="D66" s="104" t="s">
-        <v>96</v>
-      </c>
-      <c r="E66" s="105"/>
-      <c r="F66" s="106"/>
-      <c r="G66" s="96"/>
-    </row>
-    <row r="67" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B67" s="102" t="s">
+      <c r="D71" s="152" t="s">
         <v>95</v>
       </c>
-      <c r="C67" s="103">
+      <c r="E71" s="150"/>
+      <c r="F71" s="96"/>
+      <c r="G71" s="136"/>
+    </row>
+    <row r="72" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B72" s="92" t="s">
+        <v>94</v>
+      </c>
+      <c r="C72" s="151">
         <f t="shared" si="20"/>
         <v>1995</v>
       </c>
-      <c r="D67" s="104" t="s">
-        <v>75</v>
-      </c>
-      <c r="E67" s="105"/>
-      <c r="F67" s="106"/>
-      <c r="G67" s="96"/>
-    </row>
-    <row r="68" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B68" s="102" t="s">
-        <v>97</v>
-      </c>
-      <c r="C68" s="103">
+      <c r="D72" s="152" t="s">
+        <v>74</v>
+      </c>
+      <c r="E72" s="150"/>
+      <c r="F72" s="96"/>
+      <c r="G72" s="136"/>
+    </row>
+    <row r="73" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B73" s="92" t="s">
+        <v>96</v>
+      </c>
+      <c r="C73" s="151">
         <f t="shared" si="20"/>
         <v>84</v>
       </c>
-      <c r="D68" s="104" t="s">
-        <v>76</v>
-      </c>
-      <c r="E68" s="105"/>
-      <c r="F68" s="106"/>
-      <c r="G68" s="96"/>
-    </row>
-    <row r="69" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B69" s="107" t="s">
-        <v>98</v>
-      </c>
-      <c r="C69" s="103">
+      <c r="D73" s="152" t="s">
+        <v>75</v>
+      </c>
+      <c r="E73" s="150"/>
+      <c r="F73" s="96"/>
+      <c r="G73" s="137"/>
+    </row>
+    <row r="74" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B74" s="97" t="s">
+        <v>97</v>
+      </c>
+      <c r="C74" s="151">
         <f t="shared" si="20"/>
         <v>2634</v>
       </c>
-      <c r="D69" s="108" t="s">
-        <v>101</v>
-      </c>
-      <c r="E69" s="105"/>
-      <c r="F69" s="106"/>
-      <c r="G69" s="98"/>
-    </row>
-    <row r="70" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B70" s="109" t="s">
-        <v>99</v>
-      </c>
-      <c r="C70" s="103">
+      <c r="D74" s="153" t="s">
+        <v>100</v>
+      </c>
+      <c r="E74" s="150"/>
+      <c r="F74" s="96"/>
+      <c r="G74" s="138"/>
+    </row>
+    <row r="75" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B75" s="99" t="s">
+        <v>98</v>
+      </c>
+      <c r="C75" s="151">
         <f t="shared" si="20"/>
         <v>3203</v>
       </c>
-      <c r="D70" s="104" t="s">
-        <v>77</v>
-      </c>
-      <c r="E70" s="105"/>
-      <c r="F70" s="106"/>
-      <c r="G70" s="99"/>
-    </row>
-    <row r="71" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B71" s="99" t="s">
-        <v>100</v>
-      </c>
-      <c r="C71" s="90">
+      <c r="D75" s="152" t="s">
+        <v>76</v>
+      </c>
+      <c r="E75" s="150"/>
+      <c r="F75" s="96"/>
+      <c r="G75" s="138"/>
+    </row>
+    <row r="76" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B76" s="89" t="s">
+        <v>99</v>
+      </c>
+      <c r="C76" s="154">
         <f t="shared" si="20"/>
         <v>881</v>
       </c>
-      <c r="D71" s="101" t="s">
-        <v>82</v>
-      </c>
-      <c r="F71" s="47"/>
-      <c r="G71" s="99"/>
-    </row>
-    <row r="72" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B72" s="96" t="s">
-        <v>78</v>
-      </c>
-      <c r="C72" s="90">
+      <c r="D76" s="155" t="s">
+        <v>81</v>
+      </c>
+      <c r="E76" s="133"/>
+      <c r="F76" s="47"/>
+    </row>
+    <row r="77" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B77" s="88" t="s">
+        <v>77</v>
+      </c>
+      <c r="C77" s="154">
         <f t="shared" si="20"/>
         <v>256</v>
       </c>
-      <c r="D72" s="91" t="s">
+      <c r="D77" s="156" t="s">
+        <v>78</v>
+      </c>
+      <c r="E77" s="133"/>
+      <c r="F77" s="47"/>
+    </row>
+    <row r="78" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B78" s="90" t="s">
         <v>79</v>
       </c>
-      <c r="F72" s="47"/>
-    </row>
-    <row r="73" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B73" s="100" t="s">
+      <c r="C78" s="84">
+        <v>1024</v>
+      </c>
+      <c r="D78" s="85" t="s">
         <v>80</v>
       </c>
-      <c r="C73" s="92">
-        <v>1024</v>
-      </c>
-      <c r="D73" s="93" t="s">
-        <v>81</v>
-      </c>
-      <c r="E73" s="50"/>
-      <c r="F73" s="51"/>
-    </row>
-    <row r="74" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B74" s="45"/>
-      <c r="C74" s="90"/>
-    </row>
-    <row r="75" spans="2:7" ht="19" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B75" s="125" t="s">
-        <v>106</v>
-      </c>
-      <c r="C75" s="90"/>
-    </row>
-    <row r="76" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B76" s="94" t="s">
+      <c r="E78" s="50"/>
+      <c r="F78" s="51"/>
+    </row>
+    <row r="79" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B79" s="45"/>
+      <c r="C79" s="82"/>
+    </row>
+    <row r="80" spans="2:7" ht="19" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B80" s="110" t="s">
+        <v>105</v>
+      </c>
+      <c r="C80" s="82"/>
+    </row>
+    <row r="81" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B81" s="86" t="s">
         <v>7</v>
       </c>
-      <c r="C76" s="60" t="s">
+      <c r="C81" s="58" t="s">
         <v>20</v>
       </c>
-      <c r="D76" s="95" t="s">
+      <c r="D81" s="87" t="s">
         <v>8</v>
       </c>
-      <c r="E76" s="52"/>
-      <c r="F76" s="53"/>
-    </row>
-    <row r="77" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B77" s="111" t="str">
-        <f>DEC2HEX(HEX2DEC(B78)-C77)</f>
+      <c r="E81" s="52"/>
+      <c r="F81" s="53"/>
+    </row>
+    <row r="82" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B82" s="101" t="str">
+        <f>DEC2HEX(HEX2DEC(B83)-C82)</f>
         <v>3140</v>
       </c>
-      <c r="C77" s="112">
+      <c r="C82" s="102">
         <v>1728</v>
       </c>
-      <c r="D77" s="113" t="s">
-        <v>92</v>
-      </c>
-      <c r="E77" s="114"/>
-      <c r="F77" s="115"/>
-    </row>
-    <row r="78" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B78" s="116" t="str">
-        <f>DEC2HEX(HEX2DEC(B79)-C78)</f>
+      <c r="D82" s="103" t="s">
+        <v>91</v>
+      </c>
+      <c r="E82" s="104"/>
+      <c r="F82" s="105"/>
+    </row>
+    <row r="83" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B83" s="106" t="str">
+        <f>DEC2HEX(HEX2DEC(B84)-C83)</f>
         <v>3800</v>
       </c>
-      <c r="C78" s="117">
+      <c r="C83" s="107">
         <f>2048</f>
         <v>2048</v>
       </c>
-      <c r="D78" s="118" t="s">
+      <c r="D83" s="108" t="s">
         <v>30</v>
       </c>
-      <c r="E78" s="105"/>
-      <c r="F78" s="106"/>
-    </row>
-    <row r="79" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B79" s="110">
+      <c r="E83" s="95"/>
+      <c r="F83" s="96"/>
+    </row>
+    <row r="84" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B84" s="100">
         <v>4000</v>
       </c>
-      <c r="C79" s="103">
-        <f>HEX2DEC(B80)-HEX2DEC(B79)</f>
+      <c r="C84" s="93">
+        <f>HEX2DEC(B85)-HEX2DEC(B84)</f>
         <v>2</v>
       </c>
-      <c r="D79" s="104" t="s">
+      <c r="D84" s="94" t="s">
+        <v>68</v>
+      </c>
+      <c r="E84" s="95"/>
+      <c r="F84" s="96"/>
+    </row>
+    <row r="85" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B85" s="100">
+        <v>4002</v>
+      </c>
+      <c r="C85" s="93">
+        <f>HEX2DEC(B86)-HEX2DEC(B85)</f>
+        <v>28</v>
+      </c>
+      <c r="D85" s="94" t="s">
         <v>69</v>
       </c>
-      <c r="E79" s="105"/>
-      <c r="F79" s="106"/>
-    </row>
-    <row r="80" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B80" s="110">
-        <v>4002</v>
-      </c>
-      <c r="C80" s="103">
-        <f>HEX2DEC(B81)-HEX2DEC(B80)</f>
-        <v>28</v>
-      </c>
-      <c r="D80" s="104" t="s">
-        <v>70</v>
-      </c>
-      <c r="E80" s="105"/>
-      <c r="F80" s="106"/>
-    </row>
-    <row r="81" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B81" s="102" t="s">
-        <v>91</v>
-      </c>
-      <c r="C81" s="103">
-        <f t="shared" ref="C81:C91" si="21">HEX2DEC(B82)-HEX2DEC(B81)</f>
+      <c r="E85" s="95"/>
+      <c r="F85" s="96"/>
+    </row>
+    <row r="86" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B86" s="92" t="s">
+        <v>90</v>
+      </c>
+      <c r="C86" s="93">
+        <f t="shared" ref="C86:C96" si="21">HEX2DEC(B87)-HEX2DEC(B86)</f>
         <v>16</v>
       </c>
-      <c r="D81" s="104" t="s">
+      <c r="D86" s="94" t="s">
         <v>29</v>
       </c>
-      <c r="E81" s="105"/>
-      <c r="F81" s="106"/>
-    </row>
-    <row r="82" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B82" s="102" t="s">
-        <v>88</v>
-      </c>
-      <c r="C82" s="103">
+      <c r="E86" s="95"/>
+      <c r="F86" s="96"/>
+    </row>
+    <row r="87" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B87" s="92" t="s">
+        <v>87</v>
+      </c>
+      <c r="C87" s="93">
         <f t="shared" si="21"/>
         <v>5</v>
       </c>
-      <c r="D82" s="104" t="s">
-        <v>71</v>
-      </c>
-      <c r="E82" s="105"/>
-      <c r="F82" s="106"/>
-    </row>
-    <row r="83" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B83" s="102">
+      <c r="D87" s="94" t="s">
+        <v>70</v>
+      </c>
+      <c r="E87" s="95"/>
+      <c r="F87" s="96"/>
+    </row>
+    <row r="88" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B88" s="92">
         <v>4033</v>
       </c>
-      <c r="C83" s="103">
+      <c r="C88" s="93">
         <f t="shared" si="21"/>
         <v>192</v>
       </c>
-      <c r="D83" s="104" t="s">
-        <v>72</v>
-      </c>
-      <c r="E83" s="105"/>
-      <c r="F83" s="106"/>
-    </row>
-    <row r="84" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B84" s="102" t="s">
-        <v>89</v>
-      </c>
-      <c r="C84" s="103">
+      <c r="D88" s="94" t="s">
+        <v>71</v>
+      </c>
+      <c r="E88" s="95"/>
+      <c r="F88" s="96"/>
+    </row>
+    <row r="89" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B89" s="92" t="s">
+        <v>88</v>
+      </c>
+      <c r="C89" s="93">
         <f t="shared" si="21"/>
         <v>48</v>
       </c>
-      <c r="D84" s="104" t="s">
-        <v>73</v>
-      </c>
-      <c r="E84" s="105"/>
-      <c r="F84" s="106"/>
-    </row>
-    <row r="85" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B85" s="102">
+      <c r="D89" s="94" t="s">
+        <v>72</v>
+      </c>
+      <c r="E89" s="95"/>
+      <c r="F89" s="96"/>
+    </row>
+    <row r="90" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B90" s="92">
         <v>4123</v>
       </c>
-      <c r="C85" s="103">
+      <c r="C90" s="93">
         <f t="shared" si="21"/>
         <v>3712</v>
       </c>
-      <c r="D85" s="104" t="s">
-        <v>74</v>
-      </c>
-      <c r="E85" s="105"/>
-      <c r="F85" s="106"/>
-    </row>
-    <row r="86" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B86" s="102" t="s">
-        <v>90</v>
-      </c>
-      <c r="C86" s="103">
+      <c r="D90" s="94" t="s">
+        <v>73</v>
+      </c>
+      <c r="E90" s="95"/>
+      <c r="F90" s="96"/>
+    </row>
+    <row r="91" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B91" s="92" t="s">
+        <v>89</v>
+      </c>
+      <c r="C91" s="93">
         <f t="shared" si="21"/>
         <v>2304</v>
       </c>
-      <c r="D86" s="104" t="s">
-        <v>96</v>
-      </c>
-      <c r="E86" s="105"/>
-      <c r="F86" s="106"/>
-    </row>
-    <row r="87" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B87" s="102" t="s">
+      <c r="D91" s="94" t="s">
         <v>95</v>
       </c>
-      <c r="C87" s="103">
+      <c r="E91" s="95"/>
+      <c r="F91" s="96"/>
+    </row>
+    <row r="92" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B92" s="92" t="s">
+        <v>94</v>
+      </c>
+      <c r="C92" s="93">
         <f t="shared" si="21"/>
         <v>1995</v>
       </c>
-      <c r="D87" s="104" t="s">
-        <v>75</v>
-      </c>
-      <c r="E87" s="105"/>
-      <c r="F87" s="106"/>
-    </row>
-    <row r="88" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B88" s="102" t="s">
-        <v>97</v>
-      </c>
-      <c r="C88" s="103">
+      <c r="D92" s="94" t="s">
+        <v>74</v>
+      </c>
+      <c r="E92" s="95"/>
+      <c r="F92" s="96"/>
+    </row>
+    <row r="93" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B93" s="92" t="s">
+        <v>96</v>
+      </c>
+      <c r="C93" s="93">
         <f t="shared" si="21"/>
         <v>84</v>
       </c>
-      <c r="D88" s="104" t="s">
-        <v>76</v>
-      </c>
-      <c r="E88" s="105"/>
-      <c r="F88" s="106"/>
-    </row>
-    <row r="89" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B89" s="107" t="s">
-        <v>98</v>
-      </c>
-      <c r="C89" s="103">
+      <c r="D93" s="94" t="s">
+        <v>75</v>
+      </c>
+      <c r="E93" s="95"/>
+      <c r="F93" s="96"/>
+    </row>
+    <row r="94" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B94" s="97" t="s">
+        <v>97</v>
+      </c>
+      <c r="C94" s="93">
         <f t="shared" si="21"/>
         <v>2064</v>
       </c>
-      <c r="D89" s="108" t="s">
-        <v>104</v>
-      </c>
-      <c r="E89" s="105"/>
-      <c r="F89" s="106"/>
-    </row>
-    <row r="90" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B90" s="99" t="s">
+      <c r="D94" s="98" t="s">
         <v>103</v>
       </c>
-      <c r="C90" s="90">
+      <c r="E94" s="95"/>
+      <c r="F94" s="96"/>
+    </row>
+    <row r="95" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B95" s="89" t="s">
+        <v>102</v>
+      </c>
+      <c r="C95" s="82">
         <f t="shared" si="21"/>
         <v>4654</v>
       </c>
-      <c r="D90" s="101" t="s">
-        <v>82</v>
-      </c>
-      <c r="F90" s="47"/>
-    </row>
-    <row r="91" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B91" s="96" t="s">
-        <v>78</v>
-      </c>
-      <c r="C91" s="90">
+      <c r="D95" s="91" t="s">
+        <v>81</v>
+      </c>
+      <c r="F95" s="47"/>
+    </row>
+    <row r="96" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B96" s="88" t="s">
+        <v>77</v>
+      </c>
+      <c r="C96" s="82">
         <f t="shared" si="21"/>
         <v>256</v>
       </c>
-      <c r="D91" s="91" t="s">
+      <c r="D96" s="83" t="s">
+        <v>78</v>
+      </c>
+      <c r="F96" s="47"/>
+    </row>
+    <row r="97" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B97" s="90" t="s">
         <v>79</v>
       </c>
-      <c r="F91" s="47"/>
-    </row>
-    <row r="92" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B92" s="100" t="s">
+      <c r="C97" s="84">
+        <v>1024</v>
+      </c>
+      <c r="D97" s="85" t="s">
         <v>80</v>
       </c>
-      <c r="C92" s="92">
-        <v>1024</v>
-      </c>
-      <c r="D92" s="93" t="s">
-        <v>81</v>
-      </c>
-      <c r="E92" s="50"/>
-      <c r="F92" s="51"/>
-    </row>
-    <row r="93" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B93" s="45"/>
-    </row>
-    <row r="94" spans="2:6" ht="19" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B94" s="125" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="95" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B95" s="94" t="s">
+      <c r="E97" s="50"/>
+      <c r="F97" s="51"/>
+    </row>
+    <row r="98" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B98" s="45"/>
+    </row>
+    <row r="99" spans="2:6" ht="19" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B99" s="110" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="100" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B100" s="86" t="s">
         <v>7</v>
       </c>
-      <c r="C95" s="60" t="s">
+      <c r="C100" s="58" t="s">
         <v>20</v>
       </c>
-      <c r="D95" s="95" t="s">
+      <c r="D100" s="87" t="s">
         <v>8</v>
       </c>
-      <c r="E95" s="52"/>
-      <c r="F95" s="53"/>
-    </row>
-    <row r="96" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B96" s="96">
-        <v>4000</v>
-      </c>
-      <c r="C96" s="90">
-        <f>HEX2DEC(B97)-HEX2DEC(B96)</f>
-        <v>2</v>
-      </c>
-      <c r="D96" s="91" t="s">
-        <v>69</v>
-      </c>
-      <c r="F96" s="47"/>
-    </row>
-    <row r="97" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B97" s="96">
-        <v>4002</v>
-      </c>
-      <c r="C97" s="90">
-        <f>HEX2DEC(B98)-HEX2DEC(B97)</f>
-        <v>28</v>
-      </c>
-      <c r="D97" s="91" t="s">
-        <v>70</v>
-      </c>
-      <c r="F97" s="47"/>
-    </row>
-    <row r="98" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B98" s="97" t="s">
-        <v>91</v>
-      </c>
-      <c r="C98" s="90">
-        <f t="shared" ref="C98:C110" si="22">HEX2DEC(B99)-HEX2DEC(B98)</f>
-        <v>16</v>
-      </c>
-      <c r="D98" s="91" t="s">
-        <v>29</v>
-      </c>
-      <c r="F98" s="47"/>
-    </row>
-    <row r="99" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B99" s="97" t="s">
-        <v>88</v>
-      </c>
-      <c r="C99" s="90">
+      <c r="E100" s="52"/>
+      <c r="F100" s="53"/>
+    </row>
+    <row r="101" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B101" s="92" t="s">
+        <v>96</v>
+      </c>
+      <c r="C101" s="93">
+        <f t="shared" ref="C101:C106" si="22">HEX2DEC(B102)-HEX2DEC(B101)</f>
+        <v>84</v>
+      </c>
+      <c r="D101" s="94" t="s">
+        <v>75</v>
+      </c>
+      <c r="E101" s="95"/>
+      <c r="F101" s="96"/>
+    </row>
+    <row r="102" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B102" s="97" t="s">
+        <v>97</v>
+      </c>
+      <c r="C102" s="93">
         <f t="shared" si="22"/>
-        <v>5</v>
-      </c>
-      <c r="D99" s="91" t="s">
-        <v>71</v>
-      </c>
-      <c r="F99" s="47"/>
-    </row>
-    <row r="100" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B100" s="97">
-        <v>4033</v>
-      </c>
-      <c r="C100" s="90">
-        <f t="shared" si="22"/>
-        <v>192</v>
-      </c>
-      <c r="D100" s="91" t="s">
-        <v>72</v>
-      </c>
-      <c r="F100" s="47"/>
-    </row>
-    <row r="101" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B101" s="97" t="s">
-        <v>89</v>
-      </c>
-      <c r="C101" s="90">
-        <f t="shared" si="22"/>
-        <v>48</v>
-      </c>
-      <c r="D101" s="91" t="s">
-        <v>73</v>
-      </c>
-      <c r="F101" s="47"/>
-    </row>
-    <row r="102" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B102" s="97">
-        <v>4123</v>
-      </c>
-      <c r="C102" s="90">
-        <f t="shared" si="22"/>
-        <v>3712</v>
-      </c>
-      <c r="D102" s="91" t="s">
-        <v>74</v>
-      </c>
-      <c r="F102" s="47"/>
+        <v>2047</v>
+      </c>
+      <c r="D102" s="98" t="s">
+        <v>104</v>
+      </c>
+      <c r="E102" s="95"/>
+      <c r="F102" s="96"/>
     </row>
     <row r="103" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B103" s="97" t="s">
-        <v>90</v>
-      </c>
-      <c r="C103" s="90">
-        <f t="shared" si="22"/>
-        <v>2304</v>
-      </c>
-      <c r="D103" s="91" t="s">
-        <v>96</v>
-      </c>
-      <c r="F103" s="47"/>
-    </row>
-    <row r="104" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B104" s="97" t="s">
-        <v>95</v>
-      </c>
-      <c r="C104" s="90">
-        <f t="shared" si="22"/>
-        <v>1995</v>
-      </c>
-      <c r="D104" s="91" t="s">
-        <v>75</v>
-      </c>
-      <c r="F104" s="47"/>
-    </row>
-    <row r="105" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B105" s="102" t="s">
-        <v>97</v>
-      </c>
-      <c r="C105" s="103">
-        <f t="shared" si="22"/>
-        <v>84</v>
-      </c>
-      <c r="D105" s="104" t="s">
-        <v>76</v>
-      </c>
-      <c r="E105" s="105"/>
-      <c r="F105" s="106"/>
-    </row>
-    <row r="106" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B106" s="107" t="s">
-        <v>98</v>
-      </c>
-      <c r="C106" s="103">
-        <f t="shared" si="22"/>
-        <v>2047</v>
-      </c>
-      <c r="D106" s="108" t="s">
-        <v>105</v>
-      </c>
-      <c r="E106" s="105"/>
-      <c r="F106" s="106"/>
-    </row>
-    <row r="107" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B107" s="107" t="s">
-        <v>102</v>
-      </c>
-      <c r="C107" s="103">
+        <v>101</v>
+      </c>
+      <c r="C103" s="93">
         <f t="shared" si="22"/>
         <v>587</v>
       </c>
-      <c r="D107" s="124" t="s">
-        <v>82</v>
-      </c>
-      <c r="E107" s="105"/>
-      <c r="F107" s="106"/>
-    </row>
-    <row r="108" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B108" s="109" t="s">
-        <v>99</v>
-      </c>
-      <c r="C108" s="103">
+      <c r="D103" s="109" t="s">
+        <v>81</v>
+      </c>
+      <c r="E103" s="95"/>
+      <c r="F103" s="96"/>
+    </row>
+    <row r="104" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B104" s="99" t="s">
+        <v>98</v>
+      </c>
+      <c r="C104" s="93">
         <f t="shared" si="22"/>
         <v>3203</v>
       </c>
-      <c r="D108" s="104" t="s">
-        <v>77</v>
-      </c>
-      <c r="E108" s="105"/>
-      <c r="F108" s="106"/>
-    </row>
-    <row r="109" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B109" s="99" t="s">
-        <v>100</v>
-      </c>
-      <c r="C109" s="90">
+      <c r="D104" s="94" t="s">
+        <v>76</v>
+      </c>
+      <c r="E104" s="95"/>
+      <c r="F104" s="96"/>
+    </row>
+    <row r="105" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B105" s="89" t="s">
+        <v>99</v>
+      </c>
+      <c r="C105" s="82">
         <f t="shared" si="22"/>
         <v>881</v>
       </c>
-      <c r="D109" s="101" t="s">
-        <v>82</v>
-      </c>
-      <c r="F109" s="47"/>
-    </row>
-    <row r="110" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B110" s="96" t="s">
-        <v>78</v>
-      </c>
-      <c r="C110" s="90">
+      <c r="D105" s="91" t="s">
+        <v>81</v>
+      </c>
+      <c r="F105" s="47"/>
+    </row>
+    <row r="106" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B106" s="88" t="s">
+        <v>77</v>
+      </c>
+      <c r="C106" s="82">
         <f t="shared" si="22"/>
         <v>256</v>
       </c>
-      <c r="D110" s="91" t="s">
+      <c r="D106" s="83" t="s">
+        <v>78</v>
+      </c>
+      <c r="F106" s="47"/>
+    </row>
+    <row r="107" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B107" s="90" t="s">
         <v>79</v>
       </c>
-      <c r="F110" s="47"/>
-    </row>
-    <row r="111" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B111" s="100" t="s">
+      <c r="C107" s="84">
+        <v>1024</v>
+      </c>
+      <c r="D107" s="85" t="s">
         <v>80</v>
       </c>
-      <c r="C111" s="92">
-        <v>1024</v>
-      </c>
-      <c r="D111" s="93" t="s">
-        <v>81</v>
-      </c>
-      <c r="E111" s="50"/>
-      <c r="F111" s="51"/>
+      <c r="E107" s="50"/>
+      <c r="F107" s="51"/>
     </row>
   </sheetData>
   <mergeCells count="12">

</xml_diff>